<commit_message>
Actualiza el lead Omar Escamilla con la conversación real de WhatsApp (gemelos Gabriel/Rafael) y añade guion para cuando piden prueba social
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -2822,10 +2822,10 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="75" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Omar Escamilla / omare815</t>
+          <t>Omar Escamilla / omare815 — ¿mismo lead que WhatsApp +52 1 81 3408 2672? (verificar con Joel)</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -2835,12 +2835,12 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>México</t>
+          <t>México (Monterrey, 2h de la frontera con Texas)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Gemelos — lateral y mediapunta</t>
+          <t>Gemelos Gabriel (lateral izquierdo, 1.82m) y Rafael (medio, 1.82m) — Club Dallas FC filial México, titulares, buen nivel según el padre</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -2850,27 +2850,27 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Tiene, falta pedirlo</t>
+          <t>Tienen vídeo del año pasado + uno actualizado en camino (semanas)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí — edad, nivel y plazo (agosto 2027) confirmados por el padre</t>
         </is>
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>Pedir el vídeo (de mayo 2026, ya lo tienen listo)</t>
+          <t>Enviar la respuesta preparada 2026-09-11 (honestidad sobre ubicación de Joel + cifra de colocados + pedir el vídeo que ya tienen + Calendly)</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09-10 (WhatsApp)</t>
         </is>
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Datos completos, solo falta el vídeo</t>
+          <t>Preguntó dónde está Joel y por universidades/contactos de coaches/ejemplos de colocados — señal de compra fuerte, no objeción. Ver embudo-ventas.md 'Caso real: ya cualificado, pero pregunta por prueba social'</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Confirma lead Omar Escamilla y marca llamada agendada 15/09
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -2825,7 +2825,7 @@
     <row r="12" ht="75" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Omar Escamilla / omare815 — ¿mismo lead que WhatsApp +52 1 81 3408 2672? (verificar con Joel)</t>
+          <t>Omar Escamilla / omare815 — CONFIRMADO mismo lead que WhatsApp +52 1 81 3408 2672 (Gabriel y Rafael)</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Cualificado</t>
+          <t>Llamada agendada</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -2860,17 +2860,17 @@
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>Enviar la respuesta preparada 2026-09-11 (honestidad sobre ubicación de Joel + cifra de colocados + pedir el vídeo que ya tienen + Calendly)</t>
+          <t>Llamada el 15/09/2026 a las 12:00 — preparar guion específico antes, y pedir el vídeo si no ha llegado</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>2026-09-10 (WhatsApp)</t>
+          <t>2026-09-14 (WhatsApp)</t>
         </is>
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Preguntó dónde está Joel y por universidades/contactos de coaches/ejemplos de colocados — señal de compra fuerte, no objeción. Ver embudo-ventas.md 'Caso real: ya cualificado, pero pregunta por prueba social'</t>
+          <t>Confirmó que le gustó la web. Preguntó país de origen de Joel (respondido: España). Llamada agendada vía Calendly para el 15/09 12:00. Pendiente: vídeo actualizado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza el contacto de Brasil (Leonardo Uren) con historial real y mensaje de reactivación
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -140,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -166,6 +166,9 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1893,10 +1896,10 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
+    <row r="17" ht="90" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Contacto de Brasil</t>
+          <t>Leonardo Uren / equipo (Brasil) — posible partner, no solo cliente</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -1906,37 +1909,62 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Sin evaluar</t>
+          <t>N/A — colaboración institucional, no un grupo de jugadores</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Contacto personal de Joel, sin explorar todavía</t>
+          <t>Conversación real ya avanzada abril-julio 2026: exploraron modelo de colaboración Brasil-España (jugadores/equipos en ambas direcciones), con el padre de Joel involucrado. Se enfrió tras propuesta de llamada el 03/07/2026 sin respuesta</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Joel</t>
-        </is>
-      </c>
-      <c r="F17" s="12" t="inlineStr"/>
-      <c r="G17" s="6" t="inlineStr"/>
+          <t>Contacto personal de Joel</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Leonardo Uren</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Sin email — conversación por WhatsApp</t>
+        </is>
+      </c>
       <c r="H17" s="6" t="inlineStr"/>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>Sin evaluar</t>
+          <t>Listo para enviar (reactivación)</t>
         </is>
       </c>
       <c r="J17" s="12" t="inlineStr">
         <is>
-          <t>Joel decide si vale la pena explorarlo</t>
-        </is>
-      </c>
-      <c r="K17" s="12" t="inlineStr"/>
-      <c r="L17" s="12" t="inlineStr"/>
+          <t>Enviar el mensaje de reactivación de la columna Cuerpo — pendiente de que Joel lo mande</t>
+        </is>
+      </c>
+      <c r="K17" s="12" t="inlineStr">
+        <is>
+          <t>N/A — mensaje de WhatsApp, no email</t>
+        </is>
+      </c>
+      <c r="L17" s="14" t="inlineStr">
+        <is>
+          <t>Hi Leonardo! Hope you and the team are doing well.
+It's been a while since we talked - a lot has happened on our side too. We've been growing our international side, and with Spain now World Cup champions there's a lot more interest from clubs/academies wanting to connect with Spanish football, so it feels like a good moment to pick this back up.
+I still think there's real potential in a Brazil-Spain connection - players/teams coming to train in Spain, and maybe the other way around too. Would you be up for reopening that conversation? My dad would join again as well. No need to tie it to a specific trip this time - happy to find 20-30 minutes whenever works for you guys.
+Let me know!</t>
+        </is>
+      </c>
       <c r="M17" s="13" t="inlineStr"/>
-      <c r="N17" s="13" t="inlineStr"/>
-      <c r="O17" s="12" t="inlineStr"/>
+      <c r="N17" s="13" t="n">
+        <v>46206</v>
+      </c>
+      <c r="O17" s="12" t="inlineStr">
+        <is>
+          <t>Historial real: llamada en abril 2026, Leonardo mandó una presentación (enfocada en becas EEUU, poco encaje con lo que ya cubre el partner de becas), Joel propuso el ángulo real (intercambio Brasil-España de jugadores/equipos), propuso llamada con el padre para junio, luego siguió el 03/07 proponiendo martes — sin respuesta desde entonces (2+ meses). No confundir con un club prospecto normal de Segmento A — esto es más una posible relación de partner/distribución que una venta directa.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A5:O17"/>

</xml_diff>

<commit_message>
Registra resultado de la llamada con Omar y ajusta fecha de seguimiento a fin de semana
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -2873,7 +2873,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Llamada agendada</t>
+          <t>Llamada realizada</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -2888,17 +2888,17 @@
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>Llamada el 15/09/2026 a las 12:00 — preparar guion específico antes, y pedir el vídeo si no ha llegado</t>
+          <t>Esperando 'okay' de la familia para mandar evaluación/propuesta. Seguimiento suave si no hay respuesta antes del viernes 19/09/2026 (fin de semana según Joel). Confirmar con Joel si ya tiene el vídeo para tenerlo listo antes de que llegue el okay</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>2026-09-14 (WhatsApp)</t>
+          <t>2026-09-15 (llamada)</t>
         </is>
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Confirmó que le gustó la web. Preguntó país de origen de Joel (respondido: España). Llamada agendada vía Calendly para el 15/09 12:00. Pendiente: vídeo actualizado</t>
+          <t>Llamada realizada 15/09/2026. Resultado: la familia lo va a valorar 'en los próximos días', Joel manda evaluación/propuesta cuando den el okay. Joel ya envió foto de precios por WhatsApp + mensaje de cierre de llamada. Pendiente: confirmar si ya tienen el vídeo en mano, y si se aclaró en la llamada si buscan la misma universidad para los dos gemelos o están abiertos a separarse.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Añade lead Daniel (MLS NEXT U17, recién mudado a España) al CRM
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -2493,7 +2493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3221,6 +3221,58 @@
         </is>
       </c>
       <c r="J19" s="12" t="inlineStr"/>
+    </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Daniel (apellido/@ de Instagram pendiente de confirmar)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>17 (nacido sept. 2009)</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>España (recién mudado desde EEUU, ciudad por confirmar)</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Jugó MLS NEXT U17 el año pasado en EEUU (nivel alto) — posición por confirmar</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Cualificado</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>No pedido todavía</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Sí — nivel MLS NEXT es señal fuerte, falta confirmar posición y club actual</t>
+        </is>
+      </c>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>Esperar respuesta a las 3 preguntas (posición / ubicación en España / club actual) — probablemente avanza rápido a Calendly, es un lead fuerte</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="J20" s="12" t="inlineStr">
+        <is>
+          <t>Pregunta genuina sobre 1º vs 2º de Bachillerato y elegibilidad NCAA — no se improvisó respuesta, se remitió a la evaluación completa con el equipo especializado. Edad+plazo+nivel ya fuertes antes incluso de pedir vídeo.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A5:J19"/>

</xml_diff>

<commit_message>
Documenta política de adjuntos por email y crea firma con marca
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Segmento A - Clubes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Segmento B - America" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Segmento C - Becas" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="LinkedIn - Plan diario" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Oportunidades y notas" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmento A - Clubes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmento B - America" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmento C - Becas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LinkedIn - Plan diario" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oportunidades y notas" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Segmento A - Clubes'!$A$5:$O$17</definedName>
@@ -1306,7 +1306,7 @@
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>Enviar el email de la columna siguiente hoy</t>
+          <t>Enviar el email de la columna siguiente hoy — SIN adjuntos en este primer email, solo texto</t>
         </is>
       </c>
       <c r="K6" s="12" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>Enviar el email de la columna siguiente esta semana</t>
+          <t>Enviar el email de la columna siguiente esta semana — SIN adjuntos en este primer email, solo texto</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Enviar el email de la columna siguiente esta semana</t>
+          <t>Enviar el email de la columna siguiente esta semana — SIN adjuntos en este primer email, solo texto</t>
         </is>
       </c>
       <c r="K12" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Crea fichas separadas Team y Coach Experience (sin precio, con escudos y fotos oficiales) y añade columna 'qué adjuntar' al CRM
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -16,9 +16,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oportunidades y notas" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Segmento A - Clubes'!$A$5:$O$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Segmento B - America'!$A$5:$N$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Segmento C - Becas'!$A$5:$J$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Segmento A - Clubes'!$A$5:$P$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Segmento B - America'!$A$5:$O$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Segmento C - Becas'!$A$5:$K$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Oportunidades y notas'!$A$4:$F$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -140,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -169,6 +169,9 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1139,7 +1142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1157,6 +1160,7 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="55" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1255,6 +1259,11 @@
       <c r="O5" s="5" t="inlineStr">
         <is>
           <t>Notas</t>
+        </is>
+      </c>
+      <c r="P5" s="15" t="inlineStr">
+        <is>
+          <t>Qué adjuntar (por etapa)</t>
         </is>
       </c>
     </row>
@@ -1333,6 +1342,11 @@
           <t>Email ya preparado y revisado 2026-08-29 — solo falta que Joel lo envíe</t>
         </is>
       </c>
+      <c r="P6" s="12" t="inlineStr">
+        <is>
+          <t>1er email: NADA adjunto, solo texto (firma de texto plano). Si responde con interés: ficha Always-Up-Team-Experience.pdf. Antes de la llamada: deck de empresa (pendiente de crear), solo si hace falta. Tras la llamada: propuesta escrita.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -1404,6 +1418,11 @@
           <t>También: fotball@soreideil.no (contacto general del club)</t>
         </is>
       </c>
+      <c r="P7" s="12" t="inlineStr">
+        <is>
+          <t>1er email: NADA adjunto, solo texto (firma de texto plano). Si responde con interés: ficha Always-Up-Team-Experience.pdf. Antes de la llamada: deck de empresa (pendiente de crear), solo si hace falta. Tras la llamada: propuesta escrita.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -1465,6 +1484,11 @@
           <t>Llamar o contactar vía redes sociales del club para conseguir email directo</t>
         </is>
       </c>
+      <c r="P8" s="12" t="inlineStr">
+        <is>
+          <t>1er email: NADA adjunto, solo texto (firma de texto plano). Si responde con interés: ficha Always-Up-Team-Experience.pdf. Antes de la llamada: deck de empresa (pendiente de crear), solo si hace falta. Tras la llamada: propuesta escrita.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
@@ -1522,6 +1546,11 @@
           <t>Investigado 2026-08-29: club real con categorías U13-U15 chicas, pero sin decisor nombrado todavía — no está al nivel de Home Farm/Hastings todavía</t>
         </is>
       </c>
+      <c r="P9" s="12" t="inlineStr">
+        <is>
+          <t>1er email: NADA adjunto, solo texto (firma de texto plano). Si responde con interés: ficha Always-Up-Team-Experience.pdf. Antes de la llamada: deck de empresa (pendiente de crear), solo si hace falta. Tras la llamada: propuesta escrita.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -1571,6 +1600,11 @@
           <t>Investigado 2026-08-29: posible error de nombre en el research original — no gastar más tiempo hasta verificar en la fuente original</t>
         </is>
       </c>
+      <c r="P10" s="12" t="inlineStr">
+        <is>
+          <t>1er email: NADA adjunto, solo texto (firma de texto plano). Si responde con interés: ficha Always-Up-Team-Experience.pdf. Antes de la llamada: deck de empresa (pendiente de crear), solo si hace falta. Tras la llamada: propuesta escrita.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -1630,6 +1664,11 @@
       <c r="O11" s="12" t="inlineStr">
         <is>
           <t>Investigado 2026-08-29: contacto general real, falta nombre de decisor</t>
+        </is>
+      </c>
+      <c r="P11" s="12" t="inlineStr">
+        <is>
+          <t>1er email: NADA adjunto, solo texto (firma de texto plano). Si responde con interés: ficha Always-Up-Team-Experience.pdf. Antes de la llamada: deck de empresa (pendiente de crear), solo si hace falta. Tras la llamada: propuesta escrita.</t>
         </is>
       </c>
     </row>
@@ -1703,6 +1742,11 @@
           <t>Investigado 2026-08-29: el mejor de los 4 investigados hoy — decisor nombrado y academia real</t>
         </is>
       </c>
+      <c r="P12" s="12" t="inlineStr">
+        <is>
+          <t>1er email: NADA adjunto, solo texto (firma de texto plano). Si responde con interés: ficha Always-Up-Team-Experience.pdf. Antes de la llamada: deck de empresa (pendiente de crear), solo si hace falta. Tras la llamada: propuesta escrita.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -1756,6 +1800,11 @@
           <t>Investigado 2026-08-29: discrepancia entre el research original y lo encontrado hoy — no mandar nada hasta confirmar</t>
         </is>
       </c>
+      <c r="P13" s="12" t="inlineStr">
+        <is>
+          <t>1er email: NADA adjunto, solo texto (firma de texto plano). Si responde con interés: ficha Always-Up-Team-Experience.pdf. Antes de la llamada: deck de empresa (pendiente de crear), solo si hace falta. Tras la llamada: propuesta escrita.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
@@ -1801,6 +1850,11 @@
       <c r="M14" s="13" t="inlineStr"/>
       <c r="N14" s="13" t="inlineStr"/>
       <c r="O14" s="12" t="inlineStr"/>
+      <c r="P14" s="12" t="inlineStr">
+        <is>
+          <t>1er email: NADA adjunto, solo texto (firma de texto plano). Si responde con interés: ficha Always-Up-Team-Experience.pdf. Antes de la llamada: deck de empresa (pendiente de crear), solo si hace falta. Tras la llamada: propuesta escrita.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
@@ -1846,6 +1900,11 @@
       <c r="M15" s="13" t="inlineStr"/>
       <c r="N15" s="13" t="inlineStr"/>
       <c r="O15" s="12" t="inlineStr"/>
+      <c r="P15" s="12" t="inlineStr">
+        <is>
+          <t>1er email: NADA adjunto, solo texto (firma de texto plano). Si responde con interés: ficha Always-Up-Team-Experience.pdf. Antes de la llamada: deck de empresa (pendiente de crear), solo si hace falta. Tras la llamada: propuesta escrita.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
@@ -1895,6 +1954,11 @@
           <t>Ver 01-clients/pipeline.md — no duplicar seguimiento aquí, solo referencia</t>
         </is>
       </c>
+      <c r="P16" s="12" t="inlineStr">
+        <is>
+          <t>Seguimiento ya en marcha fuera del flujo de outreach: sin adjuntos nuevos.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -1965,9 +2029,14 @@
           <t>Historial real: llamada en abril 2026, Leonardo mandó una presentación (enfocada en becas EEUU, poco encaje con lo que ya cubre el partner de becas), Joel propuso el ángulo real (intercambio Brasil-España de jugadores/equipos), propuso llamada con el padre para junio, luego siguió el 03/07 proponiendo martes — sin respuesta desde entonces (2+ meses). No confundir con un club prospecto normal de Segmento A — esto es más una posible relación de partner/distribución que una venta directa.</t>
         </is>
       </c>
+      <c r="P17" s="12" t="inlineStr">
+        <is>
+          <t>Es un posible partner, no una venta estándar: sin adjuntos. Mensaje de WhatsApp y proponer llamada; llevar a la llamada ficha Team Experience + Campus Internacional (pendiente) si derivan a servicios.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:O17"/>
+  <autoFilter ref="A5:P17"/>
   <mergeCells count="3">
     <mergeCell ref="A3:O4"/>
     <mergeCell ref="A1:O1"/>
@@ -1983,7 +2052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2000,6 +2069,7 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="55" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2093,6 +2163,11 @@
       <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Notas</t>
+        </is>
+      </c>
+      <c r="O5" s="15" t="inlineStr">
+        <is>
+          <t>Qué adjuntar (por etapa)</t>
         </is>
       </c>
     </row>
@@ -2139,6 +2214,11 @@
       <c r="L6" s="13" t="inlineStr"/>
       <c r="M6" s="13" t="inlineStr"/>
       <c r="N6" s="12" t="inlineStr"/>
+      <c r="O6" s="12" t="inlineStr">
+        <is>
+          <t>1er email/LinkedIn: NADA adjunto. Si responde: ficha Team Experience (equipos) o Campus Internacional (academias, ficha pendiente). Segmento secundario: no invertir en materiales a medida hasta tener conversaciones reales.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2187,6 +2267,11 @@
           <t>Aviso: categoría IberCup es U11/U12 7v7 — confirmar que tienen categorías mayores antes de contactar</t>
         </is>
       </c>
+      <c r="O7" s="12" t="inlineStr">
+        <is>
+          <t>1er email/LinkedIn: NADA adjunto. Si responde: ficha Team Experience (equipos) o Campus Internacional (academias, ficha pendiente). Segmento secundario: no invertir en materiales a medida hasta tener conversaciones reales.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2235,6 +2320,11 @@
           <t>Mismo aviso de edad que arriba</t>
         </is>
       </c>
+      <c r="O8" s="12" t="inlineStr">
+        <is>
+          <t>1er email/LinkedIn: NADA adjunto. Si responde: ficha Team Experience (equipos) o Campus Internacional (academias, ficha pendiente). Segmento secundario: no invertir en materiales a medida hasta tener conversaciones reales.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -2283,6 +2373,11 @@
           <t>Mismo aviso de edad que arriba</t>
         </is>
       </c>
+      <c r="O9" s="12" t="inlineStr">
+        <is>
+          <t>1er email/LinkedIn: NADA adjunto. Si responde: ficha Team Experience (equipos) o Campus Internacional (academias, ficha pendiente). Segmento secundario: no invertir en materiales a medida hasta tener conversaciones reales.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -2331,6 +2426,11 @@
           <t>Mismo aviso de edad que arriba</t>
         </is>
       </c>
+      <c r="O10" s="12" t="inlineStr">
+        <is>
+          <t>1er email/LinkedIn: NADA adjunto. Si responde: ficha Team Experience (equipos) o Campus Internacional (academias, ficha pendiente). Segmento secundario: no invertir en materiales a medida hasta tener conversaciones reales.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -2379,6 +2479,11 @@
           <t>Mismo aviso de edad que arriba</t>
         </is>
       </c>
+      <c r="O11" s="12" t="inlineStr">
+        <is>
+          <t>1er email/LinkedIn: NADA adjunto. Si responde: ficha Team Experience (equipos) o Campus Internacional (academias, ficha pendiente). Segmento secundario: no invertir en materiales a medida hasta tener conversaciones reales.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -2427,6 +2532,11 @@
           <t>Programa grande con relaciones ya asentadas, mal candidato para primer contacto. Dejar como caso de estudio del mercado</t>
         </is>
       </c>
+      <c r="O12" s="12" t="inlineStr">
+        <is>
+          <t>1er email/LinkedIn: NADA adjunto. Si responde: ficha Team Experience (equipos) o Campus Internacional (academias, ficha pendiente). Segmento secundario: no invertir en materiales a medida hasta tener conversaciones reales.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -2475,9 +2585,14 @@
           <t>Búsqueda rápida (2026-08-29) no encontró candidatos concretos — requiere sesión de investigación dedicada, no una búsqueda genérica</t>
         </is>
       </c>
+      <c r="O13" s="12" t="inlineStr">
+        <is>
+          <t>1er email/LinkedIn: NADA adjunto. Si responde: ficha Team Experience (equipos) o Campus Internacional (academias, ficha pendiente). Segmento secundario: no invertir en materiales a medida hasta tener conversaciones reales.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:N13"/>
+  <autoFilter ref="A5:O13"/>
   <mergeCells count="3">
     <mergeCell ref="A3:N4"/>
     <mergeCell ref="A2:N2"/>
@@ -2493,7 +2608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2506,6 +2621,7 @@
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2581,6 +2697,11 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>Qué adjuntar (por etapa)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2631,6 +2752,11 @@
       <c r="J6" s="12" t="inlineStr">
         <is>
           <t>Dilema real: ir a EEUU 2027 vs. quedarse en Portugal a estudiar</t>
+        </is>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -2673,6 +2799,11 @@
           <t>Preguntó directamente por el sistema de becas</t>
         </is>
       </c>
+      <c r="K7" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2723,6 +2854,11 @@
       <c r="J8" s="12" t="inlineStr">
         <is>
           <t>Lead fuerte — ya en EEUU, quiere seguir compitiendo y sacar diploma</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -2761,6 +2897,11 @@
           <t>Lead muy caliente, solo falta confirmar</t>
         </is>
       </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -2797,6 +2938,11 @@
           <t>Intentaba cerrar día ('hoy o mañana'), se quedó sin respuesta</t>
         </is>
       </c>
+      <c r="K10" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -2849,6 +2995,11 @@
           <t>Originalmente pedía Inglaterra, aceptó explorar vía EEUU</t>
         </is>
       </c>
+      <c r="K11" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="75" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
@@ -2901,6 +3052,11 @@
           <t>Llamada realizada 15/09/2026. Resultado: la familia lo va a valorar 'en los próximos días', Joel manda evaluación/propuesta cuando den el okay. Joel ya envió foto de precios por WhatsApp + mensaje de cierre de llamada. Pendiente: confirmar si ya tienen el vídeo en mano, y si se aclaró en la llamada si buscan la misma universidad para los dos gemelos o están abiertos a separarse.</t>
         </is>
       </c>
+      <c r="K12" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -2947,6 +3103,11 @@
       <c r="J13" s="12" t="inlineStr">
         <is>
           <t>Pidió la guía explícitamente</t>
+        </is>
+      </c>
+      <c r="K13" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -2993,6 +3154,11 @@
           <t>Conversación avanzada que se enfrió</t>
         </is>
       </c>
+      <c r="K14" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -3041,6 +3207,11 @@
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr"/>
+      <c r="K15" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -3085,6 +3256,11 @@
         </is>
       </c>
       <c r="J16" s="12" t="inlineStr"/>
+      <c r="K16" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -3133,6 +3309,11 @@
           <t>Confirmado: Always Up sí trabaja otros deportes, no solo fútbol</t>
         </is>
       </c>
+      <c r="K17" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -3183,6 +3364,11 @@
       <c r="J18" s="12" t="inlineStr">
         <is>
           <t>Cuenta confirmada por Joel — verificar en próximo barrido</t>
+        </is>
+      </c>
+      <c r="K18" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -3221,6 +3407,11 @@
         </is>
       </c>
       <c r="J19" s="12" t="inlineStr"/>
+      <c r="K19" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -3273,9 +3464,14 @@
           <t>Pregunta genuina sobre 1º vs 2º de Bachillerato y elegibilidad NCAA — no se improvisó respuesta, se remitió a la evaluación completa con el equipo especializado. Edad+plazo+nivel ya fuertes antes incluso de pedir vídeo.</t>
         </is>
       </c>
+      <c r="K20" s="12" t="inlineStr">
+        <is>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:J19"/>
+  <autoFilter ref="A5:K20"/>
   <mergeCells count="3">
     <mergeCell ref="A3:J4"/>
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
Rehace el ejemplo de 5 días con formato real, crea la ficha de Becas EEUU y actualiza CRM y guía de materiales
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -2756,7 +2756,7 @@
       </c>
       <c r="K6" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="K7" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -2899,7 +2899,7 @@
       </c>
       <c r="K9" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -2940,7 +2940,7 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -2997,7 +2997,7 @@
       </c>
       <c r="K11" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="K13" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
       <c r="J15" s="12" t="inlineStr"/>
       <c r="K15" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
       <c r="J16" s="12" t="inlineStr"/>
       <c r="K16" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="K17" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
       </c>
       <c r="K18" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -3409,7 +3409,7 @@
       <c r="J19" s="12" t="inlineStr"/>
       <c r="K19" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3466,7 @@
       </c>
       <c r="K20" s="12" t="inlineStr">
         <is>
-          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): guía de becas con marca Always Up (pendiente de crear; hasta entonces guia-becas.md, NUNCA el deck de University Soccer). Mensajes cortos, pensados para móvil. Llamada: Calendly.</t>
+          <t>1er DM: sin adjuntos. Tras cualificar (nivel + vídeo): ficha Always-Up-Becas-EEUU.pdf (2 págs, en español, pensada para móvil, sin precio). NUNCA el deck de University Soccer. Llamada: Calendly.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Registra envío de los 3 primeros emails (13/10), estado de Omar y deck público en LinkedIn
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -1142,7 +1142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1310,12 +1310,12 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>Listo para enviar</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>Enviar el email de la columna siguiente hoy — SIN adjuntos en este primer email, solo texto</t>
+          <t>Follow-up 1 el 27/10/2026 si no responde (mensaje corto que aporte algo, sin adjuntos). Si responde con interés: ficha Team Experience</t>
         </is>
       </c>
       <c r="K6" s="12" t="inlineStr">
@@ -1335,11 +1335,15 @@
 Joel</t>
         </is>
       </c>
-      <c r="M6" s="13" t="inlineStr"/>
-      <c r="N6" s="13" t="inlineStr"/>
+      <c r="M6" s="13" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N6" s="13" t="n">
+        <v>46308</v>
+      </c>
       <c r="O6" s="12" t="inlineStr">
         <is>
-          <t>Email ya preparado y revisado 2026-08-29 — solo falta que Joel lo envíe</t>
+          <t>Email ya preparado y revisado 2026-08-29 — solo falta que Joel lo envíe | Enviado 13/10/2026 a las 15:23 (hora de Nueva York) desde joel.martinez@alwaysup.es, solo texto, sin firma ni adjuntos</t>
         </is>
       </c>
       <c r="P6" s="12" t="inlineStr">
@@ -1387,12 +1391,12 @@
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>Listo para enviar</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>Enviar el email de la columna siguiente esta semana — SIN adjuntos en este primer email, solo texto</t>
+          <t>Follow-up 1 el 27/10/2026 si no responde (mensaje corto que aporte algo, sin adjuntos). Si responde con interés: ficha Team Experience</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr">
@@ -1411,11 +1415,15 @@
 Joel</t>
         </is>
       </c>
-      <c r="M7" s="13" t="inlineStr"/>
-      <c r="N7" s="13" t="inlineStr"/>
+      <c r="M7" s="13" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N7" s="13" t="n">
+        <v>46308</v>
+      </c>
       <c r="O7" s="12" t="inlineStr">
         <is>
-          <t>También: fotball@soreideil.no (contacto general del club)</t>
+          <t>También: fotball@soreideil.no (contacto general del club) | Enviado 13/10/2026 a las 15:31 (hora de Nueva York) desde joel.martinez@alwaysup.es, solo texto, sin firma ni adjuntos</t>
         </is>
       </c>
       <c r="P7" s="12" t="inlineStr">
@@ -1711,12 +1719,12 @@
       <c r="H12" s="6" t="inlineStr"/>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Listo para enviar</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Enviar el email de la columna siguiente esta semana — SIN adjuntos en este primer email, solo texto</t>
+          <t>Follow-up 1 el 27/10/2026 si no responde (mensaje corto que aporte algo, sin adjuntos). Si responde con interés: ficha Team Experience</t>
         </is>
       </c>
       <c r="K12" s="12" t="inlineStr">
@@ -1735,11 +1743,15 @@
 Joel</t>
         </is>
       </c>
-      <c r="M12" s="13" t="inlineStr"/>
-      <c r="N12" s="13" t="inlineStr"/>
+      <c r="M12" s="13" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N12" s="13" t="n">
+        <v>46308</v>
+      </c>
       <c r="O12" s="12" t="inlineStr">
         <is>
-          <t>Investigado 2026-08-29: el mejor de los 4 investigados hoy — decisor nombrado y academia real</t>
+          <t>Investigado 2026-08-29: el mejor de los 4 investigados hoy — decisor nombrado y academia real | Enviado 13/10/2026 a las 15:33 (hora de Nueva York) desde joel.martinez@alwaysup.es, solo texto, sin firma ni adjuntos</t>
         </is>
       </c>
       <c r="P12" s="12" t="inlineStr">
@@ -2035,6 +2047,8 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
   </sheetData>
   <autoFilter ref="A5:P17"/>
   <mergeCells count="3">
@@ -2608,7 +2622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3039,17 +3053,17 @@
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>Esperando 'okay' de la familia para mandar evaluación/propuesta. Seguimiento suave si no hay respuesta antes del viernes 19/09/2026 (fin de semana según Joel). Confirmar con Joel si ya tiene el vídeo para tenerlo listo antes de que llegue el okay</t>
+          <t>Follow-up 13/10: lleva 14 días sin responder desde el 29/09; prometió vídeo y datos 'la próxima semana' (5/10) y no ha llegado. Pedir lo que tenga YA (aunque sea el del año pasado + notas) y empezar la primera lectura. NO ofrecer más descuento.</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>2026-09-15 (llamada)</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Llamada realizada 15/09/2026. Resultado: la familia lo va a valorar 'en los próximos días', Joel manda evaluación/propuesta cuando den el okay. Joel ya envió foto de precios por WhatsApp + mensaje de cierre de llamada. Pendiente: confirmar si ya tienen el vídeo en mano, y si se aclaró en la llamada si buscan la misma universidad para los dos gemelos o están abiertos a separarse.</t>
+          <t>Llamada realizada 15/09/2026. Resultado: la familia lo va a valorar 'en los próximos días', Joel manda evaluación/propuesta cuando den el okay. Joel ya envió foto de precios por WhatsApp + mensaje de cierre de llamada. Pendiente: confirmar si ya tienen el vídeo en mano, y si se aclaró en la llamada si buscan la misma universidad para los dos gemelos o están abiertos a separarse. | 17/09 objeción: precio alto 'x2', quiere evaluación antes de decidir (qué beca y qué división). 18/09 oferta de Joel por niño: pago único $2.000 (en vez de $2.500) o 2 plazos $250 + $2.500 (en vez de $3.500). 27/09 Omar: 'la próxima semana te envío vídeo y datos'. Sin datos desde entonces.</t>
         </is>
       </c>
       <c r="K12" s="12" t="inlineStr">
@@ -3470,6 +3484,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
   </sheetData>
   <autoFilter ref="A5:K20"/>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Plan de outreach 30 dias: hoja de textos listos para copiar, generador, contactos verificados y correccion del rebote de Soreide
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -8,18 +8,19 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmento A - Clubes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmento B - America" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmento C - Becas" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LinkedIn - Plan diario" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oportunidades y notas" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach - Copiar y pegar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmento A - Clubes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmento B - America" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmento C - Becas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LinkedIn - Plan diario" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oportunidades y notas" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Segmento A - Clubes'!$A$5:$P$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Segmento B - America'!$A$5:$O$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Segmento C - Becas'!$A$5:$K$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Oportunidades y notas'!$A$4:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Segmento A - Clubes'!$A$5:$P$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Segmento B - America'!$A$5:$O$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Segmento C - Becas'!$A$5:$K$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Oportunidades y notas'!$A$4:$F$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,7 +31,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,8 +96,17 @@
       <color rgb="001F4E78"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000B1F3A"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -111,6 +121,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000B1F3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F1FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF6DD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEEEEE"/>
       </patternFill>
     </fill>
   </fills>
@@ -140,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -172,6 +207,40 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -913,6 +982,2176 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="78" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Outreach: copiar y pegar (ordenado por fecha)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Cada fila es un envío listo. Fecha = día de envío. Hora = 09:30 locales del destinatario (la columna de Nueva York ya la convierte). Tras enviar: marca 'Hecho' y escribe la fecha real. Si el club contesta, deja de enviar el resto de sus filas y sigue el guion de respuestas en 02-sales/plan-outreach-30-dias.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Día</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Hora local (09:30)</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Hora Nueva York</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>Club</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Para</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Asunto</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Texto para pegar</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Cómo enviarlo</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Hecho (fecha real)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="255" customHeight="1">
+      <c r="A5" s="19" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>mié</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>Holbeach United</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>Email 1</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="inlineStr">
+        <is>
+          <t>callum@holbeachunitedacademy.com</t>
+        </is>
+      </c>
+      <c r="H5" s="20" t="inlineStr">
+        <is>
+          <t>Training week in Spain for Holbeach United's academy</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>Hi Callum,
+I'm Joel, founder of Always Up. We organise training weeks in Spain for youth clubs: sessions at the facilities of Atlético de Madrid and Real Sociedad, matches against local academy teams and a stadium tour, with accommodation and meals included.
+I saw Holbeach United was listed for the Costa Daurada Cup in Salou this year, and your Football &amp; Education Academy stood out, so I thought a week in Spain could be a good fit for your older squads.
+A longtime partner club of ours won its first-ever league title after training with us, and its coaches credit part of it to the experience.
+Would you be open to a short call next week, or would you prefer I send a one-page overview first?
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J5" s="20" t="inlineStr">
+        <is>
+          <t>Outlook &gt; Nuevo correo. Para / Asunto / Cuerpo tal cual (incluye la firma). Sin adjuntos. Usa 'Programar envío' para la hora indicada. A los 5 min de enviar, mira la bandeja por si hay rebote.</t>
+        </is>
+      </c>
+      <c r="K5" s="20" t="n"/>
+    </row>
+    <row r="6" ht="255" customHeight="1">
+      <c r="A6" s="19" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>mié</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>Søreide IL</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>Email 1</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>fotball@soreideil.no</t>
+        </is>
+      </c>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>Training week in Spain for Søreide IL's youth teams</t>
+        </is>
+      </c>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>Hi Marius and Gunn,
+I'm Joel, founder of Always Up. My first email bounced from your youth committee address, so I'm writing to you directly.
+We organise training weeks in Spain for youth clubs: sessions at the facilities of Atlético de Madrid and Real Sociedad, matches against local academy teams, and accommodation and meals included.
+I saw Søreide IL was listed for the Costa Daurada Cup in Salou this summer, so Spain may already be on your radar. A longtime partner club of ours won its first-ever league title after training with us.
+Would you be open to a short call next week, or would you prefer a one-page overview first?
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>Outlook &gt; Nuevo correo. Para / Asunto / Cuerpo tal cual (incluye la firma). Sin adjuntos. Usa 'Programar envío' para la hora indicada. A los 5 min de enviar, mira la bandeja por si hay rebote.</t>
+        </is>
+      </c>
+      <c r="K6" s="20" t="n"/>
+    </row>
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="21" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>cuando puedas</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>Hastings United (Girls Academy)</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn: conectar</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>Georgia Townsend (Head of Girls Academy, Hastings United)</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="inlineStr">
+        <is>
+          <t>(nota de conexión)</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>Hi Georgia, I'm Joel, founder of Always Up. We help youth clubs train in Spain with Atlético de Madrid and Real Sociedad. I emailed you recently and wanted to connect here too. Best, Joel</t>
+        </is>
+      </c>
+      <c r="J7" s="17" t="inlineStr">
+        <is>
+          <t>A mano en LinkedIn (no automatizar): perfil de la persona &gt; Conectar &gt; Añadir nota &gt; pegar. Máx. 300 caracteres. Si no aparece 'Añadir nota', conecta sin nota y manda este texto al aceptar. ATENCIÓN: Joel lo hace a mano.</t>
+        </is>
+      </c>
+      <c r="K7" s="17" t="n"/>
+    </row>
+    <row r="8" ht="225" customHeight="1">
+      <c r="A8" s="19" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>IA Akranes</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>Email 1</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="inlineStr">
+        <is>
+          <t>kfia@ia.is</t>
+        </is>
+      </c>
+      <c r="H8" s="20" t="inlineStr">
+        <is>
+          <t>Question about youth trips to Spain</t>
+        </is>
+      </c>
+      <c r="I8" s="20" t="inlineStr">
+        <is>
+          <t>Hi ÍA team,
+I'm Joel, founder of Always Up. We organise training weeks in Spain for youth clubs: sessions at the facilities of Atlético de Madrid and Real Sociedad, matches against local academy teams and a stadium tour, with accommodation and meals included.
+I saw ÍA Akranes was listed for the Costa Daurada Cup in Salou this year. Could you point me to the person who organises trips abroad for your youth teams (yngri flokkar)?
+A longtime partner club of ours won its first-ever league title after training with us, and its coaches credit part of it to the experience, so I'd be glad to share how it worked for them.
+Thanks a lot,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J8" s="20" t="inlineStr">
+        <is>
+          <t>Outlook &gt; Nuevo correo. Para / Asunto / Cuerpo tal cual (incluye la firma). Sin adjuntos. Usa 'Programar envío' para la hora indicada. A los 5 min de enviar, mira la bandeja por si hay rebote.</t>
+        </is>
+      </c>
+      <c r="K8" s="20" t="n"/>
+    </row>
+    <row r="9" ht="225" customHeight="1">
+      <c r="A9" s="19" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>Maidstone United (Girls Development Centre)</t>
+        </is>
+      </c>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>Email 1</t>
+        </is>
+      </c>
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>info@maidstoneunited.co.uk</t>
+        </is>
+      </c>
+      <c r="H9" s="20" t="inlineStr">
+        <is>
+          <t>Question about the Girls Development Centre</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>Hi team,
+I'm Joel, founder of Always Up. We organise training weeks in Spain for youth clubs: sessions at the facilities of Atlético de Madrid and Real Sociedad, matches against local academy teams and a stadium tour, with accommodation and meals included.
+I saw Maidstone United was in the Costa Daurada Cup line-up in Salou this summer and thought your Girls Development Centre could be a great fit. Could you point me to the right person to speak with about trips for the girls' teams?
+A longtime partner club of ours won its first-ever league title after training with us, so I'd be glad to share how it worked for them.
+Thanks a lot,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J9" s="20" t="inlineStr">
+        <is>
+          <t>Outlook &gt; Nuevo correo. Para / Asunto / Cuerpo tal cual (incluye la firma). Sin adjuntos. Usa 'Programar envío' para la hora indicada. A los 5 min de enviar, mira la bandeja por si hay rebote.</t>
+        </is>
+      </c>
+      <c r="K9" s="20" t="n"/>
+    </row>
+    <row r="10" ht="225" customHeight="1">
+      <c r="A10" s="19" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Whitehaven AFC (Juniors Girls U13-U15)</t>
+        </is>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>Email 1</t>
+        </is>
+      </c>
+      <c r="G10" s="20" t="inlineStr">
+        <is>
+          <t>Luke.johnston@whitehavenafc.com</t>
+        </is>
+      </c>
+      <c r="H10" s="20" t="inlineStr">
+        <is>
+          <t>Training week in Spain for Whitehaven's girls teams</t>
+        </is>
+      </c>
+      <c r="I10" s="20" t="inlineStr">
+        <is>
+          <t>Hi Luke,
+I'm Joel, founder of Always Up. We organise training weeks in Spain for youth clubs: sessions at the facilities of Atlético de Madrid and Real Sociedad, matches against local academy teams and a stadium tour, with accommodation and meals included.
+I saw Whitehaven AFC was listed for the Costa Daurada Cup in Salou this summer, and the girls pathway (U13-U15) caught my eye. A longtime partner club of ours won its first-ever league title after training with us.
+Would a short call next week work, or would you prefer a one-page overview first? And if you're not the right person, could you point me to whoever organises trips for the girls' section?
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J10" s="20" t="inlineStr">
+        <is>
+          <t>Outlook &gt; Nuevo correo. Para / Asunto / Cuerpo tal cual (incluye la firma). Sin adjuntos. Usa 'Programar envío' para la hora indicada. A los 5 min de enviar, mira la bandeja por si hay rebote. ATENCIÓN: Email obtenido de un buscador: comprobarlo en whitehavenafc.com/contact antes de enviar. Si es otro, usar el de la web.</t>
+        </is>
+      </c>
+      <c r="K10" s="20" t="n"/>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="21" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>vie</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>cuando puedas</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>Holbeach United</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn: conectar</t>
+        </is>
+      </c>
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>Callum Lawe (Holbeach United Football &amp; Education Academy)</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>(nota de conexión)</t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>Hi Callum, I'm Joel, founder of Always Up. We help youth clubs train in Spain with Atlético de Madrid and Real Sociedad. I emailed you recently and wanted to connect here too. Best, Joel</t>
+        </is>
+      </c>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>A mano en LinkedIn (no automatizar): perfil de la persona &gt; Conectar &gt; Añadir nota &gt; pegar. Máx. 300 caracteres. Si no aparece 'Añadir nota', conecta sin nota y manda este texto al aceptar. ATENCIÓN: Joel lo hace a mano.</t>
+        </is>
+      </c>
+      <c r="K11" s="17" t="n"/>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="21" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>vie</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>cuando puedas</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>Søreide IL</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn: conectar</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>Marius Engen (Sportslig leder, Søreide IL fotball)</t>
+        </is>
+      </c>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>(nota de conexión)</t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>Hi Marius, I'm Joel, founder of Always Up. We help youth clubs train in Spain with Atlético de Madrid and Real Sociedad. I emailed you recently and wanted to connect here too. Best, Joel</t>
+        </is>
+      </c>
+      <c r="J12" s="17" t="inlineStr">
+        <is>
+          <t>A mano en LinkedIn (no automatizar): perfil de la persona &gt; Conectar &gt; Añadir nota &gt; pegar. Máx. 300 caracteres. Si no aparece 'Añadir nota', conecta sin nota y manda este texto al aceptar. ATENCIÓN: Joel lo hace a mano.</t>
+        </is>
+      </c>
+      <c r="K12" s="17" t="n"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="21" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>lun</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>cuando puedas</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>Whitehaven AFC (Juniors Girls U13-U15)</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>LinkedIn: conectar</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>Luke Johnston (Chairman, Whitehaven AFC)</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>(nota de conexión)</t>
+        </is>
+      </c>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>Hi Luke, I'm Joel, founder of Always Up. We help youth clubs train in Spain with Atlético de Madrid and Real Sociedad. I emailed you recently and wanted to connect here too. Best, Joel</t>
+        </is>
+      </c>
+      <c r="J13" s="17" t="inlineStr">
+        <is>
+          <t>A mano en LinkedIn (no automatizar): perfil de la persona &gt; Conectar &gt; Añadir nota &gt; pegar. Máx. 300 caracteres. Si no aparece 'Añadir nota', conecta sin nota y manda este texto al aceptar. ATENCIÓN: Joel lo hace a mano.</t>
+        </is>
+      </c>
+      <c r="K13" s="17" t="n"/>
+    </row>
+    <row r="14" ht="255" customHeight="1">
+      <c r="A14" s="22" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>mar</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="inlineStr">
+        <is>
+          <t>Hastings United (Girls Academy)</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="inlineStr">
+        <is>
+          <t>Follow-up 1</t>
+        </is>
+      </c>
+      <c r="G14" s="23" t="inlineStr">
+        <is>
+          <t>georgia.townsend@hastingsunited.com</t>
+        </is>
+      </c>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>Re: Bringing Hastings United's Girls Academy to train with LaLiga clubs in Spain</t>
+        </is>
+      </c>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>Hi Georgia,
+Following up on my note from last week, in case it got buried.
+To make it concrete: a typical week with us is 5 days in Madrid, with training sessions, matches against local academy teams, a tour of the Metropolitano stadium and museum, and full accommodation and meals, all organised by us.
+If you're considering Easter or summer 2027, it's a good moment to look at dates while there is flexibility.
+Would a short call work, or shall I send a one-page overview?
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J14" s="23" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K14" s="23" t="n"/>
+    </row>
+    <row r="15" ht="255" customHeight="1">
+      <c r="A15" s="22" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>mar</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
+          <t>Home Farm FC (chicas U13-U15)</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>Follow-up 1</t>
+        </is>
+      </c>
+      <c r="G15" s="23" t="inlineStr">
+        <is>
+          <t>homefarmfc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>Re: Bringing Home Farm FC to train with Atlético de Madrid &amp; Real Sociedad in Spain</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>Hi all,
+Following up on my note from last week, in case it got buried.
+To make it concrete: a typical week with us is 5 days in Madrid, with training sessions, matches against local academy teams, a tour of the Metropolitano stadium and museum, and full accommodation and meals, all organised by us.
+If you're considering Easter or summer 2027, it's a good moment to look at dates while there is flexibility.
+Would a short call work, or shall I send a one-page overview?
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J15" s="23" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K15" s="23" t="n"/>
+    </row>
+    <row r="16" ht="255" customHeight="1">
+      <c r="A16" s="22" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>mié</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E16" s="23" t="inlineStr">
+        <is>
+          <t>Holbeach United</t>
+        </is>
+      </c>
+      <c r="F16" s="23" t="inlineStr">
+        <is>
+          <t>Follow-up 1</t>
+        </is>
+      </c>
+      <c r="G16" s="23" t="inlineStr">
+        <is>
+          <t>callum@holbeachunitedacademy.com</t>
+        </is>
+      </c>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>Re: Training week in Spain for Holbeach United's academy</t>
+        </is>
+      </c>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>Hi Callum,
+Following up on my note from last week, in case it got buried.
+To make it concrete: a typical week with us is 5 days in Madrid, with training sessions, matches against local academy teams, a tour of the Metropolitano stadium and museum, and full accommodation and meals, all organised by us.
+If you're considering Easter or summer 2027, it's a good moment to look at dates while there is flexibility.
+Would a short call work, or shall I send a one-page overview?
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J16" s="23" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K16" s="23" t="n"/>
+    </row>
+    <row r="17" ht="255" customHeight="1">
+      <c r="A17" s="22" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>mié</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="inlineStr">
+        <is>
+          <t>Søreide IL</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>Follow-up 1</t>
+        </is>
+      </c>
+      <c r="G17" s="23" t="inlineStr">
+        <is>
+          <t>fotball@soreideil.no</t>
+        </is>
+      </c>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>Re: Training week in Spain for Søreide IL's youth teams</t>
+        </is>
+      </c>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>Hi Marius and Gunn,
+Following up on my note from last week, in case it got buried.
+To make it concrete: a typical week with us is 5 days in Madrid, with training sessions, matches against local academy teams, a tour of the Metropolitano stadium and museum, and full accommodation and meals, all organised by us.
+If you're considering Easter or summer 2027, it's a good moment to look at dates while there is flexibility.
+Would a short call work, or shall I send a one-page overview?
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J17" s="23" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K17" s="23" t="n"/>
+    </row>
+    <row r="18" ht="225" customHeight="1">
+      <c r="A18" s="22" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>IA Akranes</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>Follow-up 1</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="inlineStr">
+        <is>
+          <t>kfia@ia.is</t>
+        </is>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>Re: Question about youth trips to Spain</t>
+        </is>
+      </c>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>Hi ÍA team,
+Following up on my note from last week, in case it got buried.
+I'm trying to reach whoever organises trips and tours for the youth teams. If that's not you, a name or a forward would be very much appreciated.
+In short: a 5-day week in Madrid with training sessions, matches against local academy teams, a tour of the Metropolitano stadium and museum, and full accommodation and meals, all organised by us.
+Thanks a lot,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J18" s="23" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K18" s="23" t="n"/>
+    </row>
+    <row r="19" ht="225" customHeight="1">
+      <c r="A19" s="22" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E19" s="23" t="inlineStr">
+        <is>
+          <t>Maidstone United (Girls Development Centre)</t>
+        </is>
+      </c>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>Follow-up 1</t>
+        </is>
+      </c>
+      <c r="G19" s="23" t="inlineStr">
+        <is>
+          <t>info@maidstoneunited.co.uk</t>
+        </is>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>Re: Question about the Girls Development Centre</t>
+        </is>
+      </c>
+      <c r="I19" s="23" t="inlineStr">
+        <is>
+          <t>Hi team,
+Following up on my note from last week, in case it got buried.
+I'm trying to reach whoever organises trips and tours for the youth teams. If that's not you, a name or a forward would be very much appreciated.
+In short: a 5-day week in Madrid with training sessions, matches against local academy teams, a tour of the Metropolitano stadium and museum, and full accommodation and meals, all organised by us.
+Thanks a lot,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J19" s="23" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K19" s="23" t="n"/>
+    </row>
+    <row r="20" ht="255" customHeight="1">
+      <c r="A20" s="22" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t>Whitehaven AFC (Juniors Girls U13-U15)</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="inlineStr">
+        <is>
+          <t>Follow-up 1</t>
+        </is>
+      </c>
+      <c r="G20" s="23" t="inlineStr">
+        <is>
+          <t>Luke.johnston@whitehavenafc.com</t>
+        </is>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>Re: Training week in Spain for Whitehaven's girls teams</t>
+        </is>
+      </c>
+      <c r="I20" s="23" t="inlineStr">
+        <is>
+          <t>Hi Luke,
+Following up on my note from last week, in case it got buried.
+To make it concrete: a typical week with us is 5 days in Madrid, with training sessions, matches against local academy teams, a tour of the Metropolitano stadium and museum, and full accommodation and meals, all organised by us.
+If you're considering Easter or summer 2027, it's a good moment to look at dates while there is flexibility.
+Would a short call work, or shall I send a one-page overview?
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J20" s="23" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K20" s="23" t="n"/>
+    </row>
+    <row r="21" ht="195" customHeight="1">
+      <c r="A21" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B21" s="25" t="inlineStr">
+        <is>
+          <t>mar</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D21" s="25" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="E21" s="25" t="inlineStr">
+        <is>
+          <t>Hastings United (Girls Academy)</t>
+        </is>
+      </c>
+      <c r="F21" s="25" t="inlineStr">
+        <is>
+          <t>Follow-up 2</t>
+        </is>
+      </c>
+      <c r="G21" s="25" t="inlineStr">
+        <is>
+          <t>georgia.townsend@hastingsunited.com</t>
+        </is>
+      </c>
+      <c r="H21" s="25" t="inlineStr">
+        <is>
+          <t>Re: Bringing Hastings United's Girls Academy to train with LaLiga clubs in Spain</t>
+        </is>
+      </c>
+      <c r="I21" s="25" t="inlineStr">
+        <is>
+          <t>Hi Georgia,
+I'll keep this short. Most clubs aren't sure at first whether a trip like this is realistic for their families and calendar, and that's fair.
+A 15-minute call is enough to tell you whether it fits, with no commitment. If it's not the right time, just let me know and I'll check back in the new year.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J21" s="25" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K21" s="25" t="n"/>
+    </row>
+    <row r="22" ht="195" customHeight="1">
+      <c r="A22" s="24" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B22" s="25" t="inlineStr">
+        <is>
+          <t>mar</t>
+        </is>
+      </c>
+      <c r="C22" s="25" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D22" s="25" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="E22" s="25" t="inlineStr">
+        <is>
+          <t>Home Farm FC (chicas U13-U15)</t>
+        </is>
+      </c>
+      <c r="F22" s="25" t="inlineStr">
+        <is>
+          <t>Follow-up 2</t>
+        </is>
+      </c>
+      <c r="G22" s="25" t="inlineStr">
+        <is>
+          <t>homefarmfc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H22" s="25" t="inlineStr">
+        <is>
+          <t>Re: Bringing Home Farm FC to train with Atlético de Madrid &amp; Real Sociedad in Spain</t>
+        </is>
+      </c>
+      <c r="I22" s="25" t="inlineStr">
+        <is>
+          <t>Hi all,
+I'll keep this short. Most clubs aren't sure at first whether a trip like this is realistic for their families and calendar, and that's fair.
+A 15-minute call is enough to tell you whether it fits, with no commitment. If it's not the right time, just let me know and I'll check back in the new year.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J22" s="25" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K22" s="25" t="n"/>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="21" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>mié</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>cuando puedas</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>Hastings United (Girls Academy)</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>DM en redes (opcional)</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="inlineStr">
+        <is>
+          <t>Instagram de Hastings United</t>
+        </is>
+      </c>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>(mensaje directo)</t>
+        </is>
+      </c>
+      <c r="I23" s="17" t="inlineStr">
+        <is>
+          <t>Hi! I'm Joel from Always Up. We organise training weeks in Spain for youth clubs (Atlético de Madrid, Real Sociedad). I emailed the club recently. Who is the best person to talk to about trips for the youth teams?</t>
+        </is>
+      </c>
+      <c r="J23" s="17" t="inlineStr">
+        <is>
+          <t>A mano, desde la cuenta del club en la red social indicada. Solo si NO ha contestado al email 2. Mensaje corto, sin enlaces. ATENCIÓN: Solo si no hay respuesta al follow-up 2.</t>
+        </is>
+      </c>
+      <c r="K23" s="17" t="n"/>
+    </row>
+    <row r="24" ht="195" customHeight="1">
+      <c r="A24" s="24" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B24" s="25" t="inlineStr">
+        <is>
+          <t>mié</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D24" s="25" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="E24" s="25" t="inlineStr">
+        <is>
+          <t>Holbeach United</t>
+        </is>
+      </c>
+      <c r="F24" s="25" t="inlineStr">
+        <is>
+          <t>Follow-up 2</t>
+        </is>
+      </c>
+      <c r="G24" s="25" t="inlineStr">
+        <is>
+          <t>callum@holbeachunitedacademy.com</t>
+        </is>
+      </c>
+      <c r="H24" s="25" t="inlineStr">
+        <is>
+          <t>Re: Training week in Spain for Holbeach United's academy</t>
+        </is>
+      </c>
+      <c r="I24" s="25" t="inlineStr">
+        <is>
+          <t>Hi Callum,
+I'll keep this short. Most clubs aren't sure at first whether a trip like this is realistic for their families and calendar, and that's fair.
+A 15-minute call is enough to tell you whether it fits, with no commitment. If it's not the right time, just let me know and I'll check back in the new year.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J24" s="25" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K24" s="25" t="n"/>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="21" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>mié</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>cuando puedas</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>Home Farm FC (chicas U13-U15)</t>
+        </is>
+      </c>
+      <c r="F25" s="17" t="inlineStr">
+        <is>
+          <t>DM en redes (opcional)</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="inlineStr">
+        <is>
+          <t>Facebook/Instagram de Home Farm FC</t>
+        </is>
+      </c>
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t>(mensaje directo)</t>
+        </is>
+      </c>
+      <c r="I25" s="17" t="inlineStr">
+        <is>
+          <t>Hi! I'm Joel from Always Up. We organise training weeks in Spain for youth clubs (Atlético de Madrid, Real Sociedad). I emailed the club recently. Who is the best person to talk to about trips for the youth teams?</t>
+        </is>
+      </c>
+      <c r="J25" s="17" t="inlineStr">
+        <is>
+          <t>A mano, desde la cuenta del club en la red social indicada. Solo si NO ha contestado al email 2. Mensaje corto, sin enlaces. ATENCIÓN: Solo si no hay respuesta al follow-up 2.</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="n"/>
+    </row>
+    <row r="26" ht="195" customHeight="1">
+      <c r="A26" s="24" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B26" s="25" t="inlineStr">
+        <is>
+          <t>mié</t>
+        </is>
+      </c>
+      <c r="C26" s="25" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D26" s="25" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E26" s="25" t="inlineStr">
+        <is>
+          <t>Søreide IL</t>
+        </is>
+      </c>
+      <c r="F26" s="25" t="inlineStr">
+        <is>
+          <t>Follow-up 2</t>
+        </is>
+      </c>
+      <c r="G26" s="25" t="inlineStr">
+        <is>
+          <t>fotball@soreideil.no</t>
+        </is>
+      </c>
+      <c r="H26" s="25" t="inlineStr">
+        <is>
+          <t>Re: Training week in Spain for Søreide IL's youth teams</t>
+        </is>
+      </c>
+      <c r="I26" s="25" t="inlineStr">
+        <is>
+          <t>Hi Marius and Gunn,
+I'll keep this short. Most clubs aren't sure at first whether a trip like this is realistic for their families and calendar, and that's fair.
+A 15-minute call is enough to tell you whether it fits, with no commitment. If it's not the right time, just let me know and I'll check back in the new year.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J26" s="25" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K26" s="25" t="n"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="21" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>cuando puedas</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>Holbeach United</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>DM en redes (opcional)</t>
+        </is>
+      </c>
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>Instagram @holbeachunitedcsa</t>
+        </is>
+      </c>
+      <c r="H27" s="17" t="inlineStr">
+        <is>
+          <t>(mensaje directo)</t>
+        </is>
+      </c>
+      <c r="I27" s="17" t="inlineStr">
+        <is>
+          <t>Hi! I'm Joel from Always Up. We organise training weeks in Spain for youth clubs (Atlético de Madrid, Real Sociedad). I emailed the club recently. Who is the best person to talk to about trips for the youth teams?</t>
+        </is>
+      </c>
+      <c r="J27" s="17" t="inlineStr">
+        <is>
+          <t>A mano, desde la cuenta del club en la red social indicada. Solo si NO ha contestado al email 2. Mensaje corto, sin enlaces. ATENCIÓN: Solo si no hay respuesta al follow-up 2.</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="n"/>
+    </row>
+    <row r="28" ht="195" customHeight="1">
+      <c r="A28" s="24" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B28" s="25" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C28" s="25" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D28" s="25" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="E28" s="25" t="inlineStr">
+        <is>
+          <t>IA Akranes</t>
+        </is>
+      </c>
+      <c r="F28" s="25" t="inlineStr">
+        <is>
+          <t>Follow-up 2</t>
+        </is>
+      </c>
+      <c r="G28" s="25" t="inlineStr">
+        <is>
+          <t>kfia@ia.is</t>
+        </is>
+      </c>
+      <c r="H28" s="25" t="inlineStr">
+        <is>
+          <t>Re: Question about youth trips to Spain</t>
+        </is>
+      </c>
+      <c r="I28" s="25" t="inlineStr">
+        <is>
+          <t>Hi ÍA team,
+I'll keep this short. Most clubs aren't sure at first whether a trip like this is realistic for their families and calendar, and that's fair.
+A 15-minute call is enough to tell you whether it fits, with no commitment. If it's not the right time, just let me know and I'll check back in the new year.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J28" s="25" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K28" s="25" t="n"/>
+    </row>
+    <row r="29" ht="195" customHeight="1">
+      <c r="A29" s="24" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B29" s="25" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C29" s="25" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D29" s="25" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="E29" s="25" t="inlineStr">
+        <is>
+          <t>Maidstone United (Girls Development Centre)</t>
+        </is>
+      </c>
+      <c r="F29" s="25" t="inlineStr">
+        <is>
+          <t>Follow-up 2</t>
+        </is>
+      </c>
+      <c r="G29" s="25" t="inlineStr">
+        <is>
+          <t>info@maidstoneunited.co.uk</t>
+        </is>
+      </c>
+      <c r="H29" s="25" t="inlineStr">
+        <is>
+          <t>Re: Question about the Girls Development Centre</t>
+        </is>
+      </c>
+      <c r="I29" s="25" t="inlineStr">
+        <is>
+          <t>Hi team,
+I'll keep this short. Most clubs aren't sure at first whether a trip like this is realistic for their families and calendar, and that's fair.
+A 15-minute call is enough to tell you whether it fits, with no commitment. If it's not the right time, just let me know and I'll check back in the new year.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J29" s="25" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K29" s="25" t="n"/>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="21" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>cuando puedas</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>Søreide IL</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>DM en redes (opcional)</t>
+        </is>
+      </c>
+      <c r="G30" s="17" t="inlineStr">
+        <is>
+          <t>Facebook/Instagram de Søreide IL</t>
+        </is>
+      </c>
+      <c r="H30" s="17" t="inlineStr">
+        <is>
+          <t>(mensaje directo)</t>
+        </is>
+      </c>
+      <c r="I30" s="17" t="inlineStr">
+        <is>
+          <t>Hi! I'm Joel from Always Up. We organise training weeks in Spain for youth clubs (Atlético de Madrid, Real Sociedad). I emailed the club recently. Who is the best person to talk to about trips for the youth teams?</t>
+        </is>
+      </c>
+      <c r="J30" s="17" t="inlineStr">
+        <is>
+          <t>A mano, desde la cuenta del club en la red social indicada. Solo si NO ha contestado al email 2. Mensaje corto, sin enlaces. ATENCIÓN: Solo si no hay respuesta al follow-up 2.</t>
+        </is>
+      </c>
+      <c r="K30" s="17" t="n"/>
+    </row>
+    <row r="31" ht="195" customHeight="1">
+      <c r="A31" s="24" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B31" s="25" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C31" s="25" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D31" s="25" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="E31" s="25" t="inlineStr">
+        <is>
+          <t>Whitehaven AFC (Juniors Girls U13-U15)</t>
+        </is>
+      </c>
+      <c r="F31" s="25" t="inlineStr">
+        <is>
+          <t>Follow-up 2</t>
+        </is>
+      </c>
+      <c r="G31" s="25" t="inlineStr">
+        <is>
+          <t>Luke.johnston@whitehavenafc.com</t>
+        </is>
+      </c>
+      <c r="H31" s="25" t="inlineStr">
+        <is>
+          <t>Re: Training week in Spain for Whitehaven's girls teams</t>
+        </is>
+      </c>
+      <c r="I31" s="25" t="inlineStr">
+        <is>
+          <t>Hi Luke,
+I'll keep this short. Most clubs aren't sure at first whether a trip like this is realistic for their families and calendar, and that's fair.
+A 15-minute call is enough to tell you whether it fits, with no commitment. If it's not the right time, just let me know and I'll check back in the new year.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J31" s="25" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal.</t>
+        </is>
+      </c>
+      <c r="K31" s="25" t="n"/>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="21" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>vie</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>cuando puedas</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>IA Akranes</t>
+        </is>
+      </c>
+      <c r="F32" s="17" t="inlineStr">
+        <is>
+          <t>DM en redes (opcional)</t>
+        </is>
+      </c>
+      <c r="G32" s="17" t="inlineStr">
+        <is>
+          <t>Facebook/Instagram de ÍA Akranes</t>
+        </is>
+      </c>
+      <c r="H32" s="17" t="inlineStr">
+        <is>
+          <t>(mensaje directo)</t>
+        </is>
+      </c>
+      <c r="I32" s="17" t="inlineStr">
+        <is>
+          <t>Hi! I'm Joel from Always Up. We organise training weeks in Spain for youth clubs (Atlético de Madrid, Real Sociedad). I emailed the club recently. Who is the best person to talk to about trips for the youth teams?</t>
+        </is>
+      </c>
+      <c r="J32" s="17" t="inlineStr">
+        <is>
+          <t>A mano, desde la cuenta del club en la red social indicada. Solo si NO ha contestado al email 2. Mensaje corto, sin enlaces. ATENCIÓN: Solo si no hay respuesta al follow-up 2.</t>
+        </is>
+      </c>
+      <c r="K32" s="17" t="n"/>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="21" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>vie</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>cuando puedas</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>Maidstone United (Girls Development Centre)</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="inlineStr">
+        <is>
+          <t>DM en redes (opcional)</t>
+        </is>
+      </c>
+      <c r="G33" s="17" t="inlineStr">
+        <is>
+          <t>Facebook/Instagram de Maidstone United</t>
+        </is>
+      </c>
+      <c r="H33" s="17" t="inlineStr">
+        <is>
+          <t>(mensaje directo)</t>
+        </is>
+      </c>
+      <c r="I33" s="17" t="inlineStr">
+        <is>
+          <t>Hi! I'm Joel from Always Up. We organise training weeks in Spain for youth clubs (Atlético de Madrid, Real Sociedad). I emailed the club recently. Who is the best person to talk to about trips for the youth teams?</t>
+        </is>
+      </c>
+      <c r="J33" s="17" t="inlineStr">
+        <is>
+          <t>A mano, desde la cuenta del club en la red social indicada. Solo si NO ha contestado al email 2. Mensaje corto, sin enlaces. ATENCIÓN: Solo si no hay respuesta al follow-up 2.</t>
+        </is>
+      </c>
+      <c r="K33" s="17" t="n"/>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="21" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>vie</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>cuando puedas</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>Whitehaven AFC (Juniors Girls U13-U15)</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>DM en redes (opcional)</t>
+        </is>
+      </c>
+      <c r="G34" s="17" t="inlineStr">
+        <is>
+          <t>Facebook de Whitehaven AFC</t>
+        </is>
+      </c>
+      <c r="H34" s="17" t="inlineStr">
+        <is>
+          <t>(mensaje directo)</t>
+        </is>
+      </c>
+      <c r="I34" s="17" t="inlineStr">
+        <is>
+          <t>Hi! I'm Joel from Always Up. We organise training weeks in Spain for youth clubs (Atlético de Madrid, Real Sociedad). I emailed the club recently. Who is the best person to talk to about trips for the youth teams?</t>
+        </is>
+      </c>
+      <c r="J34" s="17" t="inlineStr">
+        <is>
+          <t>A mano, desde la cuenta del club en la red social indicada. Solo si NO ha contestado al email 2. Mensaje corto, sin enlaces. ATENCIÓN: Solo si no hay respuesta al follow-up 2.</t>
+        </is>
+      </c>
+      <c r="K34" s="17" t="n"/>
+    </row>
+    <row r="35" ht="225" customHeight="1">
+      <c r="A35" s="26" t="n">
+        <v>46329</v>
+      </c>
+      <c r="B35" s="27" t="inlineStr">
+        <is>
+          <t>mar</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D35" s="27" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E35" s="27" t="inlineStr">
+        <is>
+          <t>Hastings United (Girls Academy)</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="inlineStr">
+        <is>
+          <t>Cierre (último)</t>
+        </is>
+      </c>
+      <c r="G35" s="27" t="inlineStr">
+        <is>
+          <t>georgia.townsend@hastingsunited.com</t>
+        </is>
+      </c>
+      <c r="H35" s="27" t="inlineStr">
+        <is>
+          <t>Re: Bringing Hastings United's Girls Academy to train with LaLiga clubs in Spain</t>
+        </is>
+      </c>
+      <c r="I35" s="27" t="inlineStr">
+        <is>
+          <t>Hi Georgia,
+I haven't heard back, so I'll assume the timing isn't right and I won't keep writing.
+If anything changes, or you'd like the overview for later, just reply to this email.
+Wishing Hastings United a great season.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J35" s="27" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal. ATENCIÓN: Tras esto, pasar a 'Perdido' / 'Retomar en 2027' en el CRM.</t>
+        </is>
+      </c>
+      <c r="K35" s="27" t="n"/>
+    </row>
+    <row r="36" ht="225" customHeight="1">
+      <c r="A36" s="26" t="n">
+        <v>46329</v>
+      </c>
+      <c r="B36" s="27" t="inlineStr">
+        <is>
+          <t>mar</t>
+        </is>
+      </c>
+      <c r="C36" s="27" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E36" s="27" t="inlineStr">
+        <is>
+          <t>Home Farm FC (chicas U13-U15)</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="inlineStr">
+        <is>
+          <t>Cierre (último)</t>
+        </is>
+      </c>
+      <c r="G36" s="27" t="inlineStr">
+        <is>
+          <t>homefarmfc@gmail.com</t>
+        </is>
+      </c>
+      <c r="H36" s="27" t="inlineStr">
+        <is>
+          <t>Re: Bringing Home Farm FC to train with Atlético de Madrid &amp; Real Sociedad in Spain</t>
+        </is>
+      </c>
+      <c r="I36" s="27" t="inlineStr">
+        <is>
+          <t>Hi all,
+I haven't heard back, so I'll assume the timing isn't right and I won't keep writing.
+If anything changes, or you'd like the overview for later, just reply to this email.
+Wishing Home Farm FC a great season.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J36" s="27" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal. ATENCIÓN: Tras esto, pasar a 'Perdido' / 'Retomar en 2027' en el CRM.</t>
+        </is>
+      </c>
+      <c r="K36" s="27" t="n"/>
+    </row>
+    <row r="37" ht="225" customHeight="1">
+      <c r="A37" s="26" t="n">
+        <v>46330</v>
+      </c>
+      <c r="B37" s="27" t="inlineStr">
+        <is>
+          <t>mié</t>
+        </is>
+      </c>
+      <c r="C37" s="27" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D37" s="27" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E37" s="27" t="inlineStr">
+        <is>
+          <t>Holbeach United</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="inlineStr">
+        <is>
+          <t>Cierre (último)</t>
+        </is>
+      </c>
+      <c r="G37" s="27" t="inlineStr">
+        <is>
+          <t>callum@holbeachunitedacademy.com</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="inlineStr">
+        <is>
+          <t>Re: Training week in Spain for Holbeach United's academy</t>
+        </is>
+      </c>
+      <c r="I37" s="27" t="inlineStr">
+        <is>
+          <t>Hi Callum,
+I haven't heard back, so I'll assume the timing isn't right and I won't keep writing.
+If anything changes, or you'd like the overview for later, just reply to this email.
+Wishing Holbeach United a great season.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J37" s="27" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal. ATENCIÓN: Tras esto, pasar a 'Perdido' / 'Retomar en 2027' en el CRM.</t>
+        </is>
+      </c>
+      <c r="K37" s="27" t="n"/>
+    </row>
+    <row r="38" ht="225" customHeight="1">
+      <c r="A38" s="26" t="n">
+        <v>46330</v>
+      </c>
+      <c r="B38" s="27" t="inlineStr">
+        <is>
+          <t>mié</t>
+        </is>
+      </c>
+      <c r="C38" s="27" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D38" s="27" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="E38" s="27" t="inlineStr">
+        <is>
+          <t>Søreide IL</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="inlineStr">
+        <is>
+          <t>Cierre (último)</t>
+        </is>
+      </c>
+      <c r="G38" s="27" t="inlineStr">
+        <is>
+          <t>fotball@soreideil.no</t>
+        </is>
+      </c>
+      <c r="H38" s="27" t="inlineStr">
+        <is>
+          <t>Re: Training week in Spain for Søreide IL's youth teams</t>
+        </is>
+      </c>
+      <c r="I38" s="27" t="inlineStr">
+        <is>
+          <t>Hi Marius and Gunn,
+I haven't heard back, so I'll assume the timing isn't right and I won't keep writing.
+If anything changes, or you'd like the overview for later, just reply to this email.
+Wishing Søreide IL a great season.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J38" s="27" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal. ATENCIÓN: Tras esto, pasar a 'Perdido' / 'Retomar en 2027' en el CRM.</t>
+        </is>
+      </c>
+      <c r="K38" s="27" t="n"/>
+    </row>
+    <row r="39" ht="225" customHeight="1">
+      <c r="A39" s="26" t="n">
+        <v>46331</v>
+      </c>
+      <c r="B39" s="27" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C39" s="27" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D39" s="27" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E39" s="27" t="inlineStr">
+        <is>
+          <t>IA Akranes</t>
+        </is>
+      </c>
+      <c r="F39" s="27" t="inlineStr">
+        <is>
+          <t>Cierre (último)</t>
+        </is>
+      </c>
+      <c r="G39" s="27" t="inlineStr">
+        <is>
+          <t>kfia@ia.is</t>
+        </is>
+      </c>
+      <c r="H39" s="27" t="inlineStr">
+        <is>
+          <t>Re: Question about youth trips to Spain</t>
+        </is>
+      </c>
+      <c r="I39" s="27" t="inlineStr">
+        <is>
+          <t>Hi ÍA team,
+I haven't heard back, so I'll assume the timing isn't right and I won't keep writing.
+If anything changes, or you'd like the overview for later, just reply to this email.
+Wishing ÍA Akranes a great season.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J39" s="27" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal. ATENCIÓN: Tras esto, pasar a 'Perdido' / 'Retomar en 2027' en el CRM.</t>
+        </is>
+      </c>
+      <c r="K39" s="27" t="n"/>
+    </row>
+    <row r="40" ht="225" customHeight="1">
+      <c r="A40" s="26" t="n">
+        <v>46331</v>
+      </c>
+      <c r="B40" s="27" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C40" s="27" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D40" s="27" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E40" s="27" t="inlineStr">
+        <is>
+          <t>Maidstone United (Girls Development Centre)</t>
+        </is>
+      </c>
+      <c r="F40" s="27" t="inlineStr">
+        <is>
+          <t>Cierre (último)</t>
+        </is>
+      </c>
+      <c r="G40" s="27" t="inlineStr">
+        <is>
+          <t>info@maidstoneunited.co.uk</t>
+        </is>
+      </c>
+      <c r="H40" s="27" t="inlineStr">
+        <is>
+          <t>Re: Question about the Girls Development Centre</t>
+        </is>
+      </c>
+      <c r="I40" s="27" t="inlineStr">
+        <is>
+          <t>Hi team,
+I haven't heard back, so I'll assume the timing isn't right and I won't keep writing.
+If anything changes, or you'd like the overview for later, just reply to this email.
+Wishing Maidstone United a great season.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J40" s="27" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal. ATENCIÓN: Tras esto, pasar a 'Perdido' / 'Retomar en 2027' en el CRM.</t>
+        </is>
+      </c>
+      <c r="K40" s="27" t="n"/>
+    </row>
+    <row r="41" ht="225" customHeight="1">
+      <c r="A41" s="26" t="n">
+        <v>46331</v>
+      </c>
+      <c r="B41" s="27" t="inlineStr">
+        <is>
+          <t>jue</t>
+        </is>
+      </c>
+      <c r="C41" s="27" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D41" s="27" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E41" s="27" t="inlineStr">
+        <is>
+          <t>Whitehaven AFC (Juniors Girls U13-U15)</t>
+        </is>
+      </c>
+      <c r="F41" s="27" t="inlineStr">
+        <is>
+          <t>Cierre (último)</t>
+        </is>
+      </c>
+      <c r="G41" s="27" t="inlineStr">
+        <is>
+          <t>Luke.johnston@whitehavenafc.com</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="inlineStr">
+        <is>
+          <t>Re: Training week in Spain for Whitehaven's girls teams</t>
+        </is>
+      </c>
+      <c r="I41" s="27" t="inlineStr">
+        <is>
+          <t>Hi Luke,
+I haven't heard back, so I'll assume the timing isn't right and I won't keep writing.
+If anything changes, or you'd like the overview for later, just reply to this email.
+Wishing Whitehaven AFC a great season.
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
+      <c r="J41" s="27" t="inlineStr">
+        <is>
+          <t>Responde DENTRO del hilo del email anterior (carpeta Enviados &gt; abrir el correo &gt; Responder), no un correo nuevo. Sin adjuntos. Comprueba antes en el CRM que no ha contestado por otro canal. ATENCIÓN: Tras esto, pasar a 'Perdido' / 'Retomar en 2027' en el CRM.</t>
+        </is>
+      </c>
+      <c r="K41" s="27" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:K2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1136,13 +3375,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1315,7 +3554,7 @@
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>Follow-up 1 el 27/10/2026 si no responde (mensaje corto que aporte algo, sin adjuntos). Si responde con interés: ficha Team Experience</t>
+          <t>Follow-up 1 el 20/10/2026 (en el mismo hilo). Textos en hoja 'Outreach - Copiar y pegar'.</t>
         </is>
       </c>
       <c r="K6" s="12" t="inlineStr">
@@ -1380,39 +3619,41 @@
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Comité juvenil del club</t>
+          <t>Marius Engen / Gunn Eklund Breisnes</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>ungdomsutvalget@soreideil.no</t>
+          <t>fotball@soreideil.no</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>Enviado</t>
+          <t>Listo para enviar</t>
         </is>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>Follow-up 1 el 27/10/2026 si no responde (mensaje corto que aporte algo, sin adjuntos). Si responde con interés: ficha Team Experience</t>
+          <t>Enviar el 14/10/2026 a las 09:30 hora local (Outlook: programar envío). Texto en hoja 'Outreach - Copiar y pegar'.</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr">
         <is>
-          <t>Bringing Søreide IL to train with LaLiga clubs in Spain</t>
+          <t>Training week in Spain for Søreide IL's youth teams</t>
         </is>
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>Hi,
-I'm Joel, I run Always Up — we bring international youth clubs to Spain to train directly at the facilities of Atletico de Madrid, Real Sociedad and Sporting de Gijon.
-I saw Søreide IL is a confirmed participant in the Costa Daurada Cup 2026 and thought this could be a great fit for your squad.
-One of our longtime partner clubs credited their first-ever league title partly to their Atletico de Madrid experience with us — and with Spain now World Cup Champions, interest in trips like this is only growing.
-Would you have 15 minutes this week to hear more?
+          <t>Hi Marius and Gunn,
+I'm Joel, founder of Always Up. My first email bounced from your youth committee address, so I'm writing to you directly.
+We organise training weeks in Spain for youth clubs: sessions at the facilities of Atlético de Madrid and Real Sociedad, matches against local academy teams, and accommodation and meals included.
+I saw Søreide IL was listed for the Costa Daurada Cup in Salou this summer, so Spain may already be on your radar. A longtime partner club of ours won its first-ever league title after training with us.
+Would you be open to a short call next week, or would you prefer a one-page overview first?
 Best,
-Joel</t>
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
         </is>
       </c>
       <c r="M7" s="13" t="n">
@@ -1423,7 +3664,7 @@
       </c>
       <c r="O7" s="12" t="inlineStr">
         <is>
-          <t>También: fotball@soreideil.no (contacto general del club) | Enviado 13/10/2026 a las 15:31 (hora de Nueva York) desde joel.martinez@alwaysup.es, solo texto, sin firma ni adjuntos</t>
+          <t>13/10/2026: el email 1 REBOTÓ (ungdomsutvalget@soreideil.no reenvía a una cuenta inexistente en bergensskolen.com). Contactos reales (soreideil.no/fotball/kontaktinformasjon): Gunn Eklund Breisnes (Leder), Marius Engen (Sportslig leder), fotball@soreideil.no. Reenvío el 14/10 a fotball@soreideil.no.</t>
         </is>
       </c>
       <c r="P7" s="12" t="inlineStr">
@@ -1465,7 +3706,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Pendiente — solo hay teléfono</t>
+          <t>info@maidstoneunited.co.uk</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
@@ -1475,16 +3716,31 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Pendiente investigar email</t>
+          <t>Listo para enviar</t>
         </is>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>Llamar o buscar contacto vía redes del club</t>
-        </is>
-      </c>
-      <c r="K8" s="12" t="inlineStr"/>
-      <c r="L8" s="12" t="inlineStr"/>
+          <t>Enviar el 15/10/2026 a las 09:30 hora local (Outlook: programar envío). Texto en hoja 'Outreach - Copiar y pegar'.</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>Question about the Girls Development Centre</t>
+        </is>
+      </c>
+      <c r="L8" s="12" t="inlineStr">
+        <is>
+          <t>Hi team,
+I'm Joel, founder of Always Up. We organise training weeks in Spain for youth clubs: sessions at the facilities of Atlético de Madrid and Real Sociedad, matches against local academy teams and a stadium tour, with accommodation and meals included.
+I saw Maidstone United was in the Costa Daurada Cup line-up in Salou this summer and thought your Girls Development Centre could be a great fit. Could you point me to the right person to speak with about trips for the girls' teams?
+A longtime partner club of ours won its first-ever league title after training with us, so I'd be glad to share how it worked for them.
+Thanks a lot,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
       <c r="M8" s="13" t="inlineStr"/>
       <c r="N8" s="13" t="inlineStr"/>
       <c r="O8" s="12" t="inlineStr">
@@ -1526,27 +3782,42 @@
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>Sin nombre confirmado todavía</t>
+          <t>Luke Johnston (Chairman)</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Sin email directo — solo formulario en whitehavenafc.com/contact</t>
+          <t>Luke.johnston@whitehavenafc.com</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Pendiente investigar decisor</t>
+          <t>Listo para enviar</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>Rellenar el formulario de contacto o buscar el nombre del responsable de chicas en redes del club antes de escribir</t>
-        </is>
-      </c>
-      <c r="K9" s="12" t="inlineStr"/>
-      <c r="L9" s="12" t="inlineStr"/>
+          <t>Enviar el 15/10/2026 a las 09:30 hora local (Outlook: programar envío). Texto en hoja 'Outreach - Copiar y pegar'.</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>Training week in Spain for Whitehaven's girls teams</t>
+        </is>
+      </c>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>Hi Luke,
+I'm Joel, founder of Always Up. We organise training weeks in Spain for youth clubs: sessions at the facilities of Atlético de Madrid and Real Sociedad, matches against local academy teams and a stadium tour, with accommodation and meals included.
+I saw Whitehaven AFC was listed for the Costa Daurada Cup in Salou this summer, and the girls pathway (U13-U15) caught my eye. A longtime partner club of ours won its first-ever league title after training with us.
+Would a short call next week work, or would you prefer a one-page overview first? And if you're not the right person, could you point me to whoever organises trips for the girls' section?
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
       <c r="M9" s="13" t="inlineStr"/>
       <c r="N9" s="13" t="inlineStr"/>
       <c r="O9" s="12" t="inlineStr">
@@ -1605,7 +3876,7 @@
       <c r="N10" s="13" t="inlineStr"/>
       <c r="O10" s="12" t="inlineStr">
         <is>
-          <t>Investigado 2026-08-29: posible error de nombre en el research original — no gastar más tiempo hasta verificar en la fuente original</t>
+          <t>Investigado 2026-08-29: posible error de nombre en el research original — no gastar más tiempo hasta verificar en la fuente original | 13/10/2026: costadauradacup.com lo lista como club de Inglaterra en la edición de Semana Santa 2026. Existe: falta encontrar su contacto.</t>
         </is>
       </c>
       <c r="P10" s="12" t="inlineStr">
@@ -1642,12 +3913,12 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Sin nombre confirmado todavía</t>
+          <t>Callum Lawe (Vice Chairman, Football &amp; Education Academy)</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>info@holbeachunitedcsa.org.uk</t>
+          <t>callum@holbeachunitedacademy.com</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -1657,16 +3928,32 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Pendiente investigar decisor</t>
+          <t>Listo para enviar</t>
         </is>
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>Escribir al email general pidiendo hablar con el responsable de viajes/categorías mayores antes de mandar la propuesta completa</t>
-        </is>
-      </c>
-      <c r="K11" s="12" t="inlineStr"/>
-      <c r="L11" s="12" t="inlineStr"/>
+          <t>Enviar el 14/10/2026 a las 09:30 hora local (Outlook: programar envío). Texto en hoja 'Outreach - Copiar y pegar'.</t>
+        </is>
+      </c>
+      <c r="K11" s="12" t="inlineStr">
+        <is>
+          <t>Training week in Spain for Holbeach United's academy</t>
+        </is>
+      </c>
+      <c r="L11" s="12" t="inlineStr">
+        <is>
+          <t>Hi Callum,
+I'm Joel, founder of Always Up. We organise training weeks in Spain for youth clubs: sessions at the facilities of Atlético de Madrid and Real Sociedad, matches against local academy teams and a stadium tour, with accommodation and meals included.
+I saw Holbeach United was listed for the Costa Daurada Cup in Salou this year, and your Football &amp; Education Academy stood out, so I thought a week in Spain could be a good fit for your older squads.
+A longtime partner club of ours won its first-ever league title after training with us, and its coaches credit part of it to the experience.
+Would you be open to a short call next week, or would you prefer I send a one-page overview first?
+Best,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
       <c r="M11" s="13" t="inlineStr"/>
       <c r="N11" s="13" t="inlineStr"/>
       <c r="O11" s="12" t="inlineStr">
@@ -1724,7 +4011,7 @@
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Follow-up 1 el 27/10/2026 si no responde (mensaje corto que aporte algo, sin adjuntos). Si responde con interés: ficha Team Experience</t>
+          <t>Follow-up 1 el 20/10/2026 (en el mismo hilo). Textos en hoja 'Outreach - Copiar y pegar'.</t>
         </is>
       </c>
       <c r="K12" s="12" t="inlineStr">
@@ -1845,20 +4132,39 @@
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr"/>
-      <c r="G14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>kfia@ia.is</t>
+        </is>
+      </c>
       <c r="H14" s="6" t="inlineStr"/>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Pendiente investigar</t>
+          <t>Listo para enviar</t>
         </is>
       </c>
       <c r="J14" s="12" t="inlineStr">
         <is>
-          <t>Investigar contacto (parte de la cuota diaria de 5 búsquedas)</t>
-        </is>
-      </c>
-      <c r="K14" s="12" t="inlineStr"/>
-      <c r="L14" s="12" t="inlineStr"/>
+          <t>Enviar el 15/10/2026 a las 09:30 hora local (Outlook: programar envío). Texto en hoja 'Outreach - Copiar y pegar'.</t>
+        </is>
+      </c>
+      <c r="K14" s="12" t="inlineStr">
+        <is>
+          <t>Question about youth trips to Spain</t>
+        </is>
+      </c>
+      <c r="L14" s="12" t="inlineStr">
+        <is>
+          <t>Hi ÍA team,
+I'm Joel, founder of Always Up. We organise training weeks in Spain for youth clubs: sessions at the facilities of Atlético de Madrid and Real Sociedad, matches against local academy teams and a stadium tour, with accommodation and meals included.
+I saw ÍA Akranes was listed for the Costa Daurada Cup in Salou this year. Could you point me to the person who organises trips abroad for your youth teams (yngri flokkar)?
+A longtime partner club of ours won its first-ever league title after training with us, and its coaches credit part of it to the experience, so I'd be glad to share how it worked for them.
+Thanks a lot,
+Joel Martinez
+Founder, Always Up
+joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
+        </is>
+      </c>
       <c r="M14" s="13" t="inlineStr"/>
       <c r="N14" s="13" t="inlineStr"/>
       <c r="O14" s="12" t="inlineStr"/>
@@ -1911,7 +4217,11 @@
       <c r="L15" s="12" t="inlineStr"/>
       <c r="M15" s="13" t="inlineStr"/>
       <c r="N15" s="13" t="inlineStr"/>
-      <c r="O15" s="12" t="inlineStr"/>
+      <c r="O15" s="12" t="inlineStr">
+        <is>
+          <t>13/10/2026: es un club profesional con academia (Joep Breimer, hoofd voetbalontwikkeling jeugdopleiding). Perfil distinto al club amateur viajero: prioridad baja, no incluir en la primera tanda.</t>
+        </is>
+      </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
           <t>1er email: NADA adjunto, solo texto (firma de texto plano). Si responde con interés: ficha Always-Up-Team-Experience.pdf. Antes de la llamada: deck de empresa (pendiente de crear), solo si hace falta. Tras la llamada: propuesta escrita.</t>
@@ -2047,8 +4357,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
   </sheetData>
   <autoFilter ref="A5:P17"/>
   <mergeCells count="3">
@@ -2060,7 +4368,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2616,13 +4924,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3053,7 +5361,7 @@
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>Follow-up 13/10: lleva 14 días sin responder desde el 29/09; prometió vídeo y datos 'la próxima semana' (5/10) y no ha llegado. Pedir lo que tenga YA (aunque sea el del año pasado + notas) y empezar la primera lectura. NO ofrecer más descuento.</t>
+          <t>Follow-up enviado el 13/10. Si no contesta en 7 días (20/10): un último mensaje corto y pasar a 'frío'. No bajar más el precio.</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -3063,7 +5371,7 @@
       </c>
       <c r="J12" s="12" t="inlineStr">
         <is>
-          <t>Llamada realizada 15/09/2026. Resultado: la familia lo va a valorar 'en los próximos días', Joel manda evaluación/propuesta cuando den el okay. Joel ya envió foto de precios por WhatsApp + mensaje de cierre de llamada. Pendiente: confirmar si ya tienen el vídeo en mano, y si se aclaró en la llamada si buscan la misma universidad para los dos gemelos o están abiertos a separarse. | 17/09 objeción: precio alto 'x2', quiere evaluación antes de decidir (qué beca y qué división). 18/09 oferta de Joel por niño: pago único $2.000 (en vez de $2.500) o 2 plazos $250 + $2.500 (en vez de $3.500). 27/09 Omar: 'la próxima semana te envío vídeo y datos'. Sin datos desde entonces.</t>
+          <t>Llamada realizada 15/09/2026. Resultado: la familia lo va a valorar 'en los próximos días', Joel manda evaluación/propuesta cuando den el okay. Joel ya envió foto de precios por WhatsApp + mensaje de cierre de llamada. Pendiente: confirmar si ya tienen el vídeo en mano, y si se aclaró en la llamada si buscan la misma universidad para los dos gemelos o están abiertos a separarse. | 17/09 objeción: precio alto 'x2', quiere evaluación antes de decidir (qué beca y qué división). 18/09 oferta de Joel por niño: pago único $2.000 (en vez de $2.500) o 2 plazos $250 + $2.500 (en vez de $3.500). 27/09 Omar: 'la próxima semana te envío vídeo y datos'. Sin datos desde entonces. | 13/10: Joel envió el follow-up pidiendo vídeo/datos con salida elegante.</t>
         </is>
       </c>
       <c r="K12" s="12" t="inlineStr">
@@ -3484,7 +5792,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
   </sheetData>
   <autoFilter ref="A5:K20"/>
   <mergeCells count="3">
@@ -3496,7 +5803,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3657,7 +5964,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Instrucciones de envio adaptadas a correo Hostinger (sin programar en Outlook) y plan B a las 07:30 NY
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -820,7 +820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -868,7 +868,7 @@
       </c>
       <c r="B6" s="32" t="inlineStr">
         <is>
-          <t>Programa en Outlook los correos del día siguiente. El calendario te dice cuáles, a qué hora de Nueva York y de dónde copiar el texto.</t>
+          <t>Prepara los correos del día siguiente. Si tu correo permite programar, déjalos programados. Si no, los envías a mano a las 07:30 de Nueva York. El calendario te dice cuáles y de dónde copiar el texto.</t>
         </is>
       </c>
     </row>
@@ -990,84 +990,120 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="30" t="inlineStr">
         <is>
-          <t>COMO PROGRAMAR UN CORREO EN OUTLOOK</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="47.5" customHeight="1">
+          <t>COMO ENVIAR A LA HORA CORRECTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="33" customHeight="1">
       <c r="A18" s="31" t="inlineStr">
         <is>
-          <t>Paso a paso</t>
+          <t>Tu correo</t>
         </is>
       </c>
       <c r="B18" s="32" t="inlineStr">
         <is>
-          <t>Nuevo correo &gt; pega Para, Asunto y Texto &gt; flecha junto a Enviar &gt; Programar envío &gt; elige fecha y hora de Nueva York. Si usas Outlook de escritorio clásico, el ordenador debe estar encendido a esa hora. Con Outlook web o el Outlook nuevo sale solo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="33" customHeight="1">
+          <t>joel.martinez@alwaysup.es está alojado en Hostinger, no en Microsoft. Outlook conectado a ese tipo de cuenta (IMAP) NO tiene 'Programar envío': ese botón solo funciona con cuentas de Microsoft. Por eso no lo veías.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="47.5" customHeight="1">
       <c r="A19" s="31" t="inlineStr">
         <is>
-          <t>Por qué a las 09:30 locales</t>
+          <t>Opción 1 (la mejor)</t>
         </is>
       </c>
       <c r="B19" s="32" t="inlineStr">
         <is>
-          <t>Es el momento en que el responsable del club abre el correo en su jornada. Martes a jueves funcionan mejor que lunes (bandeja llena) y viernes (desconectan).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="30" t="inlineStr">
-        <is>
-          <t>REGLAS QUE NO SE ROMPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="33" customHeight="1">
+          <t>Entra al webmail de Hostinger (hpanel.hostinger.com &gt; Correo electrónico &gt; Abrir webmail, o mail.hostinger.com) con tu cuenta. Ahí, junto al botón Enviar, suele haber una flecha con 'Programar envío'. Funciona desde el servidor, aunque tu ordenador esté apagado. Pruébalo con un correo a ti mismo antes de usarlo con un club.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="47.5" customHeight="1">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>Opción 2</t>
+        </is>
+      </c>
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t>Outlook de escritorio clásico: en el correo, pestaña Opciones &gt; Retrasar entrega &gt; 'No entregar antes de' + fecha y hora. Funciona, pero Outlook debe estar abierto y el ordenador encendido a esa hora. Outlook nuevo y Outlook web no tienen esta opción para cuentas IMAP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="47.5" customHeight="1">
       <c r="A21" s="31" t="inlineStr">
         <is>
-          <t>Nunca</t>
+          <t>Plan B (sin programar)</t>
         </is>
       </c>
       <c r="B21" s="32" t="inlineStr">
         <is>
-          <t>Adjuntos en el primer correo. Nombrar al partner de becas. Prometer becas o fichajes. Inventar urgencia. Discutir precio por escrito sin tu decisión.</t>
+          <t>Envíalo tú a mano a las 07:30 de Nueva York. Son las 12:30 o 13:30 en Reino Unido, Irlanda, Noruega o Islandia: sigue siendo horario laboral, solo que a media mañana o mediodía en vez de a primera hora. La diferencia de respuesta es pequeña: no vale la pena perder un envío por esto.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="33" customHeight="1">
       <c r="A22" s="31" t="inlineStr">
         <is>
-          <t>Si contestan</t>
+          <t>Regla</t>
         </is>
       </c>
       <c r="B22" s="32" t="inlineStr">
         <is>
-          <t>Paras la cadencia de ese club y abres 'Respuestas tipo' (hoja Textos para copiar). Menos de 4 horas de respuesta en horario del club.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="31" t="inlineStr">
-        <is>
-          <t>Si un correo rebota</t>
-        </is>
-      </c>
-      <c r="B23" s="32" t="inlineStr">
-        <is>
-          <t>Me lo dices; busco otra dirección del club y te la dejo preparada.</t>
+          <t>Lo importante es enviar martes a jueves en horario laboral del club. La hora exacta de las 09:30 es una mejora, no una condición.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>REGLAS QUE NO SE ROMPEN</t>
         </is>
       </c>
     </row>
     <row r="24" ht="33" customHeight="1">
       <c r="A24" s="31" t="inlineStr">
         <is>
+          <t>Nunca</t>
+        </is>
+      </c>
+      <c r="B24" s="32" t="inlineStr">
+        <is>
+          <t>Adjuntos en el primer correo. Nombrar al partner de becas. Prometer becas o fichajes. Inventar urgencia. Discutir precio por escrito sin tu decisión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="33" customHeight="1">
+      <c r="A25" s="31" t="inlineStr">
+        <is>
+          <t>Si contestan</t>
+        </is>
+      </c>
+      <c r="B25" s="32" t="inlineStr">
+        <is>
+          <t>Paras la cadencia de ese club y abres 'Respuestas tipo' (hoja Textos para copiar). Menos de 4 horas de respuesta en horario del club.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="31" t="inlineStr">
+        <is>
+          <t>Si un correo rebota</t>
+        </is>
+      </c>
+      <c r="B26" s="32" t="inlineStr">
+        <is>
+          <t>Me lo dices; busco otra dirección del club y te la dejo preparada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="33" customHeight="1">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
           <t>Colores</t>
         </is>
       </c>
-      <c r="B24" s="32" t="inlineStr">
+      <c r="B27" s="32" t="inlineStr">
         <is>
           <t>Azul claro = email 1, amarillo = follow-up 1, naranja = follow-up 2, gris = cierre, lila = LinkedIn o redes, rojo = pendiente atrasado.</t>
         </is>
@@ -1076,8 +1112,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A20:B20"/>
     <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="A17:B17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1896,7 +1932,7 @@
       </c>
       <c r="J7" s="39" t="n"/>
     </row>
-    <row r="8" ht="149" customHeight="1">
+    <row r="8" ht="134.5" customHeight="1">
       <c r="A8" s="38" t="n">
         <v>46308</v>
       </c>
@@ -1917,15 +1953,14 @@
       </c>
       <c r="E8" s="31" t="inlineStr">
         <is>
-          <t>Programar en Outlook los envíos del miércoles 14/10</t>
+          <t>Preparar (y programar si puedes) los envíos del miércoles 14/10</t>
         </is>
       </c>
       <c r="F8" s="39" t="inlineStr">
         <is>
-          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 14/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada.
+          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 14/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada si tu correo lo permite (ver LEEME). Si no puedes programar, no pasa nada: mañana a las 07:30 de Nueva York los envías a mano.
 • Holbeach United | Email 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 14/10.
-• Søreide IL | Email 1 | programar para las 03:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 14/10.
-Importante: si usas Outlook de escritorio clásico, el ordenador debe estar encendido y con Outlook abierto a esa hora; con Outlook web o el Outlook nuevo, el envío sale solo desde el servidor.</t>
+• Søreide IL | Email 1 | programar para las 03:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 14/10.</t>
         </is>
       </c>
       <c r="G8" s="39" t="inlineStr">
@@ -1943,7 +1978,7 @@
       </c>
       <c r="J8" s="39" t="n"/>
     </row>
-    <row r="9" ht="33" customHeight="1">
+    <row r="9" ht="47.5" customHeight="1">
       <c r="A9" s="44" t="n">
         <v>46309</v>
       </c>
@@ -1969,7 +2004,7 @@
       </c>
       <c r="F9" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G9" s="45" t="inlineStr">
@@ -1985,7 +2020,7 @@
       </c>
       <c r="J9" s="45" t="n"/>
     </row>
-    <row r="10" ht="33" customHeight="1">
+    <row r="10" ht="47.5" customHeight="1">
       <c r="A10" s="44" t="n">
         <v>46309</v>
       </c>
@@ -2011,7 +2046,7 @@
       </c>
       <c r="F10" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G10" s="45" t="inlineStr">
@@ -2287,7 +2322,7 @@
       </c>
       <c r="J16" s="39" t="n"/>
     </row>
-    <row r="17" ht="178" customHeight="1">
+    <row r="17" ht="163.5" customHeight="1">
       <c r="A17" s="38" t="n">
         <v>46309</v>
       </c>
@@ -2308,16 +2343,15 @@
       </c>
       <c r="E17" s="31" t="inlineStr">
         <is>
-          <t>Programar en Outlook los envíos del jueves 15/10</t>
+          <t>Preparar (y programar si puedes) los envíos del jueves 15/10</t>
         </is>
       </c>
       <c r="F17" s="39" t="inlineStr">
         <is>
-          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 15/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada.
+          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 15/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada si tu correo lo permite (ver LEEME). Si no puedes programar, no pasa nada: mañana a las 07:30 de Nueva York los envías a mano.
 • IA Akranes | Email 1 | programar para las 05:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 15/10.
 • Maidstone United | Email 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 15/10.
-• Whitehaven AFC | Email 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 15/10.
-Importante: si usas Outlook de escritorio clásico, el ordenador debe estar encendido y con Outlook abierto a esa hora; con Outlook web o el Outlook nuevo, el envío sale solo desde el servidor.</t>
+• Whitehaven AFC | Email 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 15/10.</t>
         </is>
       </c>
       <c r="G17" s="39" t="inlineStr">
@@ -2335,7 +2369,7 @@
       </c>
       <c r="J17" s="39" t="n"/>
     </row>
-    <row r="18" ht="33" customHeight="1">
+    <row r="18" ht="47.5" customHeight="1">
       <c r="A18" s="44" t="n">
         <v>46310</v>
       </c>
@@ -2361,7 +2395,7 @@
       </c>
       <c r="F18" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G18" s="45" t="inlineStr">
@@ -2377,7 +2411,7 @@
       </c>
       <c r="J18" s="45" t="n"/>
     </row>
-    <row r="19" ht="33" customHeight="1">
+    <row r="19" ht="47.5" customHeight="1">
       <c r="A19" s="44" t="n">
         <v>46310</v>
       </c>
@@ -2403,7 +2437,7 @@
       </c>
       <c r="F19" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G19" s="45" t="inlineStr">
@@ -2419,7 +2453,7 @@
       </c>
       <c r="J19" s="45" t="n"/>
     </row>
-    <row r="20" ht="33" customHeight="1">
+    <row r="20" ht="47.5" customHeight="1">
       <c r="A20" s="44" t="n">
         <v>46310</v>
       </c>
@@ -2445,7 +2479,7 @@
       </c>
       <c r="F20" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G20" s="45" t="inlineStr">
@@ -3248,7 +3282,7 @@
       </c>
       <c r="J39" s="39" t="n"/>
     </row>
-    <row r="40" ht="207" customHeight="1">
+    <row r="40" ht="192.5" customHeight="1">
       <c r="A40" s="38" t="n">
         <v>46314</v>
       </c>
@@ -3269,17 +3303,16 @@
       </c>
       <c r="E40" s="31" t="inlineStr">
         <is>
-          <t>Programar en Outlook los envíos del martes 20/10</t>
+          <t>Preparar (y programar si puedes) los envíos del martes 20/10</t>
         </is>
       </c>
       <c r="F40" s="39" t="inlineStr">
         <is>
-          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 20/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada.
+          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 20/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada si tu correo lo permite (ver LEEME). Si no puedes programar, no pasa nada: mañana a las 07:30 de Nueva York los envías a mano.
 • FC Porte d'Aquitaine | Email 1 | programar para las 03:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 20/10.
 • Hastings United | Follow-up 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 20/10.
 • Home Farm FC | Follow-up 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 20/10.
-• Virtu Academy | Email 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 20/10.
-Importante: si usas Outlook de escritorio clásico, el ordenador debe estar encendido y con Outlook abierto a esa hora; con Outlook web o el Outlook nuevo, el envío sale solo desde el servidor.</t>
+• Virtu Academy | Email 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 20/10.</t>
         </is>
       </c>
       <c r="G40" s="39" t="inlineStr">
@@ -3297,7 +3330,7 @@
       </c>
       <c r="J40" s="39" t="n"/>
     </row>
-    <row r="41" ht="33" customHeight="1">
+    <row r="41" ht="47.5" customHeight="1">
       <c r="A41" s="44" t="n">
         <v>46315</v>
       </c>
@@ -3323,7 +3356,7 @@
       </c>
       <c r="F41" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G41" s="45" t="inlineStr">
@@ -3339,7 +3372,7 @@
       </c>
       <c r="J41" s="45" t="n"/>
     </row>
-    <row r="42" ht="33" customHeight="1">
+    <row r="42" ht="47.5" customHeight="1">
       <c r="A42" s="44" t="n">
         <v>46315</v>
       </c>
@@ -3365,7 +3398,7 @@
       </c>
       <c r="F42" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G42" s="45" t="inlineStr">
@@ -3381,7 +3414,7 @@
       </c>
       <c r="J42" s="45" t="n"/>
     </row>
-    <row r="43" ht="33" customHeight="1">
+    <row r="43" ht="47.5" customHeight="1">
       <c r="A43" s="44" t="n">
         <v>46315</v>
       </c>
@@ -3407,7 +3440,7 @@
       </c>
       <c r="F43" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G43" s="45" t="inlineStr">
@@ -3423,7 +3456,7 @@
       </c>
       <c r="J43" s="45" t="n"/>
     </row>
-    <row r="44" ht="33" customHeight="1">
+    <row r="44" ht="47.5" customHeight="1">
       <c r="A44" s="44" t="n">
         <v>46315</v>
       </c>
@@ -3449,7 +3482,7 @@
       </c>
       <c r="F44" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G44" s="45" t="inlineStr">
@@ -3597,7 +3630,7 @@
       </c>
       <c r="J47" s="39" t="n"/>
     </row>
-    <row r="48" ht="149" customHeight="1">
+    <row r="48" ht="134.5" customHeight="1">
       <c r="A48" s="38" t="n">
         <v>46315</v>
       </c>
@@ -3618,15 +3651,14 @@
       </c>
       <c r="E48" s="31" t="inlineStr">
         <is>
-          <t>Programar en Outlook los envíos del miércoles 21/10</t>
+          <t>Preparar (y programar si puedes) los envíos del miércoles 21/10</t>
         </is>
       </c>
       <c r="F48" s="39" t="inlineStr">
         <is>
-          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 21/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada.
+          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 21/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada si tu correo lo permite (ver LEEME). Si no puedes programar, no pasa nada: mañana a las 07:30 de Nueva York los envías a mano.
 • Holbeach United | Follow-up 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 21/10.
-• Søreide IL | Follow-up 1 | programar para las 03:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 21/10.
-Importante: si usas Outlook de escritorio clásico, el ordenador debe estar encendido y con Outlook abierto a esa hora; con Outlook web o el Outlook nuevo, el envío sale solo desde el servidor.</t>
+• Søreide IL | Follow-up 1 | programar para las 03:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 21/10.</t>
         </is>
       </c>
       <c r="G48" s="39" t="inlineStr">
@@ -3644,7 +3676,7 @@
       </c>
       <c r="J48" s="39" t="n"/>
     </row>
-    <row r="49" ht="33" customHeight="1">
+    <row r="49" ht="47.5" customHeight="1">
       <c r="A49" s="44" t="n">
         <v>46316</v>
       </c>
@@ -3670,7 +3702,7 @@
       </c>
       <c r="F49" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G49" s="45" t="inlineStr">
@@ -3686,7 +3718,7 @@
       </c>
       <c r="J49" s="45" t="n"/>
     </row>
-    <row r="50" ht="33" customHeight="1">
+    <row r="50" ht="47.5" customHeight="1">
       <c r="A50" s="44" t="n">
         <v>46316</v>
       </c>
@@ -3712,7 +3744,7 @@
       </c>
       <c r="F50" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G50" s="45" t="inlineStr">
@@ -3856,7 +3888,7 @@
       </c>
       <c r="J53" s="39" t="n"/>
     </row>
-    <row r="54" ht="178" customHeight="1">
+    <row r="54" ht="163.5" customHeight="1">
       <c r="A54" s="38" t="n">
         <v>46316</v>
       </c>
@@ -3877,16 +3909,15 @@
       </c>
       <c r="E54" s="31" t="inlineStr">
         <is>
-          <t>Programar en Outlook los envíos del jueves 22/10</t>
+          <t>Preparar (y programar si puedes) los envíos del jueves 22/10</t>
         </is>
       </c>
       <c r="F54" s="39" t="inlineStr">
         <is>
-          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 22/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada.
+          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 22/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada si tu correo lo permite (ver LEEME). Si no puedes programar, no pasa nada: mañana a las 07:30 de Nueva York los envías a mano.
 • IA Akranes | Follow-up 1 | programar para las 05:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 22/10.
 • Maidstone United | Follow-up 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 22/10.
-• Whitehaven AFC | Follow-up 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 22/10.
-Importante: si usas Outlook de escritorio clásico, el ordenador debe estar encendido y con Outlook abierto a esa hora; con Outlook web o el Outlook nuevo, el envío sale solo desde el servidor.</t>
+• Whitehaven AFC | Follow-up 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 22/10.</t>
         </is>
       </c>
       <c r="G54" s="39" t="inlineStr">
@@ -3904,7 +3935,7 @@
       </c>
       <c r="J54" s="39" t="n"/>
     </row>
-    <row r="55" ht="33" customHeight="1">
+    <row r="55" ht="47.5" customHeight="1">
       <c r="A55" s="44" t="n">
         <v>46317</v>
       </c>
@@ -3930,7 +3961,7 @@
       </c>
       <c r="F55" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G55" s="45" t="inlineStr">
@@ -3946,7 +3977,7 @@
       </c>
       <c r="J55" s="45" t="n"/>
     </row>
-    <row r="56" ht="33" customHeight="1">
+    <row r="56" ht="47.5" customHeight="1">
       <c r="A56" s="44" t="n">
         <v>46317</v>
       </c>
@@ -3972,7 +4003,7 @@
       </c>
       <c r="F56" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G56" s="45" t="inlineStr">
@@ -3988,7 +4019,7 @@
       </c>
       <c r="J56" s="45" t="n"/>
     </row>
-    <row r="57" ht="33" customHeight="1">
+    <row r="57" ht="47.5" customHeight="1">
       <c r="A57" s="44" t="n">
         <v>46317</v>
       </c>
@@ -4014,7 +4045,7 @@
       </c>
       <c r="F57" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G57" s="45" t="inlineStr">
@@ -4637,7 +4668,7 @@
       </c>
       <c r="J72" s="39" t="n"/>
     </row>
-    <row r="73" ht="207" customHeight="1">
+    <row r="73" ht="192.5" customHeight="1">
       <c r="A73" s="38" t="n">
         <v>46321</v>
       </c>
@@ -4658,17 +4689,16 @@
       </c>
       <c r="E73" s="31" t="inlineStr">
         <is>
-          <t>Programar en Outlook los envíos del martes 27/10</t>
+          <t>Preparar (y programar si puedes) los envíos del martes 27/10</t>
         </is>
       </c>
       <c r="F73" s="39" t="inlineStr">
         <is>
-          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 27/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada.
+          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 27/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada si tu correo lo permite (ver LEEME). Si no puedes programar, no pasa nada: mañana a las 07:30 de Nueva York los envías a mano.
 • FC Porte d'Aquitaine | Follow-up 1 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 27/10.
 • Hastings United | Follow-up 2 | programar para las 05:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 27/10.
 • Home Farm FC | Follow-up 2 | programar para las 05:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 27/10.
-• Virtu Academy | Follow-up 1 | programar para las 05:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 27/10.
-Importante: si usas Outlook de escritorio clásico, el ordenador debe estar encendido y con Outlook abierto a esa hora; con Outlook web o el Outlook nuevo, el envío sale solo desde el servidor.</t>
+• Virtu Academy | Follow-up 1 | programar para las 05:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 27/10.</t>
         </is>
       </c>
       <c r="G73" s="39" t="inlineStr">
@@ -4686,7 +4716,7 @@
       </c>
       <c r="J73" s="39" t="n"/>
     </row>
-    <row r="74" ht="33" customHeight="1">
+    <row r="74" ht="47.5" customHeight="1">
       <c r="A74" s="44" t="n">
         <v>46322</v>
       </c>
@@ -4712,7 +4742,7 @@
       </c>
       <c r="F74" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G74" s="45" t="inlineStr">
@@ -4728,7 +4758,7 @@
       </c>
       <c r="J74" s="45" t="n"/>
     </row>
-    <row r="75" ht="33" customHeight="1">
+    <row r="75" ht="47.5" customHeight="1">
       <c r="A75" s="44" t="n">
         <v>46322</v>
       </c>
@@ -4754,7 +4784,7 @@
       </c>
       <c r="F75" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G75" s="45" t="inlineStr">
@@ -4770,7 +4800,7 @@
       </c>
       <c r="J75" s="45" t="n"/>
     </row>
-    <row r="76" ht="33" customHeight="1">
+    <row r="76" ht="47.5" customHeight="1">
       <c r="A76" s="44" t="n">
         <v>46322</v>
       </c>
@@ -4796,7 +4826,7 @@
       </c>
       <c r="F76" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G76" s="45" t="inlineStr">
@@ -4812,7 +4842,7 @@
       </c>
       <c r="J76" s="45" t="n"/>
     </row>
-    <row r="77" ht="33" customHeight="1">
+    <row r="77" ht="47.5" customHeight="1">
       <c r="A77" s="44" t="n">
         <v>46322</v>
       </c>
@@ -4838,7 +4868,7 @@
       </c>
       <c r="F77" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G77" s="45" t="inlineStr">
@@ -4986,7 +5016,7 @@
       </c>
       <c r="J80" s="39" t="n"/>
     </row>
-    <row r="81" ht="149" customHeight="1">
+    <row r="81" ht="134.5" customHeight="1">
       <c r="A81" s="38" t="n">
         <v>46322</v>
       </c>
@@ -5007,15 +5037,14 @@
       </c>
       <c r="E81" s="31" t="inlineStr">
         <is>
-          <t>Programar en Outlook los envíos del miércoles 28/10</t>
+          <t>Preparar (y programar si puedes) los envíos del miércoles 28/10</t>
         </is>
       </c>
       <c r="F81" s="39" t="inlineStr">
         <is>
-          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 28/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada.
+          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 28/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada si tu correo lo permite (ver LEEME). Si no puedes programar, no pasa nada: mañana a las 07:30 de Nueva York los envías a mano.
 • Holbeach United | Follow-up 2 | programar para las 05:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 28/10.
-• Søreide IL | Follow-up 2 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 28/10.
-Importante: si usas Outlook de escritorio clásico, el ordenador debe estar encendido y con Outlook abierto a esa hora; con Outlook web o el Outlook nuevo, el envío sale solo desde el servidor.</t>
+• Søreide IL | Follow-up 2 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 28/10.</t>
         </is>
       </c>
       <c r="G81" s="39" t="inlineStr">
@@ -5033,7 +5062,7 @@
       </c>
       <c r="J81" s="39" t="n"/>
     </row>
-    <row r="82" ht="33" customHeight="1">
+    <row r="82" ht="47.5" customHeight="1">
       <c r="A82" s="44" t="n">
         <v>46323</v>
       </c>
@@ -5059,7 +5088,7 @@
       </c>
       <c r="F82" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G82" s="45" t="inlineStr">
@@ -5075,7 +5104,7 @@
       </c>
       <c r="J82" s="45" t="n"/>
     </row>
-    <row r="83" ht="33" customHeight="1">
+    <row r="83" ht="47.5" customHeight="1">
       <c r="A83" s="44" t="n">
         <v>46323</v>
       </c>
@@ -5101,7 +5130,7 @@
       </c>
       <c r="F83" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G83" s="45" t="inlineStr">
@@ -5377,7 +5406,7 @@
       </c>
       <c r="J89" s="39" t="n"/>
     </row>
-    <row r="90" ht="178" customHeight="1">
+    <row r="90" ht="163.5" customHeight="1">
       <c r="A90" s="38" t="n">
         <v>46323</v>
       </c>
@@ -5398,16 +5427,15 @@
       </c>
       <c r="E90" s="31" t="inlineStr">
         <is>
-          <t>Programar en Outlook los envíos del jueves 29/10</t>
+          <t>Preparar (y programar si puedes) los envíos del jueves 29/10</t>
         </is>
       </c>
       <c r="F90" s="39" t="inlineStr">
         <is>
-          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 29/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada.
+          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 29/10). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada si tu correo lo permite (ver LEEME). Si no puedes programar, no pasa nada: mañana a las 07:30 de Nueva York los envías a mano.
 • IA Akranes | Follow-up 2 | programar para las 05:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 29/10.
 • Maidstone United | Follow-up 2 | programar para las 05:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 29/10.
-• Whitehaven AFC | Follow-up 2 | programar para las 05:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 29/10.
-Importante: si usas Outlook de escritorio clásico, el ordenador debe estar encendido y con Outlook abierto a esa hora; con Outlook web o el Outlook nuevo, el envío sale solo desde el servidor.</t>
+• Whitehaven AFC | Follow-up 2 | programar para las 05:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 29/10.</t>
         </is>
       </c>
       <c r="G90" s="39" t="inlineStr">
@@ -5425,7 +5453,7 @@
       </c>
       <c r="J90" s="39" t="n"/>
     </row>
-    <row r="91" ht="33" customHeight="1">
+    <row r="91" ht="47.5" customHeight="1">
       <c r="A91" s="44" t="n">
         <v>46324</v>
       </c>
@@ -5451,7 +5479,7 @@
       </c>
       <c r="F91" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G91" s="45" t="inlineStr">
@@ -5467,7 +5495,7 @@
       </c>
       <c r="J91" s="45" t="n"/>
     </row>
-    <row r="92" ht="33" customHeight="1">
+    <row r="92" ht="47.5" customHeight="1">
       <c r="A92" s="44" t="n">
         <v>46324</v>
       </c>
@@ -5493,7 +5521,7 @@
       </c>
       <c r="F92" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G92" s="45" t="inlineStr">
@@ -5509,7 +5537,7 @@
       </c>
       <c r="J92" s="45" t="n"/>
     </row>
-    <row r="93" ht="33" customHeight="1">
+    <row r="93" ht="47.5" customHeight="1">
       <c r="A93" s="44" t="n">
         <v>46324</v>
       </c>
@@ -5535,7 +5563,7 @@
       </c>
       <c r="F93" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G93" s="45" t="inlineStr">
@@ -6166,7 +6194,7 @@
       </c>
       <c r="J108" s="39" t="n"/>
     </row>
-    <row r="109" ht="207" customHeight="1">
+    <row r="109" ht="192.5" customHeight="1">
       <c r="A109" s="38" t="n">
         <v>46328</v>
       </c>
@@ -6187,17 +6215,16 @@
       </c>
       <c r="E109" s="31" t="inlineStr">
         <is>
-          <t>Programar en Outlook los envíos del martes 03/11</t>
+          <t>Preparar (y programar si puedes) los envíos del martes 03/11</t>
         </is>
       </c>
       <c r="F109" s="39" t="inlineStr">
         <is>
-          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 03/11). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada.
+          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 03/11). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada si tu correo lo permite (ver LEEME). Si no puedes programar, no pasa nada: mañana a las 07:30 de Nueva York los envías a mano.
 • FC Porte d'Aquitaine | Follow-up 2 | programar para las 03:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 03/11.
 • Hastings United | Cierre | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 03/11.
 • Home Farm FC | Cierre | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 03/11.
-• Virtu Academy | Follow-up 2 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 03/11.
-Importante: si usas Outlook de escritorio clásico, el ordenador debe estar encendido y con Outlook abierto a esa hora; con Outlook web o el Outlook nuevo, el envío sale solo desde el servidor.</t>
+• Virtu Academy | Follow-up 2 | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 03/11.</t>
         </is>
       </c>
       <c r="G109" s="39" t="inlineStr">
@@ -6215,7 +6242,7 @@
       </c>
       <c r="J109" s="39" t="n"/>
     </row>
-    <row r="110" ht="33" customHeight="1">
+    <row r="110" ht="47.5" customHeight="1">
       <c r="A110" s="44" t="n">
         <v>46329</v>
       </c>
@@ -6241,7 +6268,7 @@
       </c>
       <c r="F110" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G110" s="45" t="inlineStr">
@@ -6257,7 +6284,7 @@
       </c>
       <c r="J110" s="45" t="n"/>
     </row>
-    <row r="111" ht="33" customHeight="1">
+    <row r="111" ht="47.5" customHeight="1">
       <c r="A111" s="44" t="n">
         <v>46329</v>
       </c>
@@ -6283,7 +6310,7 @@
       </c>
       <c r="F111" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G111" s="45" t="inlineStr">
@@ -6299,7 +6326,7 @@
       </c>
       <c r="J111" s="45" t="n"/>
     </row>
-    <row r="112" ht="33" customHeight="1">
+    <row r="112" ht="47.5" customHeight="1">
       <c r="A112" s="44" t="n">
         <v>46329</v>
       </c>
@@ -6325,7 +6352,7 @@
       </c>
       <c r="F112" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G112" s="45" t="inlineStr">
@@ -6341,7 +6368,7 @@
       </c>
       <c r="J112" s="45" t="n"/>
     </row>
-    <row r="113" ht="33" customHeight="1">
+    <row r="113" ht="47.5" customHeight="1">
       <c r="A113" s="44" t="n">
         <v>46329</v>
       </c>
@@ -6367,7 +6394,7 @@
       </c>
       <c r="F113" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G113" s="45" t="inlineStr">
@@ -6515,7 +6542,7 @@
       </c>
       <c r="J116" s="39" t="n"/>
     </row>
-    <row r="117" ht="149" customHeight="1">
+    <row r="117" ht="134.5" customHeight="1">
       <c r="A117" s="38" t="n">
         <v>46329</v>
       </c>
@@ -6536,15 +6563,14 @@
       </c>
       <c r="E117" s="31" t="inlineStr">
         <is>
-          <t>Programar en Outlook los envíos del miércoles 04/11</t>
+          <t>Preparar (y programar si puedes) los envíos del miércoles 04/11</t>
         </is>
       </c>
       <c r="F117" s="39" t="inlineStr">
         <is>
-          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 04/11). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada.
+          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 04/11). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada si tu correo lo permite (ver LEEME). Si no puedes programar, no pasa nada: mañana a las 07:30 de Nueva York los envías a mano.
 • Holbeach United | Cierre | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 04/11.
-• Søreide IL | Cierre | programar para las 03:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 04/11.
-Importante: si usas Outlook de escritorio clásico, el ordenador debe estar encendido y con Outlook abierto a esa hora; con Outlook web o el Outlook nuevo, el envío sale solo desde el servidor.</t>
+• Søreide IL | Cierre | programar para las 03:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 04/11.</t>
         </is>
       </c>
       <c r="G117" s="39" t="inlineStr">
@@ -6562,7 +6588,7 @@
       </c>
       <c r="J117" s="39" t="n"/>
     </row>
-    <row r="118" ht="33" customHeight="1">
+    <row r="118" ht="47.5" customHeight="1">
       <c r="A118" s="44" t="n">
         <v>46330</v>
       </c>
@@ -6588,7 +6614,7 @@
       </c>
       <c r="F118" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G118" s="45" t="inlineStr">
@@ -6604,7 +6630,7 @@
       </c>
       <c r="J118" s="45" t="n"/>
     </row>
-    <row r="119" ht="33" customHeight="1">
+    <row r="119" ht="47.5" customHeight="1">
       <c r="A119" s="44" t="n">
         <v>46330</v>
       </c>
@@ -6630,7 +6656,7 @@
       </c>
       <c r="F119" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G119" s="45" t="inlineStr">
@@ -6862,7 +6888,7 @@
       </c>
       <c r="J124" s="39" t="n"/>
     </row>
-    <row r="125" ht="178" customHeight="1">
+    <row r="125" ht="163.5" customHeight="1">
       <c r="A125" s="38" t="n">
         <v>46330</v>
       </c>
@@ -6883,16 +6909,15 @@
       </c>
       <c r="E125" s="31" t="inlineStr">
         <is>
-          <t>Programar en Outlook los envíos del jueves 05/11</t>
+          <t>Preparar (y programar si puedes) los envíos del jueves 05/11</t>
         </is>
       </c>
       <c r="F125" s="39" t="inlineStr">
         <is>
-          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 05/11). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada.
+          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 05/11). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada si tu correo lo permite (ver LEEME). Si no puedes programar, no pasa nada: mañana a las 07:30 de Nueva York los envías a mano.
 • IA Akranes | Cierre | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 05/11.
 • Maidstone United | Cierre | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 05/11.
-• Whitehaven AFC | Cierre | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 05/11.
-Importante: si usas Outlook de escritorio clásico, el ordenador debe estar encendido y con Outlook abierto a esa hora; con Outlook web o el Outlook nuevo, el envío sale solo desde el servidor.</t>
+• Whitehaven AFC | Cierre | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 05/11.</t>
         </is>
       </c>
       <c r="G125" s="39" t="inlineStr">
@@ -6910,7 +6935,7 @@
       </c>
       <c r="J125" s="39" t="n"/>
     </row>
-    <row r="126" ht="33" customHeight="1">
+    <row r="126" ht="47.5" customHeight="1">
       <c r="A126" s="44" t="n">
         <v>46331</v>
       </c>
@@ -6936,7 +6961,7 @@
       </c>
       <c r="F126" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G126" s="45" t="inlineStr">
@@ -6952,7 +6977,7 @@
       </c>
       <c r="J126" s="45" t="n"/>
     </row>
-    <row r="127" ht="33" customHeight="1">
+    <row r="127" ht="47.5" customHeight="1">
       <c r="A127" s="44" t="n">
         <v>46331</v>
       </c>
@@ -6978,7 +7003,7 @@
       </c>
       <c r="F127" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G127" s="45" t="inlineStr">
@@ -6994,7 +7019,7 @@
       </c>
       <c r="J127" s="45" t="n"/>
     </row>
-    <row r="128" ht="33" customHeight="1">
+    <row r="128" ht="47.5" customHeight="1">
       <c r="A128" s="44" t="n">
         <v>46331</v>
       </c>
@@ -7020,7 +7045,7 @@
       </c>
       <c r="F128" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G128" s="45" t="inlineStr">
@@ -7519,7 +7544,7 @@
       </c>
       <c r="J140" s="39" t="n"/>
     </row>
-    <row r="141" ht="149" customHeight="1">
+    <row r="141" ht="134.5" customHeight="1">
       <c r="A141" s="38" t="n">
         <v>46335</v>
       </c>
@@ -7540,15 +7565,14 @@
       </c>
       <c r="E141" s="31" t="inlineStr">
         <is>
-          <t>Programar en Outlook los envíos del martes 10/11</t>
+          <t>Preparar (y programar si puedes) los envíos del martes 10/11</t>
         </is>
       </c>
       <c r="F141" s="39" t="inlineStr">
         <is>
-          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 10/11). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada.
+          <t>Para cada correo: copia Para, Asunto y Texto de la hoja 'Textos para copiar' (filtra por la fecha 10/11). Revisa en 30 segundos: saludo, nombre del club, firma abajo, sin adjuntos. Programa el envío a la hora indicada si tu correo lo permite (ver LEEME). Si no puedes programar, no pasa nada: mañana a las 07:30 de Nueva York los envías a mano.
 • FC Porte d'Aquitaine | Cierre | programar para las 03:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 10/11.
-• Virtu Academy | Cierre | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 10/11.
-Importante: si usas Outlook de escritorio clásico, el ordenador debe estar encendido y con Outlook abierto a esa hora; con Outlook web o el Outlook nuevo, el envío sale solo desde el servidor.</t>
+• Virtu Academy | Cierre | programar para las 04:30 hora Nueva York (09:30 locales). Texto: fila de la hoja Textos para copiar del 10/11.</t>
         </is>
       </c>
       <c r="G141" s="39" t="inlineStr">
@@ -7566,7 +7590,7 @@
       </c>
       <c r="J141" s="39" t="n"/>
     </row>
-    <row r="142" ht="33" customHeight="1">
+    <row r="142" ht="47.5" customHeight="1">
       <c r="A142" s="44" t="n">
         <v>46336</v>
       </c>
@@ -7592,7 +7616,7 @@
       </c>
       <c r="F142" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G142" s="45" t="inlineStr">
@@ -7608,7 +7632,7 @@
       </c>
       <c r="J142" s="45" t="n"/>
     </row>
-    <row r="143" ht="33" customHeight="1">
+    <row r="143" ht="47.5" customHeight="1">
       <c r="A143" s="44" t="n">
         <v>46336</v>
       </c>
@@ -7634,7 +7658,7 @@
       </c>
       <c r="F143" s="45" t="inlineStr">
         <is>
-          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no lo programaste, envíalo cuando te despiertes. Texto en 'Textos para copiar'.</t>
+          <t>No tienes que hacer nada a esta hora si lo programaste la víspera. Si no pudiste programar, envíalo a mano a las 07:30 de Nueva York. Texto en 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="G143" s="45" t="inlineStr">
@@ -8550,7 +8574,7 @@
       </c>
       <c r="I5" s="51" t="inlineStr">
         <is>
-          <t>En Outlook: Nuevo correo. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Flecha junto a Enviar &gt; Programar envío &gt; elige fecha y la hora de Nueva York de la columna D.</t>
+          <t>Nuevo correo desde joel.martinez@alwaysup.es. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Si tu correo permite programar (webmail de Hostinger/Titan: flecha junto a Enviar &gt; Programar), hazlo para la hora de la columna D. Si no, plan B: envíalo a mano a las 07:30 de Nueva York (ver LEEME).</t>
         </is>
       </c>
       <c r="J5" s="51" t="n"/>
@@ -8609,7 +8633,7 @@
       </c>
       <c r="I6" s="51" t="inlineStr">
         <is>
-          <t>En Outlook: Nuevo correo. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Flecha junto a Enviar &gt; Programar envío &gt; elige fecha y la hora de Nueva York de la columna D.</t>
+          <t>Nuevo correo desde joel.martinez@alwaysup.es. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Si tu correo permite programar (webmail de Hostinger/Titan: flecha junto a Enviar &gt; Programar), hazlo para la hora de la columna D. Si no, plan B: envíalo a mano a las 07:30 de Nueva York (ver LEEME).</t>
         </is>
       </c>
       <c r="J6" s="51" t="n"/>
@@ -8718,7 +8742,7 @@
       </c>
       <c r="I8" s="51" t="inlineStr">
         <is>
-          <t>En Outlook: Nuevo correo. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Flecha junto a Enviar &gt; Programar envío &gt; elige fecha y la hora de Nueva York de la columna D.</t>
+          <t>Nuevo correo desde joel.martinez@alwaysup.es. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Si tu correo permite programar (webmail de Hostinger/Titan: flecha junto a Enviar &gt; Programar), hazlo para la hora de la columna D. Si no, plan B: envíalo a mano a las 07:30 de Nueva York (ver LEEME).</t>
         </is>
       </c>
       <c r="J8" s="51" t="n"/>
@@ -8776,7 +8800,7 @@
       </c>
       <c r="I9" s="51" t="inlineStr">
         <is>
-          <t>En Outlook: Nuevo correo. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Flecha junto a Enviar &gt; Programar envío &gt; elige fecha y la hora de Nueva York de la columna D.</t>
+          <t>Nuevo correo desde joel.martinez@alwaysup.es. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Si tu correo permite programar (webmail de Hostinger/Titan: flecha junto a Enviar &gt; Programar), hazlo para la hora de la columna D. Si no, plan B: envíalo a mano a las 07:30 de Nueva York (ver LEEME).</t>
         </is>
       </c>
       <c r="J9" s="51" t="n"/>
@@ -8834,7 +8858,7 @@
       </c>
       <c r="I10" s="51" t="inlineStr">
         <is>
-          <t>En Outlook: Nuevo correo. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Flecha junto a Enviar &gt; Programar envío &gt; elige fecha y la hora de Nueva York de la columna D.</t>
+          <t>Nuevo correo desde joel.martinez@alwaysup.es. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Si tu correo permite programar (webmail de Hostinger/Titan: flecha junto a Enviar &gt; Programar), hazlo para la hora de la columna D. Si no, plan B: envíalo a mano a las 07:30 de Nueva York (ver LEEME).</t>
         </is>
       </c>
       <c r="J10" s="51" t="n"/>
@@ -9045,7 +9069,7 @@
       </c>
       <c r="I14" s="51" t="inlineStr">
         <is>
-          <t>En Outlook: Nuevo correo. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Flecha junto a Enviar &gt; Programar envío &gt; elige fecha y la hora de Nueva York de la columna D.</t>
+          <t>Nuevo correo desde joel.martinez@alwaysup.es. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Si tu correo permite programar (webmail de Hostinger/Titan: flecha junto a Enviar &gt; Programar), hazlo para la hora de la columna D. Si no, plan B: envíalo a mano a las 07:30 de Nueva York (ver LEEME).</t>
         </is>
       </c>
       <c r="J14" s="51" t="n"/>
@@ -9104,7 +9128,7 @@
       </c>
       <c r="I15" s="57" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J15" s="57" t="n"/>
@@ -9163,7 +9187,7 @@
       </c>
       <c r="I16" s="57" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J16" s="57" t="n"/>
@@ -9221,7 +9245,7 @@
       </c>
       <c r="I17" s="51" t="inlineStr">
         <is>
-          <t>En Outlook: Nuevo correo. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Flecha junto a Enviar &gt; Programar envío &gt; elige fecha y la hora de Nueva York de la columna D.</t>
+          <t>Nuevo correo desde joel.martinez@alwaysup.es. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Si tu correo permite programar (webmail de Hostinger/Titan: flecha junto a Enviar &gt; Programar), hazlo para la hora de la columna D. Si no, plan B: envíalo a mano a las 07:30 de Nueva York (ver LEEME).</t>
         </is>
       </c>
       <c r="J17" s="51" t="n"/>
@@ -9280,7 +9304,7 @@
       </c>
       <c r="I18" s="57" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J18" s="57" t="n"/>
@@ -9339,7 +9363,7 @@
       </c>
       <c r="I19" s="57" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J19" s="57" t="n"/>
@@ -9397,7 +9421,7 @@
       </c>
       <c r="I20" s="57" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J20" s="57" t="n"/>
@@ -9455,7 +9479,7 @@
       </c>
       <c r="I21" s="57" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J21" s="57" t="n"/>
@@ -9514,7 +9538,7 @@
       </c>
       <c r="I22" s="57" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J22" s="57" t="n"/>
@@ -9573,7 +9597,7 @@
       </c>
       <c r="I23" s="57" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J23" s="57" t="n"/>
@@ -9630,7 +9654,7 @@
       </c>
       <c r="I24" s="60" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J24" s="60" t="n"/>
@@ -9687,7 +9711,7 @@
       </c>
       <c r="I25" s="60" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J25" s="60" t="n"/>
@@ -9745,7 +9769,7 @@
       </c>
       <c r="I26" s="57" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J26" s="57" t="n"/>
@@ -9853,7 +9877,7 @@
       </c>
       <c r="I28" s="60" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J28" s="60" t="n"/>
@@ -9961,7 +9985,7 @@
       </c>
       <c r="I30" s="60" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J30" s="60" t="n"/>
@@ -10069,7 +10093,7 @@
       </c>
       <c r="I32" s="60" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J32" s="60" t="n"/>
@@ -10126,7 +10150,7 @@
       </c>
       <c r="I33" s="60" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J33" s="60" t="n"/>
@@ -10234,7 +10258,7 @@
       </c>
       <c r="I35" s="60" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J35" s="60" t="n"/>
@@ -10444,7 +10468,7 @@
       </c>
       <c r="I39" s="60" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J39" s="60" t="n"/>
@@ -10502,7 +10526,7 @@
       </c>
       <c r="I40" s="63" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J40" s="63" t="n"/>
@@ -10560,7 +10584,7 @@
       </c>
       <c r="I41" s="63" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J41" s="63" t="n"/>
@@ -10617,7 +10641,7 @@
       </c>
       <c r="I42" s="60" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J42" s="60" t="n"/>
@@ -10726,7 +10750,7 @@
       </c>
       <c r="I44" s="63" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J44" s="63" t="n"/>
@@ -10784,7 +10808,7 @@
       </c>
       <c r="I45" s="63" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J45" s="63" t="n"/>
@@ -10893,7 +10917,7 @@
       </c>
       <c r="I47" s="63" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J47" s="63" t="n"/>
@@ -10951,7 +10975,7 @@
       </c>
       <c r="I48" s="63" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J48" s="63" t="n"/>
@@ -11009,7 +11033,7 @@
       </c>
       <c r="I49" s="63" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J49" s="63" t="n"/>
@@ -11067,7 +11091,7 @@
       </c>
       <c r="I50" s="63" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J50" s="63" t="n"/>
@@ -11125,7 +11149,7 @@
       </c>
       <c r="I51" s="63" t="inlineStr">
         <is>
-          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D. Antes de programar, mira en el CRM que no haya contestado por otro canal.</t>
+          <t>Abre el correo original en Enviados &gt; Responder (así queda en el mismo hilo). Pega el texto. Sin adjuntos. Programa el envío a la hora de la columna D o, si no puedes programar, envíalo a mano a las 07:30 de Nueva York. Antes, mira en el CRM que no haya contestado por otro canal.</t>
         </is>
       </c>
       <c r="J51" s="63" t="n"/>
@@ -12696,7 +12720,7 @@
       <c r="N10" s="13" t="inlineStr"/>
       <c r="O10" s="12" t="inlineStr">
         <is>
-          <t>Investigado 2026-08-29: posible error de nombre en el research original — no gastar más tiempo hasta verificar en la fuente original | 13/10/2026: costadauradacup.com lo lista como club de Inglaterra en la edición de Semana Santa 2026. Existe: falta encontrar su contacto. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable.</t>
+          <t>Investigado 2026-08-29: posible error de nombre en el research original — no gastar más tiempo hasta verificar en la fuente original | 13/10/2026: costadauradacup.com lo lista como club de Inglaterra en la edición de Semana Santa 2026. Existe: falta encontrar su contacto. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable.</t>
         </is>
       </c>
       <c r="P10" s="12" t="inlineStr">

</xml_diff>

<commit_message>
El generador conserva las marcas manuales de Joel (Hecho, notas, estados) al regenerar; prueba de entregabilidad superada
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -2061,10 +2061,14 @@
       </c>
       <c r="I9" s="39" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J9" s="39" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="J9" s="39" t="inlineStr">
+        <is>
+          <t>SPF/DKIM/DMARC PASS en Gmail</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="47.5" customHeight="1">
       <c r="A10" s="44" t="n">
@@ -12828,7 +12832,7 @@
       <c r="N10" s="13" t="inlineStr"/>
       <c r="O10" s="12" t="inlineStr">
         <is>
-          <t>Investigado 2026-08-29: posible error de nombre en el research original — no gastar más tiempo hasta verificar en la fuente original | 13/10/2026: costadauradacup.com lo lista como club de Inglaterra en la edición de Semana Santa 2026. Existe: falta encontrar su contacto. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable.</t>
+          <t>Investigado 2026-08-29: posible error de nombre en el research original — no gastar más tiempo hasta verificar en la fuente original | 13/10/2026: costadauradacup.com lo lista como club de Inglaterra en la edición de Semana Santa 2026. Existe: falta encontrar su contacto. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable.</t>
         </is>
       </c>
       <c r="P10" s="12" t="inlineStr">
@@ -13300,7 +13304,7 @@
       </c>
       <c r="O17" s="12" t="inlineStr">
         <is>
-          <t>Historial real: llamada en abril 2026, Leonardo mandó una presentación (enfocada en becas EEUU, poco encaje con lo que ya cubre el partner de becas), Joel propuso el ángulo real (intercambio Brasil-España de jugadores/equipos), propuso llamada con el padre para junio, luego siguió el 03/07 proponiendo martes — sin respuesta desde entonces (2+ meses). No confundir con un club prospecto normal de Segmento A — esto es más una posible relación de partner/distribución que una venta directa. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta.</t>
+          <t>Historial real: llamada en abril 2026, Leonardo mandó una presentación (enfocada en becas EEUU, poco encaje con lo que ya cubre el partner de becas), Joel propuso el ángulo real (intercambio Brasil-España de jugadores/equipos), propuso llamada con el padre para junio, luego siguió el 03/07 proponiendo martes — sin respuesta desde entonces (2+ meses). No confundir con un club prospecto normal de Segmento A — esto es más una posible relación de partner/distribución que una venta directa. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta.</t>
         </is>
       </c>
       <c r="P17" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Follow-up a Daniel, estado de Holbeach y Soreide, nota de escala y automatizacion futura
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -33,11 +33,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="34">
     <font>
@@ -128,61 +127,72 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FF0B1F3A"/>
       <sz val="15"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <color rgb="FF444444"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <i val="1"/>
       <color rgb="FF777777"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FF0B1F3A"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <i val="1"/>
       <color rgb="FF555555"/>
       <sz val="11"/>
@@ -395,7 +405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -523,6 +533,12 @@
     <xf numFmtId="0" fontId="21" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -535,12 +551,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -652,15 +662,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="31" fillId="21" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="166" fontId="31" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="31" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1074,8 +1075,8 @@
   <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="50" min="1" max="1"/>
-    <col width="110" customWidth="1" style="50" min="2" max="2"/>
+    <col width="24" customWidth="1" style="52" min="1" max="1"/>
+    <col width="110" customWidth="1" style="52" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1092,14 +1093,14 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1" s="50">
+    <row r="4" ht="22" customHeight="1" s="52">
       <c r="A4" s="61" t="inlineStr">
         <is>
           <t>TU RUTINA</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1" s="50">
+    <row r="5" ht="20" customHeight="1" s="52">
       <c r="A5" s="62" t="inlineStr">
         <is>
           <t>Cada mañana (15 min)</t>
@@ -1111,7 +1112,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="33" customHeight="1" s="50">
+    <row r="6" ht="33" customHeight="1" s="52">
       <c r="A6" s="62" t="inlineStr">
         <is>
           <t>La víspera (20 min)</t>
@@ -1123,7 +1124,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="20" customHeight="1" s="50">
+    <row r="7" ht="20" customHeight="1" s="52">
       <c r="A7" s="62" t="inlineStr">
         <is>
           <t>Cada viernes (20 min)</t>
@@ -1135,7 +1136,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="20" customHeight="1" s="50">
+    <row r="8" ht="20" customHeight="1" s="52">
       <c r="A8" s="62" t="inlineStr">
         <is>
           <t>Cada lunes (5 min)</t>
@@ -1147,14 +1148,14 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1" s="50">
+    <row r="9" ht="22" customHeight="1" s="52">
       <c r="A9" s="61" t="inlineStr">
         <is>
           <t>PESTAÑAS</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1" s="50">
+    <row r="10" ht="20" customHeight="1" s="52">
       <c r="A10" s="62" t="inlineStr">
         <is>
           <t>Calendario diario</t>
@@ -1166,7 +1167,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1" s="50">
+    <row r="11" ht="20" customHeight="1" s="52">
       <c r="A11" s="62" t="inlineStr">
         <is>
           <t>Textos para copiar</t>
@@ -1178,7 +1179,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1" s="50">
+    <row r="12" ht="20" customHeight="1" s="52">
       <c r="A12" s="62" t="inlineStr">
         <is>
           <t>Hoy</t>
@@ -1190,7 +1191,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1" s="50">
+    <row r="13" ht="20" customHeight="1" s="52">
       <c r="A13" s="62" t="inlineStr">
         <is>
           <t>Plan por servicio</t>
@@ -1202,7 +1203,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1" s="50">
+    <row r="14" ht="20" customHeight="1" s="52">
       <c r="A14" s="62" t="inlineStr">
         <is>
           <t>Verificación</t>
@@ -1214,7 +1215,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="33" customHeight="1" s="50">
+    <row r="15" ht="33" customHeight="1" s="52">
       <c r="A15" s="62" t="inlineStr">
         <is>
           <t>Segmento A / B / C</t>
@@ -1226,7 +1227,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1" s="50">
+    <row r="16" ht="20" customHeight="1" s="52">
       <c r="A16" s="62" t="inlineStr">
         <is>
           <t>Dashboard, LinkedIn, Oportunidades</t>
@@ -1238,14 +1239,14 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1" s="50">
+    <row r="17" ht="22" customHeight="1" s="52">
       <c r="A17" s="61" t="inlineStr">
         <is>
           <t>COMO Y CUANDO ENVIAR</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="33" customHeight="1" s="50">
+    <row r="18" ht="33" customHeight="1" s="52">
       <c r="A18" s="62" t="inlineStr">
         <is>
           <t>Qué se ha comprobado (14/10/2026)</t>
@@ -1257,7 +1258,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="47.5" customHeight="1" s="50">
+    <row r="19" ht="47.5" customHeight="1" s="52">
       <c r="A19" s="62" t="inlineStr">
         <is>
           <t>Por qué parecía que no salían</t>
@@ -1269,7 +1270,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="33" customHeight="1" s="50">
+    <row r="20" ht="33" customHeight="1" s="52">
       <c r="A20" s="62" t="inlineStr">
         <is>
           <t>Cómo se programa</t>
@@ -1281,7 +1282,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="33" customHeight="1" s="50">
+    <row r="21" ht="33" customHeight="1" s="52">
       <c r="A21" s="62" t="inlineStr">
         <is>
           <t>Regla para no duplicar</t>
@@ -1293,7 +1294,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="33" customHeight="1" s="50">
+    <row r="22" ht="33" customHeight="1" s="52">
       <c r="A22" s="62" t="inlineStr">
         <is>
           <t>Control</t>
@@ -1305,7 +1306,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="33" customHeight="1" s="50">
+    <row r="23" ht="33" customHeight="1" s="52">
       <c r="A23" s="62" t="inlineStr">
         <is>
           <t>Truco opcional</t>
@@ -1317,14 +1318,14 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1" s="50">
+    <row r="24" ht="22" customHeight="1" s="52">
       <c r="A24" s="61" t="inlineStr">
         <is>
           <t>TUS FRANJAS DE LLAMADA</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="33" customHeight="1" s="50">
+    <row r="25" ht="33" customHeight="1" s="52">
       <c r="A25" s="62" t="inlineStr">
         <is>
           <t>Lo que tienes en Calendly (hora Nueva York)</t>
@@ -1336,7 +1337,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="47.5" customHeight="1" s="50">
+    <row r="26" ht="47.5" customHeight="1" s="52">
       <c r="A26" s="62" t="inlineStr">
         <is>
           <t>Clubes de Europa (+5 h en UK e Irlanda, +6 h en Noruega, Francia y Países Bajos; +4 y +5 del 25 al 31/10)</t>
@@ -1348,7 +1349,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1" s="50">
+    <row r="27" ht="20" customHeight="1" s="52">
       <c r="A27" s="62" t="inlineStr">
         <is>
           <t>Familias de América (México, Latinoamérica, EEUU)</t>
@@ -1360,7 +1361,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="47.5" customHeight="1" s="50">
+    <row r="28" ht="47.5" customHeight="1" s="52">
       <c r="A28" s="62" t="inlineStr">
         <is>
           <t>Recomendación</t>
@@ -1372,14 +1373,14 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="22" customHeight="1" s="50">
+    <row r="29" ht="22" customHeight="1" s="52">
       <c r="A29" s="61" t="inlineStr">
         <is>
           <t>REGLAS QUE NO SE ROMPEN</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="33" customHeight="1" s="50">
+    <row r="30" ht="33" customHeight="1" s="52">
       <c r="A30" s="62" t="inlineStr">
         <is>
           <t>Nunca</t>
@@ -1391,7 +1392,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="33" customHeight="1" s="50">
+    <row r="31" ht="33" customHeight="1" s="52">
       <c r="A31" s="62" t="inlineStr">
         <is>
           <t>Si contestan</t>
@@ -1403,7 +1404,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="20" customHeight="1" s="50">
+    <row r="32" ht="20" customHeight="1" s="52">
       <c r="A32" s="62" t="inlineStr">
         <is>
           <t>Si un correo rebota</t>
@@ -1415,7 +1416,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="33" customHeight="1" s="50">
+    <row r="33" ht="33" customHeight="1" s="52">
       <c r="A33" s="62" t="inlineStr">
         <is>
           <t>Colores</t>
@@ -1448,31 +1449,31 @@
   <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" style="50" min="1" max="1"/>
-    <col width="20" customWidth="1" style="50" min="2" max="2"/>
-    <col width="16" customWidth="1" style="50" min="3" max="4"/>
-    <col width="18" customWidth="1" style="50" min="5" max="5"/>
-    <col width="20" customWidth="1" style="50" min="6" max="6"/>
-    <col width="14" customWidth="1" style="50" min="7" max="7"/>
-    <col width="12" customWidth="1" style="50" min="8" max="8"/>
+    <col width="22" customWidth="1" style="52" min="1" max="1"/>
+    <col width="20" customWidth="1" style="52" min="2" max="2"/>
+    <col width="16" customWidth="1" style="52" min="3" max="4"/>
+    <col width="18" customWidth="1" style="52" min="5" max="5"/>
+    <col width="20" customWidth="1" style="52" min="6" max="6"/>
+    <col width="14" customWidth="1" style="52" min="7" max="7"/>
+    <col width="12" customWidth="1" style="52" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="50">
-      <c r="A1" s="53" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="52">
+      <c r="A1" s="55" t="inlineStr">
         <is>
           <t>Dashboard — funnel por línea de negocio</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="54" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>Estado actual de cada línea. Actualizar Estado/Etapa en las pestañas de segmento — esto se recalcula solo.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" s="50">
-      <c r="A3" s="56" t="inlineStr">
+    <row r="3" ht="60" customHeight="1" s="52">
+      <c r="A3" s="58" t="inlineStr">
         <is>
           <t>Esto es una FOTO del estado ACTUAL de cada lead (cuántos están ahora mismo en cada estado), no un histórico acumulado de conversión — para eso haría falta guardar fecha de cada cambio de estado, cosa que no hacemos todavía. Sirve igual para ver dónde se acumulan los leads y detectar el cuello de botella real.</t>
         </is>
@@ -1569,7 +1570,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1" s="50">
+    <row r="11" ht="28" customHeight="1" s="52">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Nuevo</t>
@@ -1635,7 +1636,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="56" t="inlineStr">
+      <c r="A15" s="58" t="inlineStr">
         <is>
           <t>0 leads activos todavía — esta sección se activa con el primer lead real. Ver lineas-de-negocio.md línea 3. No crear pestaña de seguimiento hasta entonces.</t>
         </is>
@@ -1649,7 +1650,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="56" t="inlineStr">
+      <c r="A18" s="58" t="inlineStr">
         <is>
           <t>Sin funnel activo — decisión explícita de Joel de no priorizar hasta tener un cliente/jugador real interesado (lineas-de-negocio.md líneas 4 y 6). Si preguntan, ver manual-embudo-ventas.md para el guion de respuesta correcto (nunca prometer prueba/contrato garantizado).</t>
         </is>
@@ -1676,37 +1677,37 @@
   <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" style="50" min="1" max="1"/>
-    <col width="20" customWidth="1" style="50" min="2" max="2"/>
-    <col width="26" customWidth="1" style="50" min="3" max="3"/>
-    <col width="30" customWidth="1" style="50" min="4" max="4"/>
-    <col width="18" customWidth="1" style="50" min="5" max="5"/>
-    <col width="40" customWidth="1" style="50" min="6" max="6"/>
+    <col width="14" customWidth="1" style="52" min="1" max="1"/>
+    <col width="20" customWidth="1" style="52" min="2" max="2"/>
+    <col width="26" customWidth="1" style="52" min="3" max="3"/>
+    <col width="30" customWidth="1" style="52" min="4" max="4"/>
+    <col width="18" customWidth="1" style="52" min="5" max="5"/>
+    <col width="40" customWidth="1" style="52" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="50">
-      <c r="A1" s="53" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="52">
+      <c r="A1" s="55" t="inlineStr">
         <is>
           <t>LinkedIn — plan diario</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="54" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>Rellenar cada día que trabajes outreach.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" s="50">
-      <c r="A3" s="56" t="inlineStr">
+    <row r="3" ht="60" customHeight="1" s="52">
+      <c r="A3" s="58" t="inlineStr">
         <is>
           <t>ACTIVA desde el 28/09/2026 — perfil de LinkedIn terminado (titular, experiencia, foto). Semana 1 (28/09-04/10): 5-10 conexiones/día con gente conocida (Mercy, Mount Aloysius, fútbol en España), sin vender nada, para construir base real antes de contactar decisores. Semana 2 en adelante: 5 conexiones/día a decisores reales de Segmento A/B (crm-ventas.xlsx), nota corta con señal real, ver plan-ventas-maestro.md sección 4.</t>
         </is>
       </c>
     </row>
     <row r="4"/>
-    <row r="5" ht="28" customHeight="1" s="50">
+    <row r="5" ht="28" customHeight="1" s="52">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -1837,30 +1838,30 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" style="50" min="1" max="1"/>
-    <col width="26" customWidth="1" style="50" min="2" max="2"/>
-    <col width="40" customWidth="1" style="50" min="3" max="3"/>
-    <col width="22" customWidth="1" style="50" min="4" max="4"/>
-    <col width="40" customWidth="1" style="50" min="5" max="5"/>
-    <col width="20" customWidth="1" style="50" min="6" max="6"/>
+    <col width="14" customWidth="1" style="52" min="1" max="1"/>
+    <col width="26" customWidth="1" style="52" min="2" max="2"/>
+    <col width="40" customWidth="1" style="52" min="3" max="3"/>
+    <col width="22" customWidth="1" style="52" min="4" max="4"/>
+    <col width="40" customWidth="1" style="52" min="5" max="5"/>
+    <col width="20" customWidth="1" style="52" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="50">
-      <c r="A1" s="53" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="52">
+      <c r="A1" s="55" t="inlineStr">
         <is>
           <t>Oportunidades y notas sueltas</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="54" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>Ideas que surgen investigando, sin operativa de venta propia todavía.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1" s="50">
-      <c r="A3" s="56" t="inlineStr">
+    <row r="3" ht="30" customHeight="1" s="52">
+      <c r="A3" s="58" t="inlineStr">
         <is>
           <t>Backlog ligero para líneas que aún no tienen operativa propia de venta — no crear pestañas dedicadas hasta que Joel las eleve de prioridad (ver roadmap-maestro.md).</t>
         </is>
@@ -1898,7 +1899,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1" s="50">
+    <row r="5" ht="28" customHeight="1" s="52">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
@@ -1930,7 +1931,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1" s="50">
+    <row r="6" ht="28" customHeight="1" s="52">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>2026-08</t>
@@ -1994,7 +1995,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1" s="50">
+    <row r="8" ht="28" customHeight="1" s="52">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>2026-07</t>
@@ -2026,7 +2027,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1" s="50">
+    <row r="9" ht="42" customHeight="1" s="52">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>2026-08-29</t>
@@ -2079,33 +2080,33 @@
   <dimension ref="A1:J140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" style="50" min="1" max="1"/>
-    <col width="11" customWidth="1" style="50" min="2" max="2"/>
-    <col width="9" customWidth="1" style="50" min="3" max="3"/>
-    <col width="16" customWidth="1" style="50" min="4" max="4"/>
-    <col width="40" customWidth="1" style="50" min="5" max="5"/>
-    <col width="78" customWidth="1" style="50" min="6" max="6"/>
-    <col width="24" customWidth="1" style="50" min="7" max="7"/>
-    <col width="6" customWidth="1" style="50" min="8" max="8"/>
-    <col width="12" customWidth="1" style="50" min="9" max="9"/>
-    <col width="36" customWidth="1" style="50" min="10" max="10"/>
+    <col width="11" customWidth="1" style="52" min="1" max="1"/>
+    <col width="11" customWidth="1" style="52" min="2" max="2"/>
+    <col width="9" customWidth="1" style="52" min="3" max="3"/>
+    <col width="16" customWidth="1" style="52" min="4" max="4"/>
+    <col width="40" customWidth="1" style="52" min="5" max="5"/>
+    <col width="78" customWidth="1" style="52" min="6" max="6"/>
+    <col width="24" customWidth="1" style="52" min="7" max="7"/>
+    <col width="6" customWidth="1" style="52" min="8" max="8"/>
+    <col width="12" customWidth="1" style="52" min="9" max="9"/>
+    <col width="36" customWidth="1" style="52" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" s="50">
+    <row r="1" ht="26" customHeight="1" s="52">
       <c r="A1" s="64" t="inlineStr">
         <is>
           <t>Calendario diario: 13 de octubre a 13 de noviembre de 2026</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="46" customHeight="1" s="50">
+    <row r="2" ht="46" customHeight="1" s="52">
       <c r="A2" s="65" t="inlineStr">
         <is>
           <t>Qué haces tú cada día, a qué hora y cómo. Las horas son de Nueva York. Los correos se programan la víspera en Apple Mail (Enviar más tarde) para las 09:30 de cada club; a las 08:00 compruebas que salieron. Cambia la columna Estado a Hecho al terminar. Hoy se marca en amarillo. Si algo queda Pendiente de un día anterior, sale en rojo.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1" s="50">
+    <row r="4" ht="30" customHeight="1" s="52">
       <c r="A4" s="66" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -2157,14 +2158,14 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1" s="50">
+    <row r="5" ht="22" customHeight="1" s="52">
       <c r="A5" s="68" t="inlineStr">
         <is>
           <t>SEMANA  12/10 a 18/10</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="62" customHeight="1" s="50">
+    <row r="6" ht="62" customHeight="1" s="52">
       <c r="A6" s="94" t="n">
         <v>46308</v>
       </c>
@@ -2208,7 +2209,7 @@
       </c>
       <c r="J6" s="70" t="n"/>
     </row>
-    <row r="7" ht="33" customHeight="1" s="50">
+    <row r="7" ht="33" customHeight="1" s="52">
       <c r="A7" s="94" t="n">
         <v>46308</v>
       </c>
@@ -2250,7 +2251,7 @@
       </c>
       <c r="J7" s="70" t="n"/>
     </row>
-    <row r="8" ht="91" customHeight="1" s="50">
+    <row r="8" ht="91" customHeight="1" s="52">
       <c r="A8" s="94" t="n">
         <v>46308</v>
       </c>
@@ -2294,7 +2295,7 @@
       </c>
       <c r="J8" s="70" t="n"/>
     </row>
-    <row r="9" ht="47.5" customHeight="1" s="50">
+    <row r="9" ht="47.5" customHeight="1" s="52">
       <c r="A9" s="94" t="n">
         <v>46309</v>
       </c>
@@ -2331,16 +2332,12 @@
       <c r="H9" s="70" t="n"/>
       <c r="I9" s="70" t="inlineStr">
         <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="J9" s="70" t="inlineStr">
-        <is>
-          <t>Enviado a mano el 14/10</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="47.5" customHeight="1" s="50">
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J9" s="70" t="n"/>
+    </row>
+    <row r="10" ht="47.5" customHeight="1" s="52">
       <c r="A10" s="94" t="n">
         <v>46309</v>
       </c>
@@ -2377,16 +2374,12 @@
       <c r="H10" s="70" t="n"/>
       <c r="I10" s="70" t="inlineStr">
         <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="J10" s="70" t="inlineStr">
-        <is>
-          <t>Enviado a mano el 14/10</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="62" customHeight="1" s="50">
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J10" s="70" t="n"/>
+    </row>
+    <row r="11" ht="62" customHeight="1" s="52">
       <c r="A11" s="94" t="n">
         <v>46309</v>
       </c>
@@ -2425,12 +2418,12 @@
       </c>
       <c r="I11" s="70" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="J11" s="70" t="n"/>
     </row>
-    <row r="12" ht="76.5" customHeight="1" s="50">
+    <row r="12" ht="76.5" customHeight="1" s="52">
       <c r="A12" s="94" t="n">
         <v>46309</v>
       </c>
@@ -2474,7 +2467,7 @@
       </c>
       <c r="J12" s="70" t="n"/>
     </row>
-    <row r="13" ht="62" customHeight="1" s="50">
+    <row r="13" ht="62" customHeight="1" s="52">
       <c r="A13" s="94" t="n">
         <v>46309</v>
       </c>
@@ -2513,12 +2506,16 @@
       </c>
       <c r="I13" s="70" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J13" s="70" t="n"/>
-    </row>
-    <row r="14" ht="47.5" customHeight="1" s="50">
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="J13" s="70" t="inlineStr">
+        <is>
+          <t>Søreide: 1 envío (14/10 8:34). Holbeach: 2 confirmados (13/10 18:50 y 14/10 4:41) y el de ~8:30 no localizado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="47.5" customHeight="1" s="52">
       <c r="A14" s="94" t="n">
         <v>46309</v>
       </c>
@@ -2557,16 +2554,12 @@
       </c>
       <c r="I14" s="70" t="inlineStr">
         <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="J14" s="70" t="inlineStr">
-        <is>
-          <t>Sale con Mail cerrado y Mac en reposo; no aparece en 'Sent' de Outlook (otra carpeta)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="76.5" customHeight="1" s="50">
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J14" s="70" t="n"/>
+    </row>
+    <row r="15" ht="76.5" customHeight="1" s="52">
       <c r="A15" s="94" t="n">
         <v>46309</v>
       </c>
@@ -2605,16 +2598,12 @@
       </c>
       <c r="I15" s="70" t="inlineStr">
         <is>
-          <t>Hecho</t>
-        </is>
-      </c>
-      <c r="J15" s="70" t="inlineStr">
-        <is>
-          <t>3 cuentas Outlook: todas en bandeja principal</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="47.5" customHeight="1" s="50">
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J15" s="70" t="n"/>
+    </row>
+    <row r="16" ht="62" customHeight="1" s="52">
       <c r="A16" s="94" t="n">
         <v>46309</v>
       </c>
@@ -2625,7 +2614,7 @@
       </c>
       <c r="C16" s="71" t="inlineStr">
         <is>
-          <t>Libre</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D16" s="73" t="inlineStr">
@@ -2635,17 +2624,17 @@
       </c>
       <c r="E16" s="62" t="inlineStr">
         <is>
-          <t>Daniel (MLS NEXT): apuntar su @usuario en el CRM</t>
+          <t>Daniel (MLS NEXT): enviar el follow-up por Instagram</t>
         </is>
       </c>
       <c r="F16" s="70" t="inlineStr">
         <is>
-          <t>Abre la conversación de Instagram con Daniel, copia su @usuario y pégalo en la fila 20 de Segmento C (columna del contacto). Solo sirve para tenerlo localizado: no bloquea nada. Si no le has contestado todavía, dímelo y preparamos la respuesta.</t>
+          <t>No contestó a tu mensaje del 21/09. Mi consejo: un único follow-up corto con salida fácil, y si no responde en 7 días, pasarlo a 'Frío'. Texto en 'Respuestas tipo' (Daniel). Mejor entre las 12:00 y las 14:00 de Nueva York (18:00 a 20:00 en España, cuando está libre de clase). Después apunta en el CRM la fecha de envío.</t>
         </is>
       </c>
       <c r="G16" s="70" t="inlineStr">
         <is>
-          <t>Segmento C - Becas</t>
+          <t>Textos para copiar (Respuestas tipo)</t>
         </is>
       </c>
       <c r="H16" s="70" t="n">
@@ -2658,7 +2647,7 @@
       </c>
       <c r="J16" s="70" t="n"/>
     </row>
-    <row r="17" ht="163.5" customHeight="1" s="50">
+    <row r="17" ht="163.5" customHeight="1" s="52">
       <c r="A17" s="94" t="n">
         <v>46309</v>
       </c>
@@ -2706,7 +2695,7 @@
       </c>
       <c r="J17" s="70" t="n"/>
     </row>
-    <row r="18" ht="47.5" customHeight="1" s="50">
+    <row r="18" ht="47.5" customHeight="1" s="52">
       <c r="A18" s="94" t="n">
         <v>46310</v>
       </c>
@@ -2748,7 +2737,7 @@
       </c>
       <c r="J18" s="70" t="n"/>
     </row>
-    <row r="19" ht="47.5" customHeight="1" s="50">
+    <row r="19" ht="47.5" customHeight="1" s="52">
       <c r="A19" s="94" t="n">
         <v>46310</v>
       </c>
@@ -2790,7 +2779,7 @@
       </c>
       <c r="J19" s="70" t="n"/>
     </row>
-    <row r="20" ht="47.5" customHeight="1" s="50">
+    <row r="20" ht="47.5" customHeight="1" s="52">
       <c r="A20" s="94" t="n">
         <v>46310</v>
       </c>
@@ -2832,7 +2821,7 @@
       </c>
       <c r="J20" s="70" t="n"/>
     </row>
-    <row r="21" ht="62" customHeight="1" s="50">
+    <row r="21" ht="62" customHeight="1" s="52">
       <c r="A21" s="94" t="n">
         <v>46310</v>
       </c>
@@ -2876,7 +2865,7 @@
       </c>
       <c r="J21" s="70" t="n"/>
     </row>
-    <row r="22" ht="76.5" customHeight="1" s="50">
+    <row r="22" ht="76.5" customHeight="1" s="52">
       <c r="A22" s="94" t="n">
         <v>46310</v>
       </c>
@@ -2920,7 +2909,7 @@
       </c>
       <c r="J22" s="70" t="n"/>
     </row>
-    <row r="23" ht="33" customHeight="1" s="50">
+    <row r="23" ht="33" customHeight="1" s="52">
       <c r="A23" s="94" t="n">
         <v>46310</v>
       </c>
@@ -2964,7 +2953,7 @@
       </c>
       <c r="J23" s="70" t="n"/>
     </row>
-    <row r="24" ht="33" customHeight="1" s="50">
+    <row r="24" ht="33" customHeight="1" s="52">
       <c r="A24" s="94" t="n">
         <v>46310</v>
       </c>
@@ -3008,7 +2997,7 @@
       </c>
       <c r="J24" s="70" t="n"/>
     </row>
-    <row r="25" ht="76.5" customHeight="1" s="50">
+    <row r="25" ht="76.5" customHeight="1" s="52">
       <c r="A25" s="94" t="n">
         <v>46310</v>
       </c>
@@ -3052,7 +3041,7 @@
       </c>
       <c r="J25" s="70" t="n"/>
     </row>
-    <row r="26" ht="62" customHeight="1" s="50">
+    <row r="26" ht="62" customHeight="1" s="52">
       <c r="A26" s="94" t="n">
         <v>46310</v>
       </c>
@@ -3092,7 +3081,7 @@
       </c>
       <c r="J26" s="70" t="n"/>
     </row>
-    <row r="27" ht="76.5" customHeight="1" s="50">
+    <row r="27" ht="76.5" customHeight="1" s="52">
       <c r="A27" s="94" t="n">
         <v>46310</v>
       </c>
@@ -3136,7 +3125,7 @@
       </c>
       <c r="J27" s="70" t="n"/>
     </row>
-    <row r="28" ht="62" customHeight="1" s="50">
+    <row r="28" ht="62" customHeight="1" s="52">
       <c r="A28" s="94" t="n">
         <v>46311</v>
       </c>
@@ -3180,7 +3169,7 @@
       </c>
       <c r="J28" s="70" t="n"/>
     </row>
-    <row r="29" ht="33" customHeight="1" s="50">
+    <row r="29" ht="33" customHeight="1" s="52">
       <c r="A29" s="94" t="n">
         <v>46311</v>
       </c>
@@ -3224,7 +3213,7 @@
       </c>
       <c r="J29" s="70" t="n"/>
     </row>
-    <row r="30" ht="76.5" customHeight="1" s="50">
+    <row r="30" ht="76.5" customHeight="1" s="52">
       <c r="A30" s="94" t="n">
         <v>46311</v>
       </c>
@@ -3268,7 +3257,7 @@
       </c>
       <c r="J30" s="70" t="n"/>
     </row>
-    <row r="31" ht="76.5" customHeight="1" s="50">
+    <row r="31" ht="76.5" customHeight="1" s="52">
       <c r="A31" s="94" t="n">
         <v>46311</v>
       </c>
@@ -3312,7 +3301,7 @@
       </c>
       <c r="J31" s="70" t="n"/>
     </row>
-    <row r="32" ht="33" customHeight="1" s="50">
+    <row r="32" ht="33" customHeight="1" s="52">
       <c r="A32" s="94" t="n">
         <v>46311</v>
       </c>
@@ -3356,7 +3345,7 @@
       </c>
       <c r="J32" s="70" t="n"/>
     </row>
-    <row r="33" ht="47.5" customHeight="1" s="50">
+    <row r="33" ht="47.5" customHeight="1" s="52">
       <c r="A33" s="94" t="n">
         <v>46312</v>
       </c>
@@ -3400,14 +3389,14 @@
       </c>
       <c r="J33" s="70" t="n"/>
     </row>
-    <row r="34" ht="22" customHeight="1" s="50">
+    <row r="34" ht="22" customHeight="1" s="52">
       <c r="A34" s="68" t="inlineStr">
         <is>
           <t>SEMANA  19/10 a 25/10</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="62" customHeight="1" s="50">
+    <row r="35" ht="62" customHeight="1" s="52">
       <c r="A35" s="94" t="n">
         <v>46314</v>
       </c>
@@ -3451,7 +3440,7 @@
       </c>
       <c r="J35" s="70" t="n"/>
     </row>
-    <row r="36" ht="33" customHeight="1" s="50">
+    <row r="36" ht="33" customHeight="1" s="52">
       <c r="A36" s="94" t="n">
         <v>46314</v>
       </c>
@@ -3495,7 +3484,7 @@
       </c>
       <c r="J36" s="70" t="n"/>
     </row>
-    <row r="37" ht="33" customHeight="1" s="50">
+    <row r="37" ht="33" customHeight="1" s="52">
       <c r="A37" s="94" t="n">
         <v>46314</v>
       </c>
@@ -3539,7 +3528,7 @@
       </c>
       <c r="J37" s="70" t="n"/>
     </row>
-    <row r="38" ht="76.5" customHeight="1" s="50">
+    <row r="38" ht="76.5" customHeight="1" s="52">
       <c r="A38" s="94" t="n">
         <v>46314</v>
       </c>
@@ -3583,7 +3572,7 @@
       </c>
       <c r="J38" s="70" t="n"/>
     </row>
-    <row r="39" ht="33" customHeight="1" s="50">
+    <row r="39" ht="33" customHeight="1" s="52">
       <c r="A39" s="94" t="n">
         <v>46314</v>
       </c>
@@ -3623,7 +3612,7 @@
       </c>
       <c r="J39" s="70" t="n"/>
     </row>
-    <row r="40" ht="192.5" customHeight="1" s="50">
+    <row r="40" ht="192.5" customHeight="1" s="52">
       <c r="A40" s="94" t="n">
         <v>46314</v>
       </c>
@@ -3672,7 +3661,7 @@
       </c>
       <c r="J40" s="70" t="n"/>
     </row>
-    <row r="41" ht="47.5" customHeight="1" s="50">
+    <row r="41" ht="47.5" customHeight="1" s="52">
       <c r="A41" s="94" t="n">
         <v>46315</v>
       </c>
@@ -3714,7 +3703,7 @@
       </c>
       <c r="J41" s="70" t="n"/>
     </row>
-    <row r="42" ht="47.5" customHeight="1" s="50">
+    <row r="42" ht="47.5" customHeight="1" s="52">
       <c r="A42" s="94" t="n">
         <v>46315</v>
       </c>
@@ -3756,7 +3745,7 @@
       </c>
       <c r="J42" s="70" t="n"/>
     </row>
-    <row r="43" ht="47.5" customHeight="1" s="50">
+    <row r="43" ht="47.5" customHeight="1" s="52">
       <c r="A43" s="94" t="n">
         <v>46315</v>
       </c>
@@ -3798,7 +3787,7 @@
       </c>
       <c r="J43" s="70" t="n"/>
     </row>
-    <row r="44" ht="47.5" customHeight="1" s="50">
+    <row r="44" ht="47.5" customHeight="1" s="52">
       <c r="A44" s="94" t="n">
         <v>46315</v>
       </c>
@@ -3840,7 +3829,7 @@
       </c>
       <c r="J44" s="70" t="n"/>
     </row>
-    <row r="45" ht="62" customHeight="1" s="50">
+    <row r="45" ht="62" customHeight="1" s="52">
       <c r="A45" s="94" t="n">
         <v>46315</v>
       </c>
@@ -3884,7 +3873,7 @@
       </c>
       <c r="J45" s="70" t="n"/>
     </row>
-    <row r="46" ht="76.5" customHeight="1" s="50">
+    <row r="46" ht="76.5" customHeight="1" s="52">
       <c r="A46" s="94" t="n">
         <v>46315</v>
       </c>
@@ -3928,7 +3917,7 @@
       </c>
       <c r="J46" s="70" t="n"/>
     </row>
-    <row r="47" ht="47.5" customHeight="1" s="50">
+    <row r="47" ht="47.5" customHeight="1" s="52">
       <c r="A47" s="94" t="n">
         <v>46315</v>
       </c>
@@ -3972,7 +3961,7 @@
       </c>
       <c r="J47" s="70" t="n"/>
     </row>
-    <row r="48" ht="149" customHeight="1" s="50">
+    <row r="48" ht="149" customHeight="1" s="52">
       <c r="A48" s="94" t="n">
         <v>46315</v>
       </c>
@@ -4019,7 +4008,7 @@
       </c>
       <c r="J48" s="70" t="n"/>
     </row>
-    <row r="49" ht="47.5" customHeight="1" s="50">
+    <row r="49" ht="47.5" customHeight="1" s="52">
       <c r="A49" s="94" t="n">
         <v>46316</v>
       </c>
@@ -4061,7 +4050,7 @@
       </c>
       <c r="J49" s="70" t="n"/>
     </row>
-    <row r="50" ht="47.5" customHeight="1" s="50">
+    <row r="50" ht="47.5" customHeight="1" s="52">
       <c r="A50" s="94" t="n">
         <v>46316</v>
       </c>
@@ -4103,7 +4092,7 @@
       </c>
       <c r="J50" s="70" t="n"/>
     </row>
-    <row r="51" ht="62" customHeight="1" s="50">
+    <row r="51" ht="62" customHeight="1" s="52">
       <c r="A51" s="94" t="n">
         <v>46316</v>
       </c>
@@ -4147,7 +4136,7 @@
       </c>
       <c r="J51" s="70" t="n"/>
     </row>
-    <row r="52" ht="76.5" customHeight="1" s="50">
+    <row r="52" ht="76.5" customHeight="1" s="52">
       <c r="A52" s="94" t="n">
         <v>46316</v>
       </c>
@@ -4191,7 +4180,7 @@
       </c>
       <c r="J52" s="70" t="n"/>
     </row>
-    <row r="53" ht="178" customHeight="1" s="50">
+    <row r="53" ht="178" customHeight="1" s="52">
       <c r="A53" s="94" t="n">
         <v>46316</v>
       </c>
@@ -4239,7 +4228,7 @@
       </c>
       <c r="J53" s="70" t="n"/>
     </row>
-    <row r="54" ht="47.5" customHeight="1" s="50">
+    <row r="54" ht="47.5" customHeight="1" s="52">
       <c r="A54" s="94" t="n">
         <v>46317</v>
       </c>
@@ -4281,7 +4270,7 @@
       </c>
       <c r="J54" s="70" t="n"/>
     </row>
-    <row r="55" ht="47.5" customHeight="1" s="50">
+    <row r="55" ht="47.5" customHeight="1" s="52">
       <c r="A55" s="94" t="n">
         <v>46317</v>
       </c>
@@ -4323,7 +4312,7 @@
       </c>
       <c r="J55" s="70" t="n"/>
     </row>
-    <row r="56" ht="47.5" customHeight="1" s="50">
+    <row r="56" ht="47.5" customHeight="1" s="52">
       <c r="A56" s="94" t="n">
         <v>46317</v>
       </c>
@@ -4365,7 +4354,7 @@
       </c>
       <c r="J56" s="70" t="n"/>
     </row>
-    <row r="57" ht="62" customHeight="1" s="50">
+    <row r="57" ht="62" customHeight="1" s="52">
       <c r="A57" s="94" t="n">
         <v>46317</v>
       </c>
@@ -4409,7 +4398,7 @@
       </c>
       <c r="J57" s="70" t="n"/>
     </row>
-    <row r="58" ht="76.5" customHeight="1" s="50">
+    <row r="58" ht="76.5" customHeight="1" s="52">
       <c r="A58" s="94" t="n">
         <v>46317</v>
       </c>
@@ -4453,7 +4442,7 @@
       </c>
       <c r="J58" s="70" t="n"/>
     </row>
-    <row r="59" ht="47.5" customHeight="1" s="50">
+    <row r="59" ht="47.5" customHeight="1" s="52">
       <c r="A59" s="94" t="n">
         <v>46317</v>
       </c>
@@ -4493,7 +4482,7 @@
       </c>
       <c r="J59" s="70" t="n"/>
     </row>
-    <row r="60" ht="62" customHeight="1" s="50">
+    <row r="60" ht="62" customHeight="1" s="52">
       <c r="A60" s="94" t="n">
         <v>46318</v>
       </c>
@@ -4537,7 +4526,7 @@
       </c>
       <c r="J60" s="70" t="n"/>
     </row>
-    <row r="61" ht="62" customHeight="1" s="50">
+    <row r="61" ht="62" customHeight="1" s="52">
       <c r="A61" s="94" t="n">
         <v>46318</v>
       </c>
@@ -4581,7 +4570,7 @@
       </c>
       <c r="J61" s="70" t="n"/>
     </row>
-    <row r="62" ht="33" customHeight="1" s="50">
+    <row r="62" ht="33" customHeight="1" s="52">
       <c r="A62" s="94" t="n">
         <v>46318</v>
       </c>
@@ -4621,7 +4610,7 @@
       </c>
       <c r="J62" s="70" t="n"/>
     </row>
-    <row r="63" ht="33" customHeight="1" s="50">
+    <row r="63" ht="33" customHeight="1" s="52">
       <c r="A63" s="94" t="n">
         <v>46318</v>
       </c>
@@ -4665,7 +4654,7 @@
       </c>
       <c r="J63" s="70" t="n"/>
     </row>
-    <row r="64" ht="33" customHeight="1" s="50">
+    <row r="64" ht="33" customHeight="1" s="52">
       <c r="A64" s="94" t="n">
         <v>46319</v>
       </c>
@@ -4709,14 +4698,14 @@
       </c>
       <c r="J64" s="70" t="n"/>
     </row>
-    <row r="65" ht="22" customHeight="1" s="50">
+    <row r="65" ht="22" customHeight="1" s="52">
       <c r="A65" s="68" t="inlineStr">
         <is>
           <t>SEMANA  26/10 a 01/11</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="62" customHeight="1" s="50">
+    <row r="66" ht="62" customHeight="1" s="52">
       <c r="A66" s="94" t="n">
         <v>46321</v>
       </c>
@@ -4760,7 +4749,7 @@
       </c>
       <c r="J66" s="70" t="n"/>
     </row>
-    <row r="67" ht="33" customHeight="1" s="50">
+    <row r="67" ht="33" customHeight="1" s="52">
       <c r="A67" s="94" t="n">
         <v>46321</v>
       </c>
@@ -4804,7 +4793,7 @@
       </c>
       <c r="J67" s="70" t="n"/>
     </row>
-    <row r="68" ht="33" customHeight="1" s="50">
+    <row r="68" ht="33" customHeight="1" s="52">
       <c r="A68" s="94" t="n">
         <v>46321</v>
       </c>
@@ -4848,7 +4837,7 @@
       </c>
       <c r="J68" s="70" t="n"/>
     </row>
-    <row r="69" ht="33" customHeight="1" s="50">
+    <row r="69" ht="33" customHeight="1" s="52">
       <c r="A69" s="94" t="n">
         <v>46321</v>
       </c>
@@ -4892,7 +4881,7 @@
       </c>
       <c r="J69" s="70" t="n"/>
     </row>
-    <row r="70" ht="207" customHeight="1" s="50">
+    <row r="70" ht="207" customHeight="1" s="52">
       <c r="A70" s="94" t="n">
         <v>46321</v>
       </c>
@@ -4941,7 +4930,7 @@
       </c>
       <c r="J70" s="70" t="n"/>
     </row>
-    <row r="71" ht="47.5" customHeight="1" s="50">
+    <row r="71" ht="47.5" customHeight="1" s="52">
       <c r="A71" s="94" t="n">
         <v>46322</v>
       </c>
@@ -4983,7 +4972,7 @@
       </c>
       <c r="J71" s="70" t="n"/>
     </row>
-    <row r="72" ht="47.5" customHeight="1" s="50">
+    <row r="72" ht="47.5" customHeight="1" s="52">
       <c r="A72" s="94" t="n">
         <v>46322</v>
       </c>
@@ -5025,7 +5014,7 @@
       </c>
       <c r="J72" s="70" t="n"/>
     </row>
-    <row r="73" ht="47.5" customHeight="1" s="50">
+    <row r="73" ht="47.5" customHeight="1" s="52">
       <c r="A73" s="94" t="n">
         <v>46322</v>
       </c>
@@ -5067,7 +5056,7 @@
       </c>
       <c r="J73" s="70" t="n"/>
     </row>
-    <row r="74" ht="47.5" customHeight="1" s="50">
+    <row r="74" ht="47.5" customHeight="1" s="52">
       <c r="A74" s="94" t="n">
         <v>46322</v>
       </c>
@@ -5109,7 +5098,7 @@
       </c>
       <c r="J74" s="70" t="n"/>
     </row>
-    <row r="75" ht="62" customHeight="1" s="50">
+    <row r="75" ht="62" customHeight="1" s="52">
       <c r="A75" s="94" t="n">
         <v>46322</v>
       </c>
@@ -5153,7 +5142,7 @@
       </c>
       <c r="J75" s="70" t="n"/>
     </row>
-    <row r="76" ht="76.5" customHeight="1" s="50">
+    <row r="76" ht="76.5" customHeight="1" s="52">
       <c r="A76" s="94" t="n">
         <v>46322</v>
       </c>
@@ -5197,7 +5186,7 @@
       </c>
       <c r="J76" s="70" t="n"/>
     </row>
-    <row r="77" ht="33" customHeight="1" s="50">
+    <row r="77" ht="33" customHeight="1" s="52">
       <c r="A77" s="94" t="n">
         <v>46322</v>
       </c>
@@ -5241,7 +5230,7 @@
       </c>
       <c r="J77" s="70" t="n"/>
     </row>
-    <row r="78" ht="149" customHeight="1" s="50">
+    <row r="78" ht="149" customHeight="1" s="52">
       <c r="A78" s="94" t="n">
         <v>46322</v>
       </c>
@@ -5288,7 +5277,7 @@
       </c>
       <c r="J78" s="70" t="n"/>
     </row>
-    <row r="79" ht="47.5" customHeight="1" s="50">
+    <row r="79" ht="47.5" customHeight="1" s="52">
       <c r="A79" s="94" t="n">
         <v>46323</v>
       </c>
@@ -5330,7 +5319,7 @@
       </c>
       <c r="J79" s="70" t="n"/>
     </row>
-    <row r="80" ht="47.5" customHeight="1" s="50">
+    <row r="80" ht="47.5" customHeight="1" s="52">
       <c r="A80" s="94" t="n">
         <v>46323</v>
       </c>
@@ -5372,7 +5361,7 @@
       </c>
       <c r="J80" s="70" t="n"/>
     </row>
-    <row r="81" ht="62" customHeight="1" s="50">
+    <row r="81" ht="62" customHeight="1" s="52">
       <c r="A81" s="94" t="n">
         <v>46323</v>
       </c>
@@ -5416,7 +5405,7 @@
       </c>
       <c r="J81" s="70" t="n"/>
     </row>
-    <row r="82" ht="76.5" customHeight="1" s="50">
+    <row r="82" ht="76.5" customHeight="1" s="52">
       <c r="A82" s="94" t="n">
         <v>46323</v>
       </c>
@@ -5460,7 +5449,7 @@
       </c>
       <c r="J82" s="70" t="n"/>
     </row>
-    <row r="83" ht="47.5" customHeight="1" s="50">
+    <row r="83" ht="47.5" customHeight="1" s="52">
       <c r="A83" s="94" t="n">
         <v>46323</v>
       </c>
@@ -5504,7 +5493,7 @@
       </c>
       <c r="J83" s="70" t="n"/>
     </row>
-    <row r="84" ht="76.5" customHeight="1" s="50">
+    <row r="84" ht="76.5" customHeight="1" s="52">
       <c r="A84" s="94" t="n">
         <v>46323</v>
       </c>
@@ -5548,7 +5537,7 @@
       </c>
       <c r="J84" s="70" t="n"/>
     </row>
-    <row r="85" ht="76.5" customHeight="1" s="50">
+    <row r="85" ht="76.5" customHeight="1" s="52">
       <c r="A85" s="94" t="n">
         <v>46323</v>
       </c>
@@ -5592,7 +5581,7 @@
       </c>
       <c r="J85" s="70" t="n"/>
     </row>
-    <row r="86" ht="178" customHeight="1" s="50">
+    <row r="86" ht="178" customHeight="1" s="52">
       <c r="A86" s="94" t="n">
         <v>46323</v>
       </c>
@@ -5640,7 +5629,7 @@
       </c>
       <c r="J86" s="70" t="n"/>
     </row>
-    <row r="87" ht="47.5" customHeight="1" s="50">
+    <row r="87" ht="47.5" customHeight="1" s="52">
       <c r="A87" s="94" t="n">
         <v>46324</v>
       </c>
@@ -5682,7 +5671,7 @@
       </c>
       <c r="J87" s="70" t="n"/>
     </row>
-    <row r="88" ht="47.5" customHeight="1" s="50">
+    <row r="88" ht="47.5" customHeight="1" s="52">
       <c r="A88" s="94" t="n">
         <v>46324</v>
       </c>
@@ -5724,7 +5713,7 @@
       </c>
       <c r="J88" s="70" t="n"/>
     </row>
-    <row r="89" ht="47.5" customHeight="1" s="50">
+    <row r="89" ht="47.5" customHeight="1" s="52">
       <c r="A89" s="94" t="n">
         <v>46324</v>
       </c>
@@ -5766,7 +5755,7 @@
       </c>
       <c r="J89" s="70" t="n"/>
     </row>
-    <row r="90" ht="62" customHeight="1" s="50">
+    <row r="90" ht="62" customHeight="1" s="52">
       <c r="A90" s="94" t="n">
         <v>46324</v>
       </c>
@@ -5810,7 +5799,7 @@
       </c>
       <c r="J90" s="70" t="n"/>
     </row>
-    <row r="91" ht="76.5" customHeight="1" s="50">
+    <row r="91" ht="76.5" customHeight="1" s="52">
       <c r="A91" s="94" t="n">
         <v>46324</v>
       </c>
@@ -5854,7 +5843,7 @@
       </c>
       <c r="J91" s="70" t="n"/>
     </row>
-    <row r="92" ht="76.5" customHeight="1" s="50">
+    <row r="92" ht="76.5" customHeight="1" s="52">
       <c r="A92" s="94" t="n">
         <v>46324</v>
       </c>
@@ -5898,7 +5887,7 @@
       </c>
       <c r="J92" s="70" t="n"/>
     </row>
-    <row r="93" ht="76.5" customHeight="1" s="50">
+    <row r="93" ht="76.5" customHeight="1" s="52">
       <c r="A93" s="94" t="n">
         <v>46324</v>
       </c>
@@ -5942,7 +5931,7 @@
       </c>
       <c r="J93" s="70" t="n"/>
     </row>
-    <row r="94" ht="62" customHeight="1" s="50">
+    <row r="94" ht="62" customHeight="1" s="52">
       <c r="A94" s="94" t="n">
         <v>46325</v>
       </c>
@@ -5986,7 +5975,7 @@
       </c>
       <c r="J94" s="70" t="n"/>
     </row>
-    <row r="95" ht="76.5" customHeight="1" s="50">
+    <row r="95" ht="76.5" customHeight="1" s="52">
       <c r="A95" s="94" t="n">
         <v>46325</v>
       </c>
@@ -6030,7 +6019,7 @@
       </c>
       <c r="J95" s="70" t="n"/>
     </row>
-    <row r="96" ht="76.5" customHeight="1" s="50">
+    <row r="96" ht="76.5" customHeight="1" s="52">
       <c r="A96" s="94" t="n">
         <v>46325</v>
       </c>
@@ -6074,7 +6063,7 @@
       </c>
       <c r="J96" s="70" t="n"/>
     </row>
-    <row r="97" ht="76.5" customHeight="1" s="50">
+    <row r="97" ht="76.5" customHeight="1" s="52">
       <c r="A97" s="94" t="n">
         <v>46325</v>
       </c>
@@ -6118,7 +6107,7 @@
       </c>
       <c r="J97" s="70" t="n"/>
     </row>
-    <row r="98" ht="33" customHeight="1" s="50">
+    <row r="98" ht="33" customHeight="1" s="52">
       <c r="A98" s="94" t="n">
         <v>46325</v>
       </c>
@@ -6162,14 +6151,14 @@
       </c>
       <c r="J98" s="70" t="n"/>
     </row>
-    <row r="99" ht="22" customHeight="1" s="50">
+    <row r="99" ht="22" customHeight="1" s="52">
       <c r="A99" s="68" t="inlineStr">
         <is>
           <t>SEMANA  02/11 a 08/11</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="62" customHeight="1" s="50">
+    <row r="100" ht="62" customHeight="1" s="52">
       <c r="A100" s="94" t="n">
         <v>46328</v>
       </c>
@@ -6213,7 +6202,7 @@
       </c>
       <c r="J100" s="70" t="n"/>
     </row>
-    <row r="101" ht="33" customHeight="1" s="50">
+    <row r="101" ht="33" customHeight="1" s="52">
       <c r="A101" s="94" t="n">
         <v>46328</v>
       </c>
@@ -6257,7 +6246,7 @@
       </c>
       <c r="J101" s="70" t="n"/>
     </row>
-    <row r="102" ht="33" customHeight="1" s="50">
+    <row r="102" ht="33" customHeight="1" s="52">
       <c r="A102" s="94" t="n">
         <v>46328</v>
       </c>
@@ -6301,7 +6290,7 @@
       </c>
       <c r="J102" s="70" t="n"/>
     </row>
-    <row r="103" ht="192.5" customHeight="1" s="50">
+    <row r="103" ht="192.5" customHeight="1" s="52">
       <c r="A103" s="94" t="n">
         <v>46328</v>
       </c>
@@ -6350,7 +6339,7 @@
       </c>
       <c r="J103" s="70" t="n"/>
     </row>
-    <row r="104" ht="47.5" customHeight="1" s="50">
+    <row r="104" ht="47.5" customHeight="1" s="52">
       <c r="A104" s="94" t="n">
         <v>46329</v>
       </c>
@@ -6392,7 +6381,7 @@
       </c>
       <c r="J104" s="70" t="n"/>
     </row>
-    <row r="105" ht="47.5" customHeight="1" s="50">
+    <row r="105" ht="47.5" customHeight="1" s="52">
       <c r="A105" s="94" t="n">
         <v>46329</v>
       </c>
@@ -6434,7 +6423,7 @@
       </c>
       <c r="J105" s="70" t="n"/>
     </row>
-    <row r="106" ht="47.5" customHeight="1" s="50">
+    <row r="106" ht="47.5" customHeight="1" s="52">
       <c r="A106" s="94" t="n">
         <v>46329</v>
       </c>
@@ -6476,7 +6465,7 @@
       </c>
       <c r="J106" s="70" t="n"/>
     </row>
-    <row r="107" ht="47.5" customHeight="1" s="50">
+    <row r="107" ht="47.5" customHeight="1" s="52">
       <c r="A107" s="94" t="n">
         <v>46329</v>
       </c>
@@ -6518,7 +6507,7 @@
       </c>
       <c r="J107" s="70" t="n"/>
     </row>
-    <row r="108" ht="62" customHeight="1" s="50">
+    <row r="108" ht="62" customHeight="1" s="52">
       <c r="A108" s="94" t="n">
         <v>46329</v>
       </c>
@@ -6562,7 +6551,7 @@
       </c>
       <c r="J108" s="70" t="n"/>
     </row>
-    <row r="109" ht="76.5" customHeight="1" s="50">
+    <row r="109" ht="76.5" customHeight="1" s="52">
       <c r="A109" s="94" t="n">
         <v>46329</v>
       </c>
@@ -6606,7 +6595,7 @@
       </c>
       <c r="J109" s="70" t="n"/>
     </row>
-    <row r="110" ht="30" customHeight="1" s="50">
+    <row r="110" ht="30" customHeight="1" s="52">
       <c r="A110" s="94" t="n">
         <v>46329</v>
       </c>
@@ -6650,7 +6639,7 @@
       </c>
       <c r="J110" s="70" t="n"/>
     </row>
-    <row r="111" ht="134.5" customHeight="1" s="50">
+    <row r="111" ht="134.5" customHeight="1" s="52">
       <c r="A111" s="94" t="n">
         <v>46329</v>
       </c>
@@ -6697,7 +6686,7 @@
       </c>
       <c r="J111" s="70" t="n"/>
     </row>
-    <row r="112" ht="47.5" customHeight="1" s="50">
+    <row r="112" ht="47.5" customHeight="1" s="52">
       <c r="A112" s="94" t="n">
         <v>46330</v>
       </c>
@@ -6739,7 +6728,7 @@
       </c>
       <c r="J112" s="70" t="n"/>
     </row>
-    <row r="113" ht="47.5" customHeight="1" s="50">
+    <row r="113" ht="47.5" customHeight="1" s="52">
       <c r="A113" s="94" t="n">
         <v>46330</v>
       </c>
@@ -6781,7 +6770,7 @@
       </c>
       <c r="J113" s="70" t="n"/>
     </row>
-    <row r="114" ht="62" customHeight="1" s="50">
+    <row r="114" ht="62" customHeight="1" s="52">
       <c r="A114" s="94" t="n">
         <v>46330</v>
       </c>
@@ -6825,7 +6814,7 @@
       </c>
       <c r="J114" s="70" t="n"/>
     </row>
-    <row r="115" ht="76.5" customHeight="1" s="50">
+    <row r="115" ht="76.5" customHeight="1" s="52">
       <c r="A115" s="94" t="n">
         <v>46330</v>
       </c>
@@ -6869,7 +6858,7 @@
       </c>
       <c r="J115" s="70" t="n"/>
     </row>
-    <row r="116" ht="91" customHeight="1" s="50">
+    <row r="116" ht="91" customHeight="1" s="52">
       <c r="A116" s="94" t="n">
         <v>46330</v>
       </c>
@@ -6913,7 +6902,7 @@
       </c>
       <c r="J116" s="70" t="n"/>
     </row>
-    <row r="117" ht="76.5" customHeight="1" s="50">
+    <row r="117" ht="76.5" customHeight="1" s="52">
       <c r="A117" s="94" t="n">
         <v>46330</v>
       </c>
@@ -6957,7 +6946,7 @@
       </c>
       <c r="J117" s="70" t="n"/>
     </row>
-    <row r="118" ht="149" customHeight="1" s="50">
+    <row r="118" ht="149" customHeight="1" s="52">
       <c r="A118" s="94" t="n">
         <v>46330</v>
       </c>
@@ -7005,7 +6994,7 @@
       </c>
       <c r="J118" s="70" t="n"/>
     </row>
-    <row r="119" ht="47.5" customHeight="1" s="50">
+    <row r="119" ht="47.5" customHeight="1" s="52">
       <c r="A119" s="94" t="n">
         <v>46331</v>
       </c>
@@ -7047,7 +7036,7 @@
       </c>
       <c r="J119" s="70" t="n"/>
     </row>
-    <row r="120" ht="47.5" customHeight="1" s="50">
+    <row r="120" ht="47.5" customHeight="1" s="52">
       <c r="A120" s="94" t="n">
         <v>46331</v>
       </c>
@@ -7089,7 +7078,7 @@
       </c>
       <c r="J120" s="70" t="n"/>
     </row>
-    <row r="121" ht="47.5" customHeight="1" s="50">
+    <row r="121" ht="47.5" customHeight="1" s="52">
       <c r="A121" s="94" t="n">
         <v>46331</v>
       </c>
@@ -7131,7 +7120,7 @@
       </c>
       <c r="J121" s="70" t="n"/>
     </row>
-    <row r="122" ht="62" customHeight="1" s="50">
+    <row r="122" ht="62" customHeight="1" s="52">
       <c r="A122" s="94" t="n">
         <v>46331</v>
       </c>
@@ -7175,7 +7164,7 @@
       </c>
       <c r="J122" s="70" t="n"/>
     </row>
-    <row r="123" ht="76.5" customHeight="1" s="50">
+    <row r="123" ht="76.5" customHeight="1" s="52">
       <c r="A123" s="94" t="n">
         <v>46331</v>
       </c>
@@ -7219,7 +7208,7 @@
       </c>
       <c r="J123" s="70" t="n"/>
     </row>
-    <row r="124" ht="62" customHeight="1" s="50">
+    <row r="124" ht="62" customHeight="1" s="52">
       <c r="A124" s="94" t="n">
         <v>46332</v>
       </c>
@@ -7263,7 +7252,7 @@
       </c>
       <c r="J124" s="70" t="n"/>
     </row>
-    <row r="125" ht="33" customHeight="1" s="50">
+    <row r="125" ht="33" customHeight="1" s="52">
       <c r="A125" s="94" t="n">
         <v>46332</v>
       </c>
@@ -7307,7 +7296,7 @@
       </c>
       <c r="J125" s="70" t="n"/>
     </row>
-    <row r="126" ht="33" customHeight="1" s="50">
+    <row r="126" ht="33" customHeight="1" s="52">
       <c r="A126" s="94" t="n">
         <v>46332</v>
       </c>
@@ -7351,14 +7340,14 @@
       </c>
       <c r="J126" s="70" t="n"/>
     </row>
-    <row r="127" ht="22" customHeight="1" s="50">
+    <row r="127" ht="22" customHeight="1" s="52">
       <c r="A127" s="68" t="inlineStr">
         <is>
           <t>SEMANA  09/11 a 15/11</t>
         </is>
       </c>
     </row>
-    <row r="128" ht="62" customHeight="1" s="50">
+    <row r="128" ht="62" customHeight="1" s="52">
       <c r="A128" s="94" t="n">
         <v>46335</v>
       </c>
@@ -7402,7 +7391,7 @@
       </c>
       <c r="J128" s="70" t="n"/>
     </row>
-    <row r="129" ht="33" customHeight="1" s="50">
+    <row r="129" ht="33" customHeight="1" s="52">
       <c r="A129" s="94" t="n">
         <v>46335</v>
       </c>
@@ -7446,7 +7435,7 @@
       </c>
       <c r="J129" s="70" t="n"/>
     </row>
-    <row r="130" ht="33" customHeight="1" s="50">
+    <row r="130" ht="33" customHeight="1" s="52">
       <c r="A130" s="94" t="n">
         <v>46335</v>
       </c>
@@ -7490,7 +7479,7 @@
       </c>
       <c r="J130" s="70" t="n"/>
     </row>
-    <row r="131" ht="33" customHeight="1" s="50">
+    <row r="131" ht="62" customHeight="1" s="52">
       <c r="A131" s="94" t="n">
         <v>46335</v>
       </c>
@@ -7516,7 +7505,7 @@
       </c>
       <c r="F131" s="70" t="inlineStr">
         <is>
-          <t>Resultados, qué cambiamos, qué dejamos y plan del segundo mes. Comprobamos si llegamos a la primera venta real.</t>
+          <t>Resultados, qué cambiamos, qué dejamos y plan del segundo mes. Comprobamos si llegamos a la primera venta real. Valoramos también la automatización del envío (objetivo de Joel: cientos de correos a la semana): Google Workspace, herramienta de envíos con calentamiento y qué se puede delegar.</t>
         </is>
       </c>
       <c r="G131" s="70" t="inlineStr">
@@ -7534,7 +7523,7 @@
       </c>
       <c r="J131" s="70" t="n"/>
     </row>
-    <row r="132" ht="134.5" customHeight="1" s="50">
+    <row r="132" ht="134.5" customHeight="1" s="52">
       <c r="A132" s="94" t="n">
         <v>46335</v>
       </c>
@@ -7581,7 +7570,7 @@
       </c>
       <c r="J132" s="70" t="n"/>
     </row>
-    <row r="133" ht="47.5" customHeight="1" s="50">
+    <row r="133" ht="47.5" customHeight="1" s="52">
       <c r="A133" s="94" t="n">
         <v>46336</v>
       </c>
@@ -7623,7 +7612,7 @@
       </c>
       <c r="J133" s="70" t="n"/>
     </row>
-    <row r="134" ht="47.5" customHeight="1" s="50">
+    <row r="134" ht="47.5" customHeight="1" s="52">
       <c r="A134" s="94" t="n">
         <v>46336</v>
       </c>
@@ -7665,7 +7654,7 @@
       </c>
       <c r="J134" s="70" t="n"/>
     </row>
-    <row r="135" ht="62" customHeight="1" s="50">
+    <row r="135" ht="62" customHeight="1" s="52">
       <c r="A135" s="94" t="n">
         <v>46336</v>
       </c>
@@ -7709,7 +7698,7 @@
       </c>
       <c r="J135" s="70" t="n"/>
     </row>
-    <row r="136" ht="76.5" customHeight="1" s="50">
+    <row r="136" ht="76.5" customHeight="1" s="52">
       <c r="A136" s="94" t="n">
         <v>46336</v>
       </c>
@@ -7753,7 +7742,7 @@
       </c>
       <c r="J136" s="70" t="n"/>
     </row>
-    <row r="137" ht="62" customHeight="1" s="50">
+    <row r="137" ht="62" customHeight="1" s="52">
       <c r="A137" s="94" t="n">
         <v>46337</v>
       </c>
@@ -7797,7 +7786,7 @@
       </c>
       <c r="J137" s="70" t="n"/>
     </row>
-    <row r="138" ht="62" customHeight="1" s="50">
+    <row r="138" ht="62" customHeight="1" s="52">
       <c r="A138" s="94" t="n">
         <v>46338</v>
       </c>
@@ -7841,7 +7830,7 @@
       </c>
       <c r="J138" s="70" t="n"/>
     </row>
-    <row r="139" ht="62" customHeight="1" s="50">
+    <row r="139" ht="62" customHeight="1" s="52">
       <c r="A139" s="94" t="n">
         <v>46339</v>
       </c>
@@ -7885,7 +7874,7 @@
       </c>
       <c r="J139" s="70" t="n"/>
     </row>
-    <row r="140" ht="33" customHeight="1" s="50">
+    <row r="140" ht="33" customHeight="1" s="52">
       <c r="A140" s="94" t="n">
         <v>46339</v>
       </c>
@@ -7970,22 +7959,22 @@
   <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" style="50" min="1" max="1"/>
-    <col width="18" customWidth="1" style="50" min="2" max="2"/>
-    <col width="16" customWidth="1" style="50" min="3" max="5"/>
-    <col width="18" customWidth="1" style="50" min="6" max="6"/>
-    <col width="12" customWidth="1" style="50" min="7" max="7"/>
+    <col width="50" customWidth="1" style="52" min="1" max="1"/>
+    <col width="18" customWidth="1" style="52" min="2" max="2"/>
+    <col width="16" customWidth="1" style="52" min="3" max="5"/>
+    <col width="18" customWidth="1" style="52" min="6" max="6"/>
+    <col width="12" customWidth="1" style="52" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="50">
-      <c r="A1" s="53" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="52">
+      <c r="A1" s="55" t="inlineStr">
         <is>
           <t>Plan de ventas — panel diario Always Up</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="54" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>Actualizar cada día de trabajo. Fecha de última actualización:</t>
         </is>
@@ -7995,14 +7984,14 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16" customHeight="1" s="50">
+    <row r="4" ht="16" customHeight="1" s="52">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>🔴 URGENTE — mirar esto primero</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1" s="50">
+    <row r="5" ht="28" customHeight="1" s="52">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Qué</t>
@@ -8047,14 +8036,14 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1" s="50">
+    <row r="10" ht="16" customHeight="1" s="52">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>🟠 OUTBOUND — lo que generas tú hoy</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1" s="50">
+    <row r="11" ht="28" customHeight="1" s="52">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Métrica</t>
@@ -8110,14 +8099,14 @@
       </c>
       <c r="C14" s="6" t="n"/>
     </row>
-    <row r="17" ht="16" customHeight="1" s="50">
+    <row r="17" ht="16" customHeight="1" s="52">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>🟢 INBOUND — lo que te llega a ti</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1" s="50">
+    <row r="18" ht="28" customHeight="1" s="52">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Qué</t>
@@ -8140,7 +8129,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1" s="50">
+    <row r="21" ht="16" customHeight="1" s="52">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>📊 PIPELINE — resumen por segmento (detalle completo en pestaña Dashboard)</t>
@@ -8347,37 +8336,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" style="50" min="1" max="1"/>
-    <col width="9" customWidth="1" style="50" min="2" max="2"/>
-    <col width="14" customWidth="1" style="50" min="3" max="3"/>
-    <col width="26" customWidth="1" style="50" min="4" max="4"/>
-    <col width="15" customWidth="1" style="50" min="5" max="5"/>
-    <col width="30" customWidth="1" style="50" min="6" max="6"/>
-    <col width="34" customWidth="1" style="50" min="7" max="7"/>
-    <col width="78" customWidth="1" style="50" min="8" max="8"/>
-    <col width="44" customWidth="1" style="50" min="9" max="9"/>
-    <col width="14" customWidth="1" style="50" min="10" max="10"/>
-    <col width="36" customWidth="1" style="50" min="11" max="11"/>
+    <col width="11" customWidth="1" style="52" min="1" max="1"/>
+    <col width="9" customWidth="1" style="52" min="2" max="2"/>
+    <col width="14" customWidth="1" style="52" min="3" max="3"/>
+    <col width="26" customWidth="1" style="52" min="4" max="4"/>
+    <col width="15" customWidth="1" style="52" min="5" max="5"/>
+    <col width="30" customWidth="1" style="52" min="6" max="6"/>
+    <col width="34" customWidth="1" style="52" min="7" max="7"/>
+    <col width="78" customWidth="1" style="52" min="8" max="8"/>
+    <col width="44" customWidth="1" style="52" min="9" max="9"/>
+    <col width="14" customWidth="1" style="52" min="10" max="10"/>
+    <col width="36" customWidth="1" style="52" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" s="50">
+    <row r="1" ht="26" customHeight="1" s="52">
       <c r="A1" s="64" t="inlineStr">
         <is>
           <t>Textos para copiar y pegar</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="46" customHeight="1" s="50">
+    <row r="2" ht="46" customHeight="1" s="52">
       <c r="A2" s="65" t="inlineStr">
         <is>
           <t>Una fila por envío, ordenada por fecha. Filtra la columna Fecha para ver solo el día que toca. Copia Para, Asunto y Texto sin cambiar nada: la firma ya va incluida. Hora = a qué hora de Nueva York programar el envío (son las 09:30 en el país del club). Los textos están revisados por Claude: sin guiones largos, sin placeholders, saludo a una sola persona.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1" s="50">
+    <row r="4" ht="30" customHeight="1" s="52">
       <c r="A4" s="66" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -8434,7 +8423,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="279.5" customHeight="1" s="50">
+    <row r="5" ht="279.5" customHeight="1" s="52">
       <c r="A5" s="95" t="n">
         <v>46309</v>
       </c>
@@ -8486,16 +8475,14 @@
           <t>En Mail: correo nuevo desde joel.martinez@alwaysup.es. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Flecha junto a Enviar &gt; Enviar más tarde &gt; fecha y la hora de la columna C. Una vez programado, no lo envíes a mano.</t>
         </is>
       </c>
-      <c r="J5" s="102" t="n">
-        <v>46309</v>
-      </c>
+      <c r="J5" s="78" t="n"/>
       <c r="K5" s="78" t="inlineStr">
         <is>
           <t>Rebota: avísame y busco otra dirección. Contesta: para la cadencia y mira 'Respuestas tipo' abajo.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="294" customHeight="1" s="50">
+    <row r="6" ht="294" customHeight="1" s="52">
       <c r="A6" s="95" t="n">
         <v>46309</v>
       </c>
@@ -8547,16 +8534,14 @@
           <t>En Mail: correo nuevo desde joel.martinez@alwaysup.es. Pega Para, Asunto y Texto tal cual (la firma ya va dentro). Sin adjuntos. Flecha junto a Enviar &gt; Enviar más tarde &gt; fecha y la hora de la columna C. Una vez programado, no lo envíes a mano.</t>
         </is>
       </c>
-      <c r="J6" s="102" t="n">
-        <v>46309</v>
-      </c>
+      <c r="J6" s="78" t="n"/>
       <c r="K6" s="78" t="inlineStr">
         <is>
           <t>Rebota: avísame y busco otra dirección. Contesta: para la cadencia y mira 'Respuestas tipo' abajo.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="62" customHeight="1" s="50">
+    <row r="7" ht="62" customHeight="1" s="52">
       <c r="A7" s="96" t="n">
         <v>46310</v>
       </c>
@@ -8607,7 +8592,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="236" customHeight="1" s="50">
+    <row r="8" ht="236" customHeight="1" s="52">
       <c r="A8" s="95" t="n">
         <v>46310</v>
       </c>
@@ -8665,7 +8650,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="250.5" customHeight="1" s="50">
+    <row r="9" ht="250.5" customHeight="1" s="52">
       <c r="A9" s="95" t="n">
         <v>46310</v>
       </c>
@@ -8723,7 +8708,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="265" customHeight="1" s="50">
+    <row r="10" ht="265" customHeight="1" s="52">
       <c r="A10" s="95" t="n">
         <v>46310</v>
       </c>
@@ -8781,7 +8766,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="62" customHeight="1" s="50">
+    <row r="11" ht="62" customHeight="1" s="52">
       <c r="A11" s="96" t="n">
         <v>46311</v>
       </c>
@@ -8832,7 +8817,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="62" customHeight="1" s="50">
+    <row r="12" ht="62" customHeight="1" s="52">
       <c r="A12" s="96" t="n">
         <v>46311</v>
       </c>
@@ -8883,7 +8868,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="62" customHeight="1" s="50">
+    <row r="13" ht="62" customHeight="1" s="52">
       <c r="A13" s="96" t="n">
         <v>46314</v>
       </c>
@@ -8934,7 +8919,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="279.5" customHeight="1" s="50">
+    <row r="14" ht="279.5" customHeight="1" s="52">
       <c r="A14" s="95" t="n">
         <v>46315</v>
       </c>
@@ -8992,7 +8977,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="250.5" customHeight="1" s="50">
+    <row r="15" ht="250.5" customHeight="1" s="52">
       <c r="A15" s="97" t="n">
         <v>46315</v>
       </c>
@@ -9051,7 +9036,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="250.5" customHeight="1" s="50">
+    <row r="16" ht="250.5" customHeight="1" s="52">
       <c r="A16" s="97" t="n">
         <v>46315</v>
       </c>
@@ -9110,7 +9095,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="236" customHeight="1" s="50">
+    <row r="17" ht="236" customHeight="1" s="52">
       <c r="A17" s="95" t="n">
         <v>46315</v>
       </c>
@@ -9168,7 +9153,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="250.5" customHeight="1" s="50">
+    <row r="18" ht="250.5" customHeight="1" s="52">
       <c r="A18" s="97" t="n">
         <v>46316</v>
       </c>
@@ -9227,7 +9212,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="250.5" customHeight="1" s="50">
+    <row r="19" ht="250.5" customHeight="1" s="52">
       <c r="A19" s="97" t="n">
         <v>46316</v>
       </c>
@@ -9286,7 +9271,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="221.5" customHeight="1" s="50">
+    <row r="20" ht="221.5" customHeight="1" s="52">
       <c r="A20" s="97" t="n">
         <v>46317</v>
       </c>
@@ -9344,7 +9329,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="221.5" customHeight="1" s="50">
+    <row r="21" ht="221.5" customHeight="1" s="52">
       <c r="A21" s="97" t="n">
         <v>46317</v>
       </c>
@@ -9402,7 +9387,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="250.5" customHeight="1" s="50">
+    <row r="22" ht="250.5" customHeight="1" s="52">
       <c r="A22" s="97" t="n">
         <v>46317</v>
       </c>
@@ -9461,7 +9446,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="279.5" customHeight="1" s="50">
+    <row r="23" ht="279.5" customHeight="1" s="52">
       <c r="A23" s="97" t="n">
         <v>46322</v>
       </c>
@@ -9520,7 +9505,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="178" customHeight="1" s="50">
+    <row r="24" ht="178" customHeight="1" s="52">
       <c r="A24" s="98" t="n">
         <v>46322</v>
       </c>
@@ -9577,7 +9562,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="178" customHeight="1" s="50">
+    <row r="25" ht="178" customHeight="1" s="52">
       <c r="A25" s="98" t="n">
         <v>46322</v>
       </c>
@@ -9634,7 +9619,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="221.5" customHeight="1" s="50">
+    <row r="26" ht="221.5" customHeight="1" s="52">
       <c r="A26" s="97" t="n">
         <v>46322</v>
       </c>
@@ -9692,7 +9677,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1" s="50">
+    <row r="27" ht="60" customHeight="1" s="52">
       <c r="A27" s="96" t="n">
         <v>46323</v>
       </c>
@@ -9743,7 +9728,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="178" customHeight="1" s="50">
+    <row r="28" ht="178" customHeight="1" s="52">
       <c r="A28" s="98" t="n">
         <v>46323</v>
       </c>
@@ -9800,7 +9785,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="60" customHeight="1" s="50">
+    <row r="29" ht="60" customHeight="1" s="52">
       <c r="A29" s="96" t="n">
         <v>46323</v>
       </c>
@@ -9851,7 +9836,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="178" customHeight="1" s="50">
+    <row r="30" ht="178" customHeight="1" s="52">
       <c r="A30" s="98" t="n">
         <v>46323</v>
       </c>
@@ -9908,7 +9893,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="60" customHeight="1" s="50">
+    <row r="31" ht="60" customHeight="1" s="52">
       <c r="A31" s="96" t="n">
         <v>46324</v>
       </c>
@@ -9959,7 +9944,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="178" customHeight="1" s="50">
+    <row r="32" ht="178" customHeight="1" s="52">
       <c r="A32" s="98" t="n">
         <v>46324</v>
       </c>
@@ -10016,7 +10001,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="178" customHeight="1" s="50">
+    <row r="33" ht="178" customHeight="1" s="52">
       <c r="A33" s="98" t="n">
         <v>46324</v>
       </c>
@@ -10073,7 +10058,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="60" customHeight="1" s="50">
+    <row r="34" ht="60" customHeight="1" s="52">
       <c r="A34" s="96" t="n">
         <v>46324</v>
       </c>
@@ -10124,7 +10109,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="178" customHeight="1" s="50">
+    <row r="35" ht="178" customHeight="1" s="52">
       <c r="A35" s="98" t="n">
         <v>46324</v>
       </c>
@@ -10181,7 +10166,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="60" customHeight="1" s="50">
+    <row r="36" ht="60" customHeight="1" s="52">
       <c r="A36" s="96" t="n">
         <v>46325</v>
       </c>
@@ -10232,7 +10217,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="60" customHeight="1" s="50">
+    <row r="37" ht="60" customHeight="1" s="52">
       <c r="A37" s="96" t="n">
         <v>46325</v>
       </c>
@@ -10283,7 +10268,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="60" customHeight="1" s="50">
+    <row r="38" ht="60" customHeight="1" s="52">
       <c r="A38" s="96" t="n">
         <v>46325</v>
       </c>
@@ -10334,7 +10319,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="207" customHeight="1" s="50">
+    <row r="39" ht="207" customHeight="1" s="52">
       <c r="A39" s="98" t="n">
         <v>46329</v>
       </c>
@@ -10391,7 +10376,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="192.5" customHeight="1" s="50">
+    <row r="40" ht="192.5" customHeight="1" s="52">
       <c r="A40" s="99" t="n">
         <v>46329</v>
       </c>
@@ -10449,7 +10434,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="192.5" customHeight="1" s="50">
+    <row r="41" ht="192.5" customHeight="1" s="52">
       <c r="A41" s="99" t="n">
         <v>46329</v>
       </c>
@@ -10507,7 +10492,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="178" customHeight="1" s="50">
+    <row r="42" ht="178" customHeight="1" s="52">
       <c r="A42" s="98" t="n">
         <v>46329</v>
       </c>
@@ -10564,7 +10549,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="62" customHeight="1" s="50">
+    <row r="43" ht="62" customHeight="1" s="52">
       <c r="A43" s="96" t="n">
         <v>46330</v>
       </c>
@@ -10615,7 +10600,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="192.5" customHeight="1" s="50">
+    <row r="44" ht="192.5" customHeight="1" s="52">
       <c r="A44" s="99" t="n">
         <v>46330</v>
       </c>
@@ -10673,7 +10658,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="192.5" customHeight="1" s="50">
+    <row r="45" ht="192.5" customHeight="1" s="52">
       <c r="A45" s="99" t="n">
         <v>46330</v>
       </c>
@@ -10731,7 +10716,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="60" customHeight="1" s="50">
+    <row r="46" ht="60" customHeight="1" s="52">
       <c r="A46" s="96" t="n">
         <v>46330</v>
       </c>
@@ -10782,7 +10767,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="192.5" customHeight="1" s="50">
+    <row r="47" ht="192.5" customHeight="1" s="52">
       <c r="A47" s="99" t="n">
         <v>46331</v>
       </c>
@@ -10840,7 +10825,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="192.5" customHeight="1" s="50">
+    <row r="48" ht="192.5" customHeight="1" s="52">
       <c r="A48" s="99" t="n">
         <v>46331</v>
       </c>
@@ -10898,7 +10883,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="192.5" customHeight="1" s="50">
+    <row r="49" ht="192.5" customHeight="1" s="52">
       <c r="A49" s="99" t="n">
         <v>46331</v>
       </c>
@@ -10956,7 +10941,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="207" customHeight="1" s="50">
+    <row r="50" ht="207" customHeight="1" s="52">
       <c r="A50" s="99" t="n">
         <v>46336</v>
       </c>
@@ -11014,7 +10999,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="192.5" customHeight="1" s="50">
+    <row r="51" ht="192.5" customHeight="1" s="52">
       <c r="A51" s="99" t="n">
         <v>46336</v>
       </c>
@@ -11079,7 +11064,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="120" customHeight="1" s="50">
+    <row r="55" ht="120" customHeight="1" s="52">
       <c r="D55" s="62" t="inlineStr">
         <is>
           <t>Responde: quiere hablar</t>
@@ -11100,7 +11085,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="120" customHeight="1" s="50">
+    <row r="56" ht="120" customHeight="1" s="52">
       <c r="D56" s="62" t="inlineStr">
         <is>
           <t>Responde: pide información</t>
@@ -11121,7 +11106,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="120" customHeight="1" s="50">
+    <row r="57" ht="120" customHeight="1" s="52">
       <c r="D57" s="62" t="inlineStr">
         <is>
           <t>Responde: pregunta el precio</t>
@@ -11142,7 +11127,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="105.5" customHeight="1" s="50">
+    <row r="58" ht="105.5" customHeight="1" s="52">
       <c r="D58" s="62" t="inlineStr">
         <is>
           <t>Responde: ahora no</t>
@@ -11163,7 +11148,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="105.5" customHeight="1" s="50">
+    <row r="59" ht="105.5" customHeight="1" s="52">
       <c r="D59" s="62" t="inlineStr">
         <is>
           <t>Responde: no soy la persona</t>
@@ -11184,19 +11169,38 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="120" customHeight="1" s="50">
+    <row r="60" ht="134.5" customHeight="1" s="52">
       <c r="D60" s="62" t="inlineStr">
         <is>
+          <t>Daniel (MLS NEXT): follow-up por Instagram</t>
+        </is>
+      </c>
+      <c r="H60" s="63" t="inlineStr">
+        <is>
+          <t>Hola Daniel, ¿qué tal? Hace unas semanas hablamos de tu duda entre 1º y 2º de Bachillerato y de cómo encajaría con el proceso universitario en EEUU. Te escribo solo para saber si sigues con ganas de explorarlo.
+Si es así, mándame tu posición y, si tienes, un vídeo o enlace de algún partido de la MLS NEXT, y te cuento con calma qué opciones reales habría en tu caso. Cuanto antes lo veamos, más margen hay para decidir bien lo del curso.
+Y si ahora no es el momento, no pasa nada, dímelo y lo dejamos aquí.</t>
+        </is>
+      </c>
+      <c r="I60" s="63" t="inlineStr">
+        <is>
+          <t>Instagram. Un solo follow-up. Si no contesta en 7 días, pasa a Frío en el CRM. No pidas más datos en este mensaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="120" customHeight="1" s="52">
+      <c r="D61" s="62" t="inlineStr">
+        <is>
           <t>Pedir testimonio y presentaciones al club irlandés</t>
         </is>
       </c>
-      <c r="H60" s="63" t="inlineStr">
+      <c r="H61" s="63" t="inlineStr">
         <is>
           <t>Hi [nombre], hope you and the squad are doing well. I have a small favour to ask. We're building up Always Up and your league title story means a lot to us. Would you be happy to share two or three lines about what the experience did for the players, or even a short video message? And if you know any other clubs who would enjoy a trip like yours, an introduction from you would help us enormously. Thank you so much.
 Joel</t>
         </is>
       </c>
-      <c r="I60" s="63" t="inlineStr">
+      <c r="I61" s="63" t="inlineStr">
         <is>
           <t>Mándalo tú o Enrique, por WhatsApp. El nombre del contacto lo pones tú. Si dice que sí, pídele una foto del trofeo con los jugadores (con permiso del club).</t>
         </is>
@@ -11222,32 +11226,32 @@
   <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="50" min="1" max="1"/>
-    <col width="11" customWidth="1" style="50" min="2" max="2"/>
-    <col width="28" customWidth="1" style="50" min="3" max="3"/>
-    <col width="46" customWidth="1" style="50" min="4" max="4"/>
-    <col width="40" customWidth="1" style="50" min="5" max="5"/>
-    <col width="44" customWidth="1" style="50" min="6" max="6"/>
-    <col width="30" customWidth="1" style="50" min="7" max="7"/>
-    <col width="26" customWidth="1" style="50" min="8" max="8"/>
-    <col width="40" customWidth="1" style="50" min="9" max="9"/>
+    <col width="24" customWidth="1" style="52" min="1" max="1"/>
+    <col width="11" customWidth="1" style="52" min="2" max="2"/>
+    <col width="28" customWidth="1" style="52" min="3" max="3"/>
+    <col width="46" customWidth="1" style="52" min="4" max="4"/>
+    <col width="40" customWidth="1" style="52" min="5" max="5"/>
+    <col width="44" customWidth="1" style="52" min="6" max="6"/>
+    <col width="30" customWidth="1" style="52" min="7" max="7"/>
+    <col width="26" customWidth="1" style="52" min="8" max="8"/>
+    <col width="40" customWidth="1" style="52" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" s="50">
+    <row r="1" ht="26" customHeight="1" s="52">
       <c r="A1" s="64" t="inlineStr">
         <is>
           <t>Plan de captación por servicio</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="46" customHeight="1" s="50">
+    <row r="2" ht="46" customHeight="1" s="52">
       <c r="A2" s="65" t="inlineStr">
         <is>
           <t>Un único plan para conseguir clientes en todos los servicios, con prioridades. Con 10 a 20 horas semanales no se pueden empujar siete líneas a la vez: se trabajan a fondo las dos primeras, se cuida el resto con contactos cálidos y se documenta lo demás. Detalle completo en 02-sales/plan-captacion-todos-los-servicios.md.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1" s="50">
+    <row r="4" ht="30" customHeight="1" s="52">
       <c r="A4" s="66" t="inlineStr">
         <is>
           <t>Servicio</t>
@@ -11294,7 +11298,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="91" customHeight="1" s="50">
+    <row r="5" ht="91" customHeight="1" s="52">
       <c r="A5" s="62" t="inlineStr">
         <is>
           <t>Team Experience</t>
@@ -11345,7 +11349,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" s="50">
+    <row r="6" ht="60" customHeight="1" s="52">
       <c r="A6" s="62" t="inlineStr">
         <is>
           <t>Coach Experience</t>
@@ -11392,7 +11396,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="91" customHeight="1" s="50">
+    <row r="7" ht="91" customHeight="1" s="52">
       <c r="A7" s="62" t="inlineStr">
         <is>
           <t>Becas EEUU (Study &amp; Play USA)</t>
@@ -11442,7 +11446,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1" s="50">
+    <row r="8" ht="60" customHeight="1" s="52">
       <c r="A8" s="62" t="inlineStr">
         <is>
           <t>Campus Internacional (ATM y Real Sociedad fuera de España)</t>
@@ -11489,7 +11493,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1" s="50">
+    <row r="9" ht="60" customHeight="1" s="52">
       <c r="A9" s="62" t="inlineStr">
         <is>
           <t>International Program (Real Sociedad)</t>
@@ -11536,7 +11540,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1" s="50">
+    <row r="10" ht="60" customHeight="1" s="52">
       <c r="A10" s="62" t="inlineStr">
         <is>
           <t>GEE (colegios privados en EEUU)</t>
@@ -11583,7 +11587,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1" s="50">
+    <row r="11" ht="60" customHeight="1" s="52">
       <c r="A11" s="62" t="inlineStr">
         <is>
           <t>Oportunidades profesionales (Alemania y España) y Player Development</t>
@@ -11630,7 +11634,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="62" customHeight="1" s="50">
+    <row r="12" ht="62" customHeight="1" s="52">
       <c r="A12" s="62" t="inlineStr">
         <is>
           <t>Transversal: marca y canales</t>
@@ -11695,30 +11699,30 @@
   <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="50" min="1" max="1"/>
-    <col width="36" customWidth="1" style="50" min="2" max="2"/>
-    <col width="56" customWidth="1" style="50" min="3" max="3"/>
-    <col width="18" customWidth="1" style="50" min="4" max="4"/>
-    <col width="28" customWidth="1" style="50" min="5" max="5"/>
-    <col width="12" customWidth="1" style="50" min="6" max="6"/>
-    <col width="46" customWidth="1" style="50" min="7" max="7"/>
+    <col width="24" customWidth="1" style="52" min="1" max="1"/>
+    <col width="36" customWidth="1" style="52" min="2" max="2"/>
+    <col width="56" customWidth="1" style="52" min="3" max="3"/>
+    <col width="18" customWidth="1" style="52" min="4" max="4"/>
+    <col width="28" customWidth="1" style="52" min="5" max="5"/>
+    <col width="12" customWidth="1" style="52" min="6" max="6"/>
+    <col width="46" customWidth="1" style="52" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" s="50">
+    <row r="1" ht="26" customHeight="1" s="52">
       <c r="A1" s="64" t="inlineStr">
         <is>
           <t>Verificación de contactos (control de calidad)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="46" customHeight="1" s="50">
+    <row r="2" ht="46" customHeight="1" s="52">
       <c r="A2" s="65" t="inlineStr">
         <is>
           <t>Qué he comprobado de cada dirección y con qué fiabilidad. Importante: ningún método permite saber al 100 % que un buzón existe hasta enviar. Por eso, tras cada envío miras los rebotes a los pocos minutos (tarea diaria del calendario). «Dominio recibe correo» significa que el dominio tiene servidor de correo activo.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1" s="50">
+    <row r="4" ht="30" customHeight="1" s="52">
       <c r="A4" s="66" t="inlineStr">
         <is>
           <t>Club</t>
@@ -11755,7 +11759,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1" s="50">
+    <row r="5" ht="30" customHeight="1" s="52">
       <c r="A5" s="63" t="inlineStr">
         <is>
           <t>Home Farm FC</t>
@@ -11792,7 +11796,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" s="50">
+    <row r="6" ht="30" customHeight="1" s="52">
       <c r="A6" s="63" t="inlineStr">
         <is>
           <t>Hastings United</t>
@@ -11829,7 +11833,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="33" customHeight="1" s="50">
+    <row r="7" ht="33" customHeight="1" s="52">
       <c r="A7" s="63" t="inlineStr">
         <is>
           <t>Søreide IL</t>
@@ -11866,7 +11870,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="33" customHeight="1" s="50">
+    <row r="8" ht="33" customHeight="1" s="52">
       <c r="A8" s="63" t="inlineStr">
         <is>
           <t>Holbeach United</t>
@@ -11903,7 +11907,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="47.5" customHeight="1" s="50">
+    <row r="9" ht="47.5" customHeight="1" s="52">
       <c r="A9" s="63" t="inlineStr">
         <is>
           <t>Whitehaven AFC</t>
@@ -11940,7 +11944,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1" s="50">
+    <row r="10" ht="30" customHeight="1" s="52">
       <c r="A10" s="63" t="inlineStr">
         <is>
           <t>Maidstone United</t>
@@ -11977,7 +11981,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1" s="50">
+    <row r="11" ht="30" customHeight="1" s="52">
       <c r="A11" s="63" t="inlineStr">
         <is>
           <t>IA Akranes</t>
@@ -12014,7 +12018,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1" s="50">
+    <row r="12" ht="30" customHeight="1" s="52">
       <c r="A12" s="63" t="inlineStr">
         <is>
           <t>Virtu Academy</t>
@@ -12051,7 +12055,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="33" customHeight="1" s="50">
+    <row r="13" ht="33" customHeight="1" s="52">
       <c r="A13" s="63" t="inlineStr">
         <is>
           <t>FC Porte d'Aquitaine</t>
@@ -12088,15 +12092,15 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1" s="50">
-      <c r="A15" s="55" t="inlineStr">
+    <row r="15" ht="32" customHeight="1" s="52">
+      <c r="A15" s="57" t="inlineStr">
         <is>
           <t>Descartados tras investigar (13/10): Morecambe Hawks United (equipo local pequeño, no encaja), Team ALTI (sin datos fiables), Lower Ormond (existe en la lista de Semana Santa pero no encuentro contacto).</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="32" customHeight="1" s="50">
-      <c r="A16" s="55" t="inlineStr">
+    <row r="16" ht="32" customHeight="1" s="52">
+      <c r="A16" s="57" t="inlineStr">
         <is>
           <t>Excelsior Rotterdam: club profesional con academia (Joep Breimer, jefe de desarrollo de la cantera). Perfil distinto, prioridad baja.</t>
         </is>
@@ -12121,46 +12125,46 @@
   <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" style="50" min="1" max="1"/>
-    <col width="12" customWidth="1" style="50" min="2" max="2"/>
-    <col width="14" customWidth="1" style="50" min="3" max="3"/>
-    <col width="30" customWidth="1" style="50" min="4" max="4"/>
-    <col width="16" customWidth="1" style="50" min="5" max="5"/>
-    <col width="22" customWidth="1" style="50" min="6" max="7"/>
-    <col width="20" customWidth="1" style="50" min="8" max="8"/>
-    <col width="18" customWidth="1" style="50" min="9" max="9"/>
-    <col width="28" customWidth="1" style="50" min="10" max="10"/>
-    <col width="30" customWidth="1" style="50" min="11" max="11"/>
-    <col width="45" customWidth="1" style="50" min="12" max="12"/>
-    <col width="12" customWidth="1" style="50" min="13" max="13"/>
-    <col width="14" customWidth="1" style="50" min="14" max="14"/>
-    <col width="30" customWidth="1" style="50" min="15" max="15"/>
-    <col width="55" customWidth="1" style="50" min="16" max="16"/>
+    <col width="26" customWidth="1" style="52" min="1" max="1"/>
+    <col width="12" customWidth="1" style="52" min="2" max="2"/>
+    <col width="14" customWidth="1" style="52" min="3" max="3"/>
+    <col width="30" customWidth="1" style="52" min="4" max="4"/>
+    <col width="16" customWidth="1" style="52" min="5" max="5"/>
+    <col width="22" customWidth="1" style="52" min="6" max="7"/>
+    <col width="20" customWidth="1" style="52" min="8" max="8"/>
+    <col width="18" customWidth="1" style="52" min="9" max="9"/>
+    <col width="28" customWidth="1" style="52" min="10" max="10"/>
+    <col width="30" customWidth="1" style="52" min="11" max="11"/>
+    <col width="45" customWidth="1" style="52" min="12" max="12"/>
+    <col width="12" customWidth="1" style="52" min="13" max="13"/>
+    <col width="14" customWidth="1" style="52" min="14" max="14"/>
+    <col width="30" customWidth="1" style="52" min="15" max="15"/>
+    <col width="55" customWidth="1" style="52" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="50">
-      <c r="A1" s="53" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="52">
+      <c r="A1" s="55" t="inlineStr">
         <is>
           <t>Segmento A — Clubes juveniles internacionales</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="54" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>Perfil Greystones/Homefarm: decide un entrenador o comité de club, ciclo de venta corto.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" s="50">
-      <c r="A3" s="56" t="inlineStr">
+    <row r="3" ht="60" customHeight="1" s="52">
+      <c r="A3" s="58" t="inlineStr">
         <is>
           <t>Prioridad principal (ver plan-ventas-maestro.md sección 3). Estado: usar exactamente estos valores para que las fórmulas de la pestaña Hoy funcionen — Pendiente investigar / Listo para enviar / Enviado / Respondido / Llamada agendada / Llamada realizada / Cerrado / Perdido / En negociación / Solo info.</t>
         </is>
       </c>
     </row>
     <row r="4"/>
-    <row r="5" ht="28" customHeight="1" s="50">
+    <row r="5" ht="28" customHeight="1" s="52">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Club/Academia</t>
@@ -12242,7 +12246,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" s="50">
+    <row r="6" ht="60" customHeight="1" s="52">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Home Farm FC (chicas U13-U15)</t>
@@ -12327,7 +12331,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1" s="50">
+    <row r="7" ht="60" customHeight="1" s="52">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Søreide IL</t>
@@ -12366,12 +12370,12 @@
       <c r="H7" s="4" t="n"/>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Enviado</t>
+          <t>Listo para enviar</t>
         </is>
       </c>
       <c r="J7" s="9" t="inlineStr">
         <is>
-          <t>Follow-up 1 el 21/10/2026 en el mismo hilo (enviar a las 07:30 hora Nueva York). Textos en la hoja 'Textos para copiar'.</t>
+          <t>Enviar el 14/10/2026 a las 07:30 hora Nueva York. Textos en la hoja 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr">
@@ -12392,11 +12396,11 @@
 joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
         </is>
       </c>
-      <c r="M7" s="100" t="n">
-        <v>46309</v>
-      </c>
-      <c r="N7" s="100" t="n">
-        <v>46309</v>
+      <c r="M7" s="10" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N7" s="10" t="n">
+        <v>46308</v>
       </c>
       <c r="O7" s="9" t="inlineStr">
         <is>
@@ -12409,7 +12413,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" s="50">
+    <row r="8" ht="18" customHeight="1" s="52">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Maidstone United (Girls Development Centre)</t>
@@ -12490,7 +12494,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" s="50">
+    <row r="9" ht="18" customHeight="1" s="52">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Whitehaven AFC (Juniors Girls U13-U15)</t>
@@ -12567,7 +12571,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" s="50">
+    <row r="10" ht="18" customHeight="1" s="52">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Lower Ormond</t>
@@ -12612,7 +12616,7 @@
       <c r="N10" s="10" t="n"/>
       <c r="O10" s="9" t="inlineStr">
         <is>
-          <t>Investigado 2026-08-29: posible error de nombre en el research original — no gastar más tiempo hasta verificar en la fuente original | 13/10/2026: costadauradacup.com lo lista como club de Inglaterra en la edición de Semana Santa 2026. Existe: falta encontrar su contacto. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable.</t>
+          <t>Investigado 2026-08-29: posible error de nombre en el research original — no gastar más tiempo hasta verificar en la fuente original | 13/10/2026: costadauradacup.com lo lista como club de Inglaterra en la edición de Semana Santa 2026. Existe: falta encontrar su contacto. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable. | 13/10/2026: aparece como club de Inglaterra en la edición de Semana Santa de la Costa Daurada Cup. No encuentro contacto fiable.</t>
         </is>
       </c>
       <c r="P10" s="9" t="inlineStr">
@@ -12621,7 +12625,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" s="50">
+    <row r="11" ht="18" customHeight="1" s="52">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Holbeach United</t>
@@ -12664,12 +12668,12 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Enviado</t>
+          <t>Listo para enviar</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>Follow-up 1 el 21/10/2026 en el mismo hilo (enviar a las 07:30 hora Nueva York). Textos en la hoja 'Textos para copiar'.</t>
+          <t>Enviar el 14/10/2026 a las 07:30 hora Nueva York. Textos en la hoja 'Textos para copiar'.</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr">
@@ -12690,15 +12694,11 @@
 joel.martinez@alwaysup.es | +1 (814) 329 1929 | alwaysup.es</t>
         </is>
       </c>
-      <c r="M11" s="100" t="n">
-        <v>46309</v>
-      </c>
-      <c r="N11" s="100" t="n">
-        <v>46309</v>
-      </c>
+      <c r="M11" s="10" t="n"/>
+      <c r="N11" s="10" t="n"/>
       <c r="O11" s="9" t="inlineStr">
         <is>
-          <t>Investigado 2026-08-29: contacto general real, falta nombre de decisor | Enviado a mano el 14/10/2026 (el envío programado con Apple Mail no salió).</t>
+          <t>Investigado 2026-08-29: contacto general real, falta nombre de decisor | Posible duplicado: 13/10 18:50, 14/10 04:41 y 14/10 ~08:30 (el último no localizado). No pedir disculpas salvo que lo mencionen.</t>
         </is>
       </c>
       <c r="P11" s="9" t="inlineStr">
@@ -12707,7 +12707,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1" s="50">
+    <row r="12" ht="60" customHeight="1" s="52">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Hastings United (Girls Academy)</t>
@@ -12787,7 +12787,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1" s="50">
+    <row r="13" ht="18" customHeight="1" s="52">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Morecambe Hawks</t>
@@ -12845,7 +12845,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1" s="50">
+    <row r="14" ht="18" customHeight="1" s="52">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>IA Akranes</t>
@@ -12914,7 +12914,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" s="50">
+    <row r="15" ht="18" customHeight="1" s="52">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Excelsior Rotterdam</t>
@@ -12968,7 +12968,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" s="50">
+    <row r="16" ht="18" customHeight="1" s="52">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Deportivo de la Coruña</t>
@@ -13022,7 +13022,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="90" customHeight="1" s="50">
+    <row r="17" ht="90" customHeight="1" s="52">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Leonardo Uren / equipo (Brasil) — posible partner, no solo cliente</t>
@@ -13088,7 +13088,7 @@
       </c>
       <c r="O17" s="9" t="inlineStr">
         <is>
-          <t>Historial real: llamada en abril 2026, Leonardo mandó una presentación (enfocada en becas EEUU, poco encaje con lo que ya cubre el partner de becas), Joel propuso el ángulo real (intercambio Brasil-España de jugadores/equipos), propuso llamada con el padre para junio, luego siguió el 03/07 proponiendo martes — sin respuesta desde entonces (2+ meses). No confundir con un club prospecto normal de Segmento A — esto es más una posible relación de partner/distribución que una venta directa. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta.</t>
+          <t>Historial real: llamada en abril 2026, Leonardo mandó una presentación (enfocada en becas EEUU, poco encaje con lo que ya cubre el partner de becas), Joel propuso el ángulo real (intercambio Brasil-España de jugadores/equipos), propuso llamada con el padre para junio, luego siguió el 03/07 proponiendo martes — sin respuesta desde entonces (2+ meses). No confundir con un club prospecto normal de Segmento A — esto es más una posible relación de partner/distribución que una venta directa. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta. | 13/10/2026: Joel decide no reactivar: varios intentos y las dos últimas sin respuesta.</t>
         </is>
       </c>
       <c r="P17" s="9" t="inlineStr">
@@ -13097,7 +13097,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="293" customHeight="1" s="50">
+    <row r="18" ht="293" customHeight="1" s="52">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Virtu Academy</t>
@@ -13170,7 +13170,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="332" customHeight="1" s="50">
+    <row r="19" ht="332" customHeight="1" s="52">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>FC Porte d'Aquitaine</t>
@@ -13303,44 +13303,44 @@
   <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" style="50" min="1" max="1"/>
-    <col width="18" customWidth="1" style="50" min="2" max="3"/>
-    <col width="34" customWidth="1" style="50" min="4" max="4"/>
-    <col width="20" customWidth="1" style="50" min="5" max="5"/>
-    <col width="18" customWidth="1" style="50" min="6" max="7"/>
-    <col width="26" customWidth="1" style="50" min="8" max="8"/>
-    <col width="28" customWidth="1" style="50" min="9" max="9"/>
-    <col width="26" customWidth="1" style="50" min="10" max="10"/>
-    <col width="40" customWidth="1" style="50" min="11" max="11"/>
-    <col width="12" customWidth="1" style="50" min="12" max="12"/>
-    <col width="14" customWidth="1" style="50" min="13" max="13"/>
-    <col width="36" customWidth="1" style="50" min="14" max="14"/>
-    <col width="55" customWidth="1" style="50" min="15" max="15"/>
+    <col width="30" customWidth="1" style="52" min="1" max="1"/>
+    <col width="18" customWidth="1" style="52" min="2" max="3"/>
+    <col width="34" customWidth="1" style="52" min="4" max="4"/>
+    <col width="20" customWidth="1" style="52" min="5" max="5"/>
+    <col width="18" customWidth="1" style="52" min="6" max="7"/>
+    <col width="26" customWidth="1" style="52" min="8" max="8"/>
+    <col width="28" customWidth="1" style="52" min="9" max="9"/>
+    <col width="26" customWidth="1" style="52" min="10" max="10"/>
+    <col width="40" customWidth="1" style="52" min="11" max="11"/>
+    <col width="12" customWidth="1" style="52" min="12" max="12"/>
+    <col width="14" customWidth="1" style="52" min="13" max="13"/>
+    <col width="36" customWidth="1" style="52" min="14" max="14"/>
+    <col width="55" customWidth="1" style="52" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="50">
-      <c r="A1" s="53" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="52">
+      <c r="A1" s="55" t="inlineStr">
         <is>
           <t>Segmento B — Universidades y clubes de América</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="54" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>NCAA + clubes/academias EEUU. Incluye fútbol femenino universitario (segmento en crecimiento, menos competido).</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" s="50">
-      <c r="A3" s="56" t="inlineStr">
+    <row r="3" ht="60" customHeight="1" s="52">
+      <c r="A3" s="58" t="inlineStr">
         <is>
           <t>PRIORIDAD SECUNDARIA — ver plan-ventas-maestro.md sección 3. Mercado ya servido por competidores establecidos (Alandis Travel + Sevilla FC, WorldStrides...) y con ciclos de decisión institucionales largos. No forzar volumen aquí hasta tener 2-3 conversaciones reales avanzando en Segmento A.</t>
         </is>
       </c>
     </row>
     <row r="4"/>
-    <row r="5" ht="28" customHeight="1" s="50">
+    <row r="5" ht="28" customHeight="1" s="52">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Programa/Club</t>
@@ -13417,7 +13417,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="56" customHeight="1" s="50">
+    <row r="6" ht="56" customHeight="1" s="52">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>ODP Louisiana</t>
@@ -13466,7 +13466,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="56" customHeight="1" s="50">
+    <row r="7" ht="56" customHeight="1" s="52">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Dallas Texans</t>
@@ -13519,7 +13519,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="56" customHeight="1" s="50">
+    <row r="8" ht="56" customHeight="1" s="52">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Charlotte SA</t>
@@ -13572,7 +13572,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="56" customHeight="1" s="50">
+    <row r="9" ht="56" customHeight="1" s="52">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Philadelphia Union Academy</t>
@@ -13625,7 +13625,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="56" customHeight="1" s="50">
+    <row r="10" ht="56" customHeight="1" s="52">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Seattle United</t>
@@ -13678,7 +13678,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="56" customHeight="1" s="50">
+    <row r="11" ht="56" customHeight="1" s="52">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>San Diego Surf</t>
@@ -13731,7 +13731,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="56" customHeight="1" s="50">
+    <row r="12" ht="56" customHeight="1" s="52">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>UNC Women's Soccer</t>
@@ -13784,7 +13784,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="56" customHeight="1" s="50">
+    <row r="13" ht="56" customHeight="1" s="52">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Programas NCAA D2/D3 sin partnership visible (por identificar)</t>
@@ -13857,42 +13857,42 @@
   <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" style="50" min="1" max="1"/>
-    <col width="8" customWidth="1" style="50" min="2" max="2"/>
-    <col width="18" customWidth="1" style="50" min="3" max="3"/>
-    <col width="30" customWidth="1" style="50" min="4" max="4"/>
-    <col width="18" customWidth="1" style="50" min="5" max="5"/>
-    <col width="16" customWidth="1" style="50" min="6" max="6"/>
-    <col width="28" customWidth="1" style="50" min="7" max="7"/>
-    <col width="34" customWidth="1" style="50" min="8" max="8"/>
-    <col width="16" customWidth="1" style="50" min="9" max="9"/>
-    <col width="40" customWidth="1" style="50" min="10" max="10"/>
-    <col width="55" customWidth="1" style="50" min="11" max="11"/>
+    <col width="30" customWidth="1" style="52" min="1" max="1"/>
+    <col width="8" customWidth="1" style="52" min="2" max="2"/>
+    <col width="18" customWidth="1" style="52" min="3" max="3"/>
+    <col width="30" customWidth="1" style="52" min="4" max="4"/>
+    <col width="18" customWidth="1" style="52" min="5" max="5"/>
+    <col width="16" customWidth="1" style="52" min="6" max="6"/>
+    <col width="28" customWidth="1" style="52" min="7" max="7"/>
+    <col width="34" customWidth="1" style="52" min="8" max="8"/>
+    <col width="16" customWidth="1" style="52" min="9" max="9"/>
+    <col width="40" customWidth="1" style="52" min="10" max="10"/>
+    <col width="55" customWidth="1" style="52" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="50">
-      <c r="A1" s="53" t="inlineStr">
+    <row r="1" ht="18" customHeight="1" s="52">
+      <c r="A1" s="55" t="inlineStr">
         <is>
           <t>Segmento C — Becas deportivas (inbound Instagram)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="54" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>No es outreach frío — es inbound que ya llega solo. El trabajo es cualificar y cerrar mejor.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1" s="50">
-      <c r="A3" s="56" t="inlineStr">
+    <row r="3" ht="60" customHeight="1" s="52">
+      <c r="A3" s="58" t="inlineStr">
         <is>
           <t>MIGRADO desde 01-clients/pipeline.md (tabla 'Embudo — seguimiento de leads inbound') el 2026-08-29 — esta pestaña sustituye esa tabla como fuente única de verdad para leads de becas. Etapa: usar Nuevo / Cualificado / Llamada agendada / Llamada realizada / Cerrado / Perdido para que las fórmulas de Hoy funcionen.</t>
         </is>
       </c>
     </row>
     <row r="4"/>
-    <row r="5" ht="28" customHeight="1" s="50">
+    <row r="5" ht="28" customHeight="1" s="52">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Nombre / contacto (IG)</t>
@@ -13949,7 +13949,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1" s="50">
+    <row r="6" ht="42" customHeight="1" s="52">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Francisco Ferreira / francisco_7ferreira</t>
@@ -14006,7 +14006,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1" s="50">
+    <row r="7" ht="42" customHeight="1" s="52">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Bauti / bautimoransalzano</t>
@@ -14051,7 +14051,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1" s="50">
+    <row r="8" ht="42" customHeight="1" s="52">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Pavel Gomez / paixvi.b</t>
@@ -14108,7 +14108,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1" s="50">
+    <row r="9" ht="42" customHeight="1" s="52">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Gonzalo Caro / gonzalocarocontreras</t>
@@ -14149,7 +14149,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1" s="50">
+    <row r="10" ht="42" customHeight="1" s="52">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Tania Coeto / tania_coeto</t>
@@ -14190,7 +14190,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1" s="50">
+    <row r="11" ht="42" customHeight="1" s="52">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Barbara Cuellar / bcshisha</t>
@@ -14247,7 +14247,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="75" customHeight="1" s="50">
+    <row r="12" ht="75" customHeight="1" s="52">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Omar Escamilla / omare815 — CONFIRMADO mismo lead que WhatsApp +52 1 81 3408 2672 (Gabriel y Rafael)</t>
@@ -14304,7 +14304,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="42" customHeight="1" s="50">
+    <row r="13" ht="42" customHeight="1" s="52">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Angelica Suarez Rivera / angelicamiami</t>
@@ -14357,7 +14357,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="42" customHeight="1" s="50">
+    <row r="14" ht="42" customHeight="1" s="52">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Ana Aida Uribe / aauribe</t>
@@ -14406,7 +14406,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="42" customHeight="1" s="50">
+    <row r="15" ht="42" customHeight="1" s="52">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Jeinz Alzate / jeinzalzate</t>
@@ -14459,7 +14459,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1" s="50">
+    <row r="16" ht="42" customHeight="1" s="52">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Anita / ani_0487</t>
@@ -14508,7 +14508,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="42" customHeight="1" s="50">
+    <row r="17" ht="42" customHeight="1" s="52">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Margarita Vanegas / margaritavanegasoficial</t>
@@ -14561,7 +14561,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1" s="50">
+    <row r="18" ht="42" customHeight="1" s="52">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Edwin Serrato / edwinserrato84</t>
@@ -14618,7 +14618,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="42" customHeight="1" s="50">
+    <row r="19" ht="42" customHeight="1" s="52">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Juan Roberto / juan_roberto_16</t>
@@ -14659,10 +14659,10 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1" s="50">
+    <row r="20" ht="60" customHeight="1" s="52">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Daniel (apellido/@ de Instagram pendiente de confirmar)</t>
+          <t>Daniel / Instagram: Danny (confirmar @usuario exacto)</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -14697,7 +14697,7 @@
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>Esperar respuesta a las 3 preguntas (posición / ubicación en España / club actual) — probablemente avanza rápido a Calendly, es un lead fuerte</t>
+          <t>Enviar follow-up el 14/10 (texto en Textos para copiar). Si no responde en 7 días: pasar a Frío.</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -14707,7 +14707,7 @@
       </c>
       <c r="J20" s="9" t="inlineStr">
         <is>
-          <t>Pregunta genuina sobre 1º vs 2º de Bachillerato y elegibilidad NCAA — no se improvisó respuesta, se remitió a la evaluación completa con el equipo especializado. Edad+plazo+nivel ya fuertes antes incluso de pedir vídeo.</t>
+          <t>Pregunta genuina sobre 1º vs 2º de Bachillerato y elegibilidad NCAA — no se improvisó respuesta, se remitió a la evaluación completa con el equipo especializado. Edad+plazo+nivel ya fuertes antes incluso de pedir vídeo. | 14/10: sin respuesta desde el 21/09 (3 semanas). Un solo follow-up.</t>
         </is>
       </c>
       <c r="K20" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Marca follow-up de Daniel y programacion del jueves como hechos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -33,10 +33,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="34">
     <font>
@@ -405,7 +406,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -663,6 +664,9 @@
     </xf>
     <xf numFmtId="165" fontId="31" fillId="21" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2642,10 +2646,14 @@
       </c>
       <c r="I16" s="70" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J16" s="70" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="J16" s="70" t="inlineStr">
+        <is>
+          <t>Enviado el 14/10</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="163.5" customHeight="1" s="52">
       <c r="A17" s="94" t="n">
@@ -2690,10 +2698,14 @@
       </c>
       <c r="I17" s="70" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="J17" s="70" t="n"/>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="J17" s="70" t="inlineStr">
+        <is>
+          <t>Programados los 3 (confirmar mañana a las 08:00)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="47.5" customHeight="1" s="52">
       <c r="A18" s="94" t="n">
@@ -12122,7 +12134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="52" min="1" max="1"/>
@@ -13243,46 +13255,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <autoFilter ref="A5:P17"/>
   <mergeCells count="3">
@@ -14697,13 +14669,11 @@
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>Enviar follow-up el 14/10 (texto en Textos para copiar). Si no responde en 7 días: pasar a Frío.</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
+          <t>Follow-up enviado el 14/10. Si no responde el 21/10: pasar a Frío y no insistir.</t>
+        </is>
+      </c>
+      <c r="I20" s="100" t="n">
+        <v>46309</v>
       </c>
       <c r="J20" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Propuesta de colaboracion 2028 para Gonzalo (Argentina): presentacion de 10 diapositivas, generador y registro en el CRM
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -34,12 +34,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="168" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="31">
     <font>
@@ -379,7 +378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -629,7 +628,10 @@
     <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -1860,7 +1862,7 @@
           <t>Frío: sin respuesta al follow-up del 13/10 ni al último mensaje del 20/10. Retomar en enero 2027 con el gancho de los plazos de la temporada siguiente. No insistir.</t>
         </is>
       </c>
-      <c r="I12" s="97" t="n">
+      <c r="I12" s="98" t="n">
         <v>46322</v>
       </c>
       <c r="J12" s="9" t="inlineStr">
@@ -2270,7 +2272,7 @@
           <t>Frío: sin respuesta al mensaje del 21/09 ni al follow-up del 14/10. Retomar en enero 2027 si él escribe. No insistir.</t>
         </is>
       </c>
-      <c r="I20" s="97" t="n">
+      <c r="I20" s="98" t="n">
         <v>46322</v>
       </c>
       <c r="J20" s="9" t="inlineStr">
@@ -2690,7 +2692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="47" min="1" max="1"/>
@@ -2911,6 +2913,38 @@
       <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Pendiente investigación</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Socio / canal Argentina</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Gonzalo (Argentina): mueve unas 1.000 personas a España en 2027 (jugadores y acompañantes) con red de familias, niños y clubes. Quiere ver opciones y cómo trabajar juntos para 2028.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Reunión con Joel (semana del 19/10/2026)</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Propuesta enviada el 27/10 (01-clients/propuestas/Always-Up-Propuesta-Gonzalo-Argentina.pdf). Siguiente: llamada de 30 min esta semana o la próxima y preguntas de descubrimiento (grupos, volumen 2028, presupuesto, cómo viajan hoy). Modelo de colaboración y condiciones: decisión de Joel y Enrique antes de dar números.</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Propuesta preparada</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Presentacion definitiva para Gonzalo (Argentina 2028): mezcla de la version de Enrique y la de Joel, con identidad corporativa, aguila y 19 diapositivas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -2692,7 +2692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="47" min="1" max="1"/>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Propuesta enviada el 27/10 (01-clients/propuestas/Always-Up-Propuesta-Gonzalo-Argentina.pdf). Siguiente: llamada de 30 min esta semana o la próxima y preguntas de descubrimiento (grupos, volumen 2028, presupuesto, cómo viajan hoy). Modelo de colaboración y condiciones: decisión de Joel y Enrique antes de dar números.</t>
+          <t>Propuesta definitiva (mezcla de Joel y Enrique) lista el 27/10 (01-clients/propuestas/Always-Up-Propuesta-Gonzalo-Argentina-2028.pdf). Siguiente: llamada de 30 min esta semana o la próxima y preguntas de descubrimiento (grupos, volumen 2028, presupuesto, cómo viajan hoy). Modelo de colaboración y condiciones: decisión de Joel y Enrique antes de dar números.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Propuesta final para Gonzalo Lamas: apellido, fotos de la academia del Atletico, nueva diapositiva de jugadores en Espana, servicios reordenados y cierre solo con contacto de Joel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01-clients/crm-ventas.xlsx
+++ b/01-clients/crm-ventas.xlsx
@@ -2929,7 +2929,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Gonzalo (Argentina): mueve unas 1.000 personas a España en 2027 (jugadores y acompañantes) con red de familias, niños y clubes. Quiere ver opciones y cómo trabajar juntos para 2028.</t>
+          <t>Gonzalo Lamas (Argentina): mueve unas 1.000 personas a España en 2027 (jugadores y acompañantes) con red de familias, niños y clubes. Quiere ver opciones y cómo trabajar juntos para 2028.</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Propuesta definitiva (mezcla de Joel y Enrique) lista el 27/10 (01-clients/propuestas/Always-Up-Propuesta-Gonzalo-Argentina-2028.pdf). Siguiente: llamada de 30 min esta semana o la próxima y preguntas de descubrimiento (grupos, volumen 2028, presupuesto, cómo viajan hoy). Modelo de colaboración y condiciones: decisión de Joel y Enrique antes de dar números.</t>
+          <t>Propuesta definitiva (mezcla de Joel y Enrique) lista el 27/10 (01-clients/propuestas/Always-Up-Propuesta-Gonzalo-Lamas-Argentina-2028.pdf). Siguiente: llamada de 30 min esta semana o la próxima y preguntas de descubrimiento (grupos, volumen 2028, presupuesto, cómo viajan hoy). Modelo de colaboración y condiciones: decisión de Joel y Enrique antes de dar números.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">

</xml_diff>